<commit_message>
Actualización lógica colorimetría y correcciones CIELAB
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="643" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1A676981-FB0B-4C62-B661-3AB43A3EB4BE}"/>
+  <xr:revisionPtr revIDLastSave="720" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E38495-5D83-4C02-A15C-130A53967ECC}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4560" yWindow="615" windowWidth="16200" windowHeight="9270" activeTab="2" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
   <sheets>
     <sheet name="CALCULO MEDICION " sheetId="3" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="54">
   <si>
     <t>MEDICIONES</t>
   </si>
@@ -88,9 +88,6 @@
     <t>Foron RED</t>
   </si>
   <si>
-    <t>A  o CWF</t>
-  </si>
-  <si>
     <t>[ Total ]</t>
   </si>
   <si>
@@ -109,12 +106,6 @@
     <t>CALCULOS REALIZADOS</t>
   </si>
   <si>
-    <t xml:space="preserve">PROMEDIO </t>
-  </si>
-  <si>
-    <t>PROMEDIO</t>
-  </si>
-  <si>
     <t xml:space="preserve"> RECETA  (A o CWF)</t>
   </si>
   <si>
@@ -206,15 +197,19 @@
   </si>
   <si>
     <t>% a corregir B</t>
+  </si>
+  <si>
+    <t>Promedio Chroma</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -283,7 +278,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -293,6 +288,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -380,7 +381,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="40">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -410,45 +411,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -465,15 +427,69 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -490,10 +506,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -839,25 +851,25 @@
     <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D2" s="2"/>
       <c r="E2" s="2" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="10" t="s">
-        <v>36</v>
-      </c>
-      <c r="I2" s="10"/>
+      <c r="H2" s="22" t="s">
+        <v>33</v>
+      </c>
+      <c r="I2" s="22"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2">
         <v>82.83</v>
@@ -865,27 +877,27 @@
       <c r="C3" s="2">
         <v>80.680000000000007</v>
       </c>
-      <c r="D3" s="27">
+      <c r="D3" s="14">
         <f>+C3-B3</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="E3" s="27">
+      <c r="E3" s="14">
         <f>+ABS(D3)</f>
         <v>2.1499999999999915</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="28">
+      <c r="H3" s="15">
         <f>+E3/B3</f>
         <v>2.5956778944826651E-2</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" s="2" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="B4" s="2">
         <v>-14.24</v>
@@ -893,27 +905,27 @@
       <c r="C4" s="2">
         <v>-13.01</v>
       </c>
-      <c r="D4" s="27">
+      <c r="D4" s="14">
         <f t="shared" ref="D4:D5" si="0">+C4-B4</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="E4" s="27">
+      <c r="E4" s="14">
         <f>+ABS(D4)</f>
         <v>1.2300000000000004</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="28">
-        <f t="shared" ref="H4:H5" si="1">+E4/B4</f>
+      <c r="H4" s="15">
+        <f>+E4/B4</f>
         <v>-8.6376404494382053E-2</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
     </row>
     <row r="5" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A5" s="2" t="s">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="B5" s="2">
         <v>3.6</v>
@@ -921,351 +933,366 @@
       <c r="C5" s="2">
         <v>-3.47</v>
       </c>
-      <c r="D5" s="27">
+      <c r="D5" s="14">
         <f t="shared" si="0"/>
         <v>-7.07</v>
       </c>
-      <c r="E5" s="27">
+      <c r="E5" s="14">
         <f>+ABS(D5)</f>
         <v>7.07</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="28">
-        <f t="shared" si="1"/>
+      <c r="H5" s="15">
+        <f t="shared" ref="H5" si="1">+E5/B5</f>
         <v>1.963888888888889</v>
       </c>
       <c r="I5" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B8" s="16"/>
+      <c r="C8" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="E8" s="16" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="29"/>
-      <c r="C8" s="29" t="s">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B9" s="16" t="s">
+        <v>7</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>43</v>
       </c>
-      <c r="D8" s="29" t="s">
+      <c r="D9" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E9" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B10" s="16" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E10" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B11" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="C11" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D11" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="E11" s="16" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B13" s="16"/>
+      <c r="C13" s="16"/>
+      <c r="D13" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="E13" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="G13" s="16" t="s">
         <v>44</v>
       </c>
-      <c r="E8" s="29" t="s">
+      <c r="H13" s="16" t="s">
         <v>45</v>
       </c>
-    </row>
-    <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="29" t="s">
+      <c r="I13" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="J13" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="K13" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="L13" s="16" t="s">
+        <v>49</v>
+      </c>
+      <c r="M13" s="16" t="s">
+        <v>50</v>
+      </c>
+      <c r="N13" s="16" t="s">
+        <v>51</v>
+      </c>
+      <c r="O13" s="16" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="B14" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D9" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="E9" s="29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="29" t="s">
-        <v>8</v>
-      </c>
-      <c r="C10" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D10" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="E10" s="29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="C11" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="D11" s="29" t="s">
-        <v>46</v>
-      </c>
-      <c r="E11" s="29" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="29"/>
-      <c r="C13" s="29"/>
-      <c r="D13" s="29" t="s">
-        <v>43</v>
-      </c>
-      <c r="E13" s="29" t="s">
-        <v>44</v>
-      </c>
-      <c r="F13" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="G13" s="29" t="s">
-        <v>47</v>
-      </c>
-      <c r="H13" s="29" t="s">
-        <v>48</v>
-      </c>
-      <c r="I13" s="29" t="s">
-        <v>49</v>
-      </c>
-      <c r="J13" s="29" t="s">
-        <v>50</v>
-      </c>
-      <c r="K13" s="29" t="s">
-        <v>51</v>
-      </c>
-      <c r="L13" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="M13" s="29" t="s">
-        <v>53</v>
-      </c>
-      <c r="N13" s="29" t="s">
-        <v>54</v>
-      </c>
-      <c r="O13" s="29" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="30" t="s">
-        <v>7</v>
-      </c>
-      <c r="C14" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D14" s="29">
+      <c r="C14" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D14" s="16">
         <v>82.83</v>
       </c>
-      <c r="E14" s="29">
+      <c r="E14" s="16">
         <v>-14.24</v>
       </c>
-      <c r="F14" s="29">
+      <c r="F14" s="16">
         <v>-3.6</v>
       </c>
-      <c r="G14" s="30">
+      <c r="G14" s="20">
         <f>+D15-D14</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H14" s="30">
+      <c r="H14" s="20">
         <f>+E15-E14</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I14" s="30">
+      <c r="I14" s="20">
         <f>+F15-F14</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J14" s="30">
+      <c r="J14" s="20">
         <f>+ABS(G14)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K14" s="30">
+      <c r="K14" s="20">
         <f>+ABS(H14)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L14" s="30">
+      <c r="L14" s="20">
         <f>+ABS(I14)</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="M14" s="31">
+      <c r="M14" s="21">
         <f>+K14/F14</f>
         <v>-0.34166666666666679</v>
       </c>
-      <c r="N14" s="31">
+      <c r="N14" s="21">
         <f>+K14/E14</f>
         <v>-8.6376404494382053E-2</v>
       </c>
-      <c r="O14" s="31">
+      <c r="O14" s="21">
         <f>+L14/F14</f>
         <v>-3.611111111111108E-2</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="30"/>
-      <c r="C15" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D15" s="29">
+      <c r="B15" s="20"/>
+      <c r="C15" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="16">
         <v>80.680000000000007</v>
       </c>
-      <c r="E15" s="29">
+      <c r="E15" s="16">
         <v>-13.01</v>
       </c>
-      <c r="F15" s="29">
+      <c r="F15" s="16">
         <v>-3.47</v>
       </c>
-      <c r="G15" s="30"/>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-      <c r="J15" s="30"/>
-      <c r="K15" s="30"/>
-      <c r="L15" s="30"/>
-      <c r="M15" s="31"/>
-      <c r="N15" s="31"/>
-      <c r="O15" s="31"/>
+      <c r="G15" s="20"/>
+      <c r="H15" s="20"/>
+      <c r="I15" s="20"/>
+      <c r="J15" s="20"/>
+      <c r="K15" s="20"/>
+      <c r="L15" s="20"/>
+      <c r="M15" s="21"/>
+      <c r="N15" s="21"/>
+      <c r="O15" s="21"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D16" s="29">
+      <c r="C16" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D16" s="16">
         <v>81.81</v>
       </c>
-      <c r="E16" s="29">
+      <c r="E16" s="16">
         <v>-12.77</v>
       </c>
-      <c r="F16" s="29">
+      <c r="F16" s="16">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G16" s="30">
+      <c r="G16" s="20">
         <f>+D17-D16</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H16" s="30">
+      <c r="H16" s="20">
         <f t="shared" ref="H16:I16" si="2">+E17-E16</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I16" s="30">
+      <c r="I16" s="20">
         <f t="shared" si="2"/>
         <v>-9.39</v>
       </c>
-      <c r="J16" s="30">
+      <c r="J16" s="20">
         <f t="shared" ref="J16:L16" si="3">+ABS(G16)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K16" s="30">
+      <c r="K16" s="20">
         <f t="shared" si="3"/>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L16" s="30">
+      <c r="L16" s="20">
         <f t="shared" si="3"/>
         <v>9.39</v>
       </c>
-      <c r="M16" s="31">
+      <c r="M16" s="21">
         <f>+J16/D16</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="N16" s="31">
+      <c r="N16" s="21">
         <f>+K16/E16</f>
         <v>-5.7165231010180145E-2</v>
       </c>
-      <c r="O16" s="31">
+      <c r="O16" s="21">
         <f t="shared" ref="O16" si="4">+L16/F16</f>
         <v>1.8557312252964429</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="30"/>
-      <c r="C17" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D17" s="29">
+      <c r="B17" s="20"/>
+      <c r="C17" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D17" s="16">
         <v>79.78</v>
       </c>
-      <c r="E17" s="29">
+      <c r="E17" s="16">
         <v>-12.04</v>
       </c>
-      <c r="F17" s="29">
+      <c r="F17" s="16">
         <v>-4.33</v>
       </c>
-      <c r="G17" s="30"/>
-      <c r="H17" s="30"/>
-      <c r="I17" s="30"/>
-      <c r="J17" s="30"/>
-      <c r="K17" s="30"/>
-      <c r="L17" s="30"/>
-      <c r="M17" s="31"/>
-      <c r="N17" s="31"/>
-      <c r="O17" s="31"/>
+      <c r="G17" s="20"/>
+      <c r="H17" s="20"/>
+      <c r="I17" s="20"/>
+      <c r="J17" s="20"/>
+      <c r="K17" s="20"/>
+      <c r="L17" s="20"/>
+      <c r="M17" s="21"/>
+      <c r="N17" s="21"/>
+      <c r="O17" s="21"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="30" t="s">
-        <v>44</v>
-      </c>
-      <c r="C18" s="29" t="s">
-        <v>33</v>
-      </c>
-      <c r="D18" s="29">
+      <c r="B18" s="20" t="s">
+        <v>41</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="16">
         <v>80.94</v>
       </c>
-      <c r="E18" s="29">
+      <c r="E18" s="16">
         <v>-15.03</v>
       </c>
-      <c r="F18" s="29">
+      <c r="F18" s="16">
         <v>7.39</v>
       </c>
-      <c r="G18" s="30">
+      <c r="G18" s="20">
         <f>+D19-D18</f>
         <v>-4</v>
       </c>
-      <c r="H18" s="30">
+      <c r="H18" s="20">
         <f t="shared" ref="H18:I18" si="5">+E19-E18</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I18" s="30">
+      <c r="I18" s="20">
         <f t="shared" si="5"/>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J18" s="30">
+      <c r="J18" s="20">
         <f t="shared" ref="J18:L18" si="6">+ABS(G18)</f>
         <v>4</v>
       </c>
-      <c r="K18" s="30">
+      <c r="K18" s="20">
         <f t="shared" si="6"/>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L18" s="30">
+      <c r="L18" s="20">
         <f t="shared" si="6"/>
         <v>0.58999999999999986</v>
       </c>
-      <c r="M18" s="31">
+      <c r="M18" s="21">
         <f>+J18/D18</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="N18" s="31">
+      <c r="N18" s="21">
         <f>+K18/E18</f>
         <v>-5.7884231536926095E-2</v>
       </c>
-      <c r="O18" s="31">
+      <c r="O18" s="21">
         <f t="shared" ref="O18" si="7">+L18/F18</f>
         <v>7.9837618403247615E-2</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="30"/>
-      <c r="C19" s="29" t="s">
-        <v>34</v>
-      </c>
-      <c r="D19" s="29">
+      <c r="B19" s="20"/>
+      <c r="C19" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D19" s="16">
         <v>76.94</v>
       </c>
-      <c r="E19" s="29">
+      <c r="E19" s="16">
         <v>-14.16</v>
       </c>
-      <c r="F19" s="29">
+      <c r="F19" s="16">
         <v>6.8</v>
       </c>
-      <c r="G19" s="30"/>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-      <c r="J19" s="30"/>
-      <c r="K19" s="30"/>
-      <c r="L19" s="30"/>
-      <c r="M19" s="31"/>
-      <c r="N19" s="31"/>
-      <c r="O19" s="31"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="J18:J19"/>
     <mergeCell ref="L18:L19"/>
     <mergeCell ref="M18:M19"/>
     <mergeCell ref="N18:N19"/>
@@ -1275,27 +1302,12 @@
     <mergeCell ref="M16:M17"/>
     <mergeCell ref="N16:N17"/>
     <mergeCell ref="O16:O17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="J18:J19"/>
     <mergeCell ref="K18:K19"/>
     <mergeCell ref="L14:L15"/>
     <mergeCell ref="M14:M15"/>
     <mergeCell ref="N14:N15"/>
     <mergeCell ref="O14:O15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
     <mergeCell ref="K16:K17"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
     <mergeCell ref="K14:K15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1317,21 +1329,21 @@
     <col min="11" max="11" width="18.28515625" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
     <col min="13" max="15" width="9.140625" style="1"/>
-    <col min="16" max="16" width="10.7109375" style="1" customWidth="1"/>
+    <col min="16" max="16" width="17.28515625" style="1" customWidth="1"/>
     <col min="17" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E2" s="16" t="s">
+      <c r="E2" s="27" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="16"/>
-      <c r="G2" s="16"/>
-      <c r="H2" s="16"/>
-      <c r="I2" s="16"/>
-      <c r="N2" s="14"/>
-      <c r="O2" s="14"/>
-      <c r="P2" s="14"/>
+      <c r="F2" s="27"/>
+      <c r="G2" s="27"/>
+      <c r="H2" s="27"/>
+      <c r="I2" s="27"/>
+      <c r="N2" s="33"/>
+      <c r="O2" s="33"/>
+      <c r="P2" s="33"/>
     </row>
     <row r="3" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E3" s="2"/>
@@ -1364,160 +1376,158 @@
       </c>
     </row>
     <row r="5" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="26" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="20">
+      <c r="F5" s="31">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="20">
+      <c r="G5" s="31">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="21">
+      <c r="H5" s="32">
         <v>0.17</v>
       </c>
-      <c r="I5" s="19">
+      <c r="I5" s="30">
         <v>1.17</v>
       </c>
-      <c r="J5" s="15">
+      <c r="J5" s="26">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="15">
+      <c r="K5" s="26">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="15"/>
-      <c r="F6" s="20"/>
-      <c r="G6" s="20"/>
-      <c r="H6" s="21"/>
-      <c r="I6" s="19"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
+      <c r="E6" s="26"/>
+      <c r="F6" s="31"/>
+      <c r="G6" s="31"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="30"/>
+      <c r="J6" s="26"/>
+      <c r="K6" s="26"/>
       <c r="O6" s="3"/>
     </row>
     <row r="7" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E7" s="10" t="s">
+      <c r="E7" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="17">
+      <c r="F7" s="28">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="18">
+      <c r="G7" s="29">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="18">
+      <c r="H7" s="29">
         <v>0.1</v>
       </c>
-      <c r="I7" s="10">
+      <c r="I7" s="22">
         <v>0.92</v>
       </c>
-      <c r="J7" s="10">
+      <c r="J7" s="22">
         <f t="shared" ref="J7" si="0">+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="10">
+      <c r="K7" s="22">
         <f t="shared" ref="K7" si="1">+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E8" s="10"/>
-      <c r="F8" s="17"/>
-      <c r="G8" s="18"/>
-      <c r="H8" s="18"/>
-      <c r="I8" s="10"/>
-      <c r="J8" s="10"/>
-      <c r="K8" s="10"/>
+      <c r="E8" s="22"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="29"/>
+      <c r="H8" s="29"/>
+      <c r="I8" s="22"/>
+      <c r="J8" s="22"/>
+      <c r="K8" s="22"/>
     </row>
     <row r="9" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E9" s="10" t="s">
+      <c r="E9" s="22" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="17">
+      <c r="F9" s="28">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="18">
+      <c r="G9" s="29">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="18">
+      <c r="H9" s="29">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="10">
+      <c r="I9" s="22">
         <v>1.01</v>
       </c>
-      <c r="J9" s="10">
+      <c r="J9" s="22">
         <f t="shared" ref="J9" si="2">+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="10">
+      <c r="K9" s="22">
         <f t="shared" ref="K9" si="3">+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="10" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E10" s="10"/>
-      <c r="F10" s="17"/>
-      <c r="G10" s="18"/>
-      <c r="H10" s="18"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="10"/>
-      <c r="K10" s="10"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="28"/>
+      <c r="G10" s="29"/>
+      <c r="H10" s="29"/>
+      <c r="I10" s="22"/>
+      <c r="J10" s="22"/>
+      <c r="K10" s="22"/>
     </row>
     <row r="12" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E12" s="12" t="s">
-        <v>27</v>
-      </c>
-      <c r="F12" s="22"/>
-      <c r="G12" s="22"/>
-      <c r="H12" s="22"/>
-      <c r="I12" s="13"/>
-      <c r="J12" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="K12" s="22"/>
-      <c r="L12" s="22"/>
-      <c r="M12" s="22"/>
-      <c r="N12" s="22"/>
-      <c r="O12" s="22"/>
-      <c r="P12" s="13"/>
+      <c r="E12" s="23" t="s">
+        <v>24</v>
+      </c>
+      <c r="F12" s="24"/>
+      <c r="G12" s="24"/>
+      <c r="H12" s="24"/>
+      <c r="I12" s="25"/>
+      <c r="J12" s="23" t="s">
+        <v>21</v>
+      </c>
+      <c r="K12" s="24"/>
+      <c r="L12" s="24"/>
+      <c r="M12" s="24"/>
+      <c r="N12" s="24"/>
+      <c r="O12" s="24"/>
+      <c r="P12" s="25"/>
     </row>
     <row r="13" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E13" s="2"/>
-      <c r="F13" s="12" t="s">
+      <c r="F13" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="13"/>
-      <c r="H13" s="10" t="s">
+      <c r="G13" s="25"/>
+      <c r="H13" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="10"/>
-      <c r="J13" s="10" t="s">
+      <c r="I13" s="22"/>
+      <c r="J13" s="22" t="s">
+        <v>18</v>
+      </c>
+      <c r="K13" s="22"/>
+      <c r="L13" s="22" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="10"/>
-      <c r="L13" s="10" t="s">
+      <c r="M13" s="22"/>
+      <c r="N13" s="22" t="s">
         <v>20</v>
       </c>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10" t="s">
-        <v>21</v>
-      </c>
-      <c r="O13" s="10"/>
+      <c r="O13" s="22"/>
       <c r="P13" s="2" t="s">
-        <v>24</v>
+        <v>53</v>
       </c>
     </row>
     <row r="14" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D14" s="11" t="s">
-        <v>7</v>
-      </c>
+      <c r="D14" s="34"/>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="7">
+      <c r="F14" s="35">
         <v>1.1782600000000001</v>
       </c>
       <c r="G14" s="5">
@@ -1532,7 +1542,7 @@
         <f>H14/$H$17</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J14" s="7">
+      <c r="J14" s="37">
         <f>+H14*(1-$K$5/100)</f>
         <v>0.99292912808000011</v>
       </c>
@@ -1540,182 +1550,184 @@
         <f>+J14/$J$17</f>
         <v>0.60805259681281487</v>
       </c>
-      <c r="L14" s="7">
-        <f>+$H$22*(1-$K$7/100)</f>
-        <v>1.0321510469599999</v>
+      <c r="L14" s="37">
+        <f>+$H$14*(1-$K$7/100)</f>
+        <v>1.0276925111199999</v>
       </c>
       <c r="M14" s="5">
         <f>+L14/$J$25</f>
-        <v>0.60805259681281476</v>
-      </c>
-      <c r="N14" s="7">
-        <f>+$H$30*(1-$K$9/100)</f>
-        <v>1.0179742226399999</v>
+        <v>0.60542601972075083</v>
+      </c>
+      <c r="N14" s="37">
+        <f>+$H$14*(1-$K$9/100)</f>
+        <v>1.01248353104</v>
       </c>
       <c r="O14" s="5">
         <f>+N14/$J$33</f>
-        <v>0.60805259681281476</v>
-      </c>
-      <c r="P14" s="7">
+        <v>0.60477291721835513</v>
+      </c>
+      <c r="P14" s="4">
         <f>AVERAGE(J14,L14,N14)</f>
-        <v>1.0143514658933335</v>
+        <v>1.0110350567466666</v>
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D15" s="11"/>
+      <c r="D15" s="34"/>
       <c r="E15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="7">
+      <c r="F15" s="35">
         <v>0.38450000000000001</v>
       </c>
       <c r="G15" s="5">
-        <f t="shared" ref="G15:G16" si="4">+F15/$F$17</f>
+        <f>+F15/$F$17</f>
         <v>0.19842498555032614</v>
       </c>
       <c r="H15" s="7">
-        <f t="shared" ref="H15:H16" si="5">+F15*(1-$J$5/100)</f>
+        <f>+F15*(1-$J$5/100)</f>
         <v>0.35450899999999996</v>
       </c>
       <c r="I15" s="5">
-        <f t="shared" ref="I15:I16" si="6">H15/$H$17</f>
+        <f t="shared" ref="I15:I16" si="4">H15/$H$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J15" s="7">
-        <f t="shared" ref="J15:J16" si="7">+H15*(1-$K$5/100)</f>
+      <c r="J15" s="37">
+        <f>+H15*(1-$K$5/100)</f>
         <v>0.324021226</v>
       </c>
       <c r="K15" s="5">
-        <f t="shared" ref="K15:K16" si="8">+J15/$J$17</f>
+        <f t="shared" ref="K15:K16" si="5">+J15/$J$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L15" s="7">
-        <f>+$H$23*(1-$K$7/100)</f>
-        <v>0.33682046199999999</v>
+      <c r="L15" s="37">
+        <f>$H$15*(1-$K$7/100)</f>
+        <v>0.33536551399999998</v>
       </c>
       <c r="M15" s="5">
-        <f t="shared" ref="M15:M16" si="9">+L15/$J$25</f>
-        <v>0.19842498555032614</v>
-      </c>
-      <c r="N15" s="7">
-        <f>+$H$31*(1-$K$9/100)</f>
-        <v>0.33219415800000002</v>
+        <f t="shared" ref="M15:M16" si="6">+L15/$J$25</f>
+        <v>0.19756785818293812</v>
+      </c>
+      <c r="N15" s="37">
+        <f>+$H$15*(1-$K$9/100)</f>
+        <v>0.33040238799999994</v>
       </c>
       <c r="O15" s="5">
-        <f t="shared" ref="O15:O17" si="10">+N15/$J$33</f>
-        <v>0.19842498555032617</v>
-      </c>
-      <c r="P15" s="7">
+        <f t="shared" ref="O15:O17" si="7">+N15/$J$33</f>
+        <v>0.19735473212233082</v>
+      </c>
+      <c r="P15" s="4">
         <f>AVERAGE(J15,L15,N15)</f>
-        <v>0.33101194866666667</v>
+        <v>0.32992970933333332</v>
       </c>
     </row>
     <row r="16" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D16" s="11"/>
+      <c r="D16" s="34"/>
       <c r="E16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="7">
+      <c r="F16" s="35">
         <v>0.375</v>
       </c>
       <c r="G16" s="5">
+        <f t="shared" ref="G16" si="8">+F16/$F$17</f>
+        <v>0.19352241763685904</v>
+      </c>
+      <c r="H16" s="7">
+        <f>+F16*(1-$J$5/100)</f>
+        <v>0.34575</v>
+      </c>
+      <c r="I16" s="5">
         <f t="shared" si="4"/>
+        <v>0.19352241763685907</v>
+      </c>
+      <c r="J16" s="37">
+        <f>+H16*(1-$K$5/100)</f>
+        <v>0.3160155</v>
+      </c>
+      <c r="K16" s="5">
+        <f t="shared" si="5"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="H16" s="7">
-        <f t="shared" si="5"/>
-        <v>0.34575</v>
-      </c>
-      <c r="I16" s="5">
+      <c r="L16" s="37">
+        <f>+$H$16*(1-$K$7/100)</f>
+        <v>0.32707949999999997</v>
+      </c>
+      <c r="M16" s="5">
         <f t="shared" si="6"/>
-        <v>0.19352241763685907</v>
-      </c>
-      <c r="J16" s="7">
+        <v>0.19268646766866526</v>
+      </c>
+      <c r="N16" s="37">
+        <f>+$H$16*(1-$K$9/100)</f>
+        <v>0.322239</v>
+      </c>
+      <c r="O16" s="5">
         <f t="shared" si="7"/>
-        <v>0.3160155</v>
-      </c>
-      <c r="K16" s="5">
-        <f t="shared" si="8"/>
-        <v>0.19352241763685904</v>
-      </c>
-      <c r="L16" s="7">
-        <f>+$H$24*(1-$K$7/100)</f>
-        <v>0.32849849999999992</v>
-      </c>
-      <c r="M16" s="5">
+        <v>0.19247860740149306</v>
+      </c>
+      <c r="P16" s="4">
+        <f>AVERAGE(J16,L16,N16)</f>
+        <v>0.32177799999999995</v>
+      </c>
+    </row>
+    <row r="17" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D17" s="34"/>
+      <c r="E17" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F17" s="36">
+        <f t="shared" ref="F17:M17" si="9">SUM(F14:F16)</f>
+        <v>1.9377600000000001</v>
+      </c>
+      <c r="G17" s="6">
         <f t="shared" si="9"/>
-        <v>0.19352241763685901</v>
-      </c>
-      <c r="N16" s="7">
-        <f>+$H$32*(1-$K$9/100)</f>
-        <v>0.32398650000000001</v>
-      </c>
-      <c r="O16" s="5">
-        <f t="shared" si="10"/>
-        <v>0.19352241763685907</v>
-      </c>
-      <c r="P16" s="7">
-        <f>AVERAGE(J16,L16,N16)</f>
-        <v>0.3228335</v>
-      </c>
-    </row>
-    <row r="17" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D17" s="11"/>
-      <c r="E17" s="2" t="s">
+        <v>1</v>
+      </c>
+      <c r="H17" s="8">
+        <f t="shared" si="9"/>
+        <v>1.78661472</v>
+      </c>
+      <c r="I17" s="6">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="J17" s="38">
+        <f>SUM(J14:J16)</f>
+        <v>1.6329658540800001</v>
+      </c>
+      <c r="K17" s="4">
+        <f t="shared" si="9"/>
+        <v>1</v>
+      </c>
+      <c r="L17" s="38">
+        <f t="shared" si="9"/>
+        <v>1.6901375251199999</v>
+      </c>
+      <c r="M17" s="4">
+        <f t="shared" si="9"/>
+        <v>0.99568034557235419</v>
+      </c>
+      <c r="N17" s="38">
+        <f>SUM(N14:N16)</f>
+        <v>1.6651249190399999</v>
+      </c>
+      <c r="O17" s="4">
+        <f t="shared" si="7"/>
+        <v>0.99460625674217906</v>
+      </c>
+      <c r="P17" s="4">
+        <f>AVERAGE(J17,L17,N17)</f>
+        <v>1.66274276608</v>
+      </c>
+    </row>
+    <row r="18" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D18" s="34"/>
+      <c r="E18" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="F17" s="8">
-        <f t="shared" ref="F17:M17" si="11">SUM(F14:F16)</f>
-        <v>1.9377600000000001</v>
-      </c>
-      <c r="G17" s="6">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
-      <c r="H17" s="8">
-        <f t="shared" si="11"/>
-        <v>1.78661472</v>
-      </c>
-      <c r="I17" s="6">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
-      <c r="J17" s="8">
-        <f t="shared" si="11"/>
-        <v>1.6329658540800001</v>
-      </c>
-      <c r="K17" s="4">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
-      <c r="L17" s="8">
-        <f t="shared" si="11"/>
-        <v>1.6974700089599999</v>
-      </c>
-      <c r="M17" s="4">
-        <f t="shared" si="11"/>
-        <v>1</v>
-      </c>
-      <c r="N17" s="8">
-        <f>SUM(N14:N16)</f>
-        <v>1.67415488064</v>
-      </c>
-      <c r="O17" s="4">
-        <f t="shared" si="10"/>
-        <v>1</v>
-      </c>
-      <c r="P17" s="7">
-        <f>AVERAGE(J17,L17,N17)</f>
-        <v>1.66819691456</v>
-      </c>
-    </row>
-    <row r="18" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D18" s="11"/>
-      <c r="E18" s="2" t="s">
-        <v>18</v>
-      </c>
       <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+      <c r="G18" s="2" t="s">
+        <v>2</v>
+      </c>
       <c r="H18" s="9">
         <f>+H17/F17-1</f>
         <v>-7.8000000000000069E-2</v>
@@ -1723,57 +1735,53 @@
       <c r="I18" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J18" s="5">
+      <c r="J18" s="39">
         <f>+J17/I17-1</f>
         <v>0.63296585408000006</v>
       </c>
       <c r="K18" s="2"/>
-      <c r="L18" s="5">
+      <c r="L18" s="39">
         <f>+L17/K17-1</f>
-        <v>0.69747000895999989</v>
+        <v>0.69013752511999993</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="N18" s="5">
+      <c r="N18" s="39">
         <f>+N17/M17-1</f>
-        <v>0.67415488063999995</v>
+        <v>0.67234888831999995</v>
       </c>
       <c r="O18" s="2"/>
       <c r="P18" s="2"/>
     </row>
     <row r="20" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E20" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="F20" s="10"/>
-      <c r="G20" s="10"/>
-      <c r="H20" s="10"/>
-      <c r="I20" s="10"/>
-      <c r="J20" s="10"/>
-      <c r="K20" s="10"/>
-      <c r="L20" s="10"/>
+      <c r="E20" s="22" t="s">
+        <v>23</v>
+      </c>
+      <c r="F20" s="22"/>
+      <c r="G20" s="22"/>
+      <c r="H20" s="22"/>
+      <c r="I20" s="22"/>
+      <c r="J20" s="22"/>
+      <c r="K20" s="22"/>
+      <c r="L20" s="22"/>
     </row>
     <row r="21" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E21" s="2"/>
-      <c r="F21" s="12" t="s">
+      <c r="F21" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="13"/>
-      <c r="H21" s="10" t="s">
+      <c r="G21" s="25"/>
+      <c r="H21" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="10"/>
-      <c r="J21" s="10" t="s">
+      <c r="I21" s="22"/>
+      <c r="J21" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="10"/>
-      <c r="L21" s="23" t="s">
-        <v>23</v>
-      </c>
+      <c r="K21" s="22"/>
+      <c r="L21" s="10"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D22" s="11" t="s">
-        <v>8</v>
-      </c>
+      <c r="D22" s="34"/>
       <c r="E22" s="2" t="s">
         <v>13</v>
       </c>
@@ -1792,7 +1800,7 @@
         <f>H22/$H$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J22" s="7">
+      <c r="J22" s="37">
         <f>+$H$22*(1-$K$7/100)</f>
         <v>1.0321510469599999</v>
       </c>
@@ -1800,13 +1808,10 @@
         <f>+J22/$J$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L22" s="7">
-        <f>AVERAGE(F22,H22,J22)</f>
-        <v>1.1004932689866667</v>
-      </c>
+      <c r="L22" s="7"/>
     </row>
     <row r="23" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D23" s="11"/>
+      <c r="D23" s="34"/>
       <c r="E23" s="2" t="s">
         <v>14</v>
       </c>
@@ -1814,32 +1819,29 @@
         <v>0.38450000000000001</v>
       </c>
       <c r="G23" s="5">
-        <f t="shared" ref="G23:G24" si="12">+F23/$F$25</f>
+        <f t="shared" ref="G23:G24" si="10">+F23/$F$25</f>
         <v>0.19842498555032614</v>
       </c>
       <c r="H23" s="7">
-        <f t="shared" ref="H23:H25" si="13">+F23*(1-$J$7/100)</f>
+        <f t="shared" ref="H23:H25" si="11">+F23*(1-$J$7/100)</f>
         <v>0.356047</v>
       </c>
       <c r="I23" s="5">
         <f>H23/$H$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J23" s="7">
+      <c r="J23" s="37">
         <f>+$H$23*(1-$K$7/100)</f>
         <v>0.33682046199999999</v>
       </c>
       <c r="K23" s="5">
-        <f t="shared" ref="K23:K24" si="14">+J23/$J$25</f>
+        <f t="shared" ref="K23:K24" si="12">+J23/$J$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L23" s="7">
-        <f>AVERAGE(F23,H23,J23)</f>
-        <v>0.35912248733333335</v>
-      </c>
+      <c r="L23" s="7"/>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D24" s="11"/>
+      <c r="D24" s="34"/>
       <c r="E24" s="2" t="s">
         <v>15</v>
       </c>
@@ -1847,68 +1849,62 @@
         <v>0.375</v>
       </c>
       <c r="G24" s="5">
-        <f t="shared" si="12"/>
+        <f t="shared" si="10"/>
         <v>0.19352241763685904</v>
       </c>
       <c r="H24" s="7">
-        <f t="shared" si="13"/>
+        <f t="shared" si="11"/>
         <v>0.34724999999999995</v>
       </c>
       <c r="I24" s="5">
         <f>H24/$H$25</f>
         <v>0.19352241763685901</v>
       </c>
-      <c r="J24" s="7">
+      <c r="J24" s="37">
         <f>+$H$24*(1-$K$7/100)</f>
         <v>0.32849849999999992</v>
       </c>
       <c r="K24" s="5">
-        <f t="shared" si="14"/>
+        <f t="shared" si="12"/>
         <v>0.19352241763685901</v>
       </c>
-      <c r="L24" s="7">
-        <f>AVERAGE(F24,H24,J24)</f>
-        <v>0.35024949999999994</v>
-      </c>
+      <c r="L24" s="7"/>
     </row>
     <row r="25" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D25" s="11"/>
+      <c r="D25" s="34"/>
       <c r="E25" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F25" s="8">
+        <f t="shared" ref="F25:K25" si="13">SUM(F22:F24)</f>
+        <v>1.9377600000000001</v>
+      </c>
+      <c r="G25" s="6">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="H25" s="7">
+        <f t="shared" si="11"/>
+        <v>1.79436576</v>
+      </c>
+      <c r="I25" s="6">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="J25" s="38">
+        <f t="shared" si="13"/>
+        <v>1.6974700089599999</v>
+      </c>
+      <c r="K25" s="4">
+        <f t="shared" si="13"/>
+        <v>1</v>
+      </c>
+      <c r="L25" s="7"/>
+    </row>
+    <row r="26" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="D26" s="34"/>
+      <c r="E26" s="2" t="s">
         <v>17</v>
-      </c>
-      <c r="F25" s="8">
-        <f t="shared" ref="F25:K25" si="15">SUM(F22:F24)</f>
-        <v>1.9377600000000001</v>
-      </c>
-      <c r="G25" s="6">
-        <f t="shared" si="15"/>
-        <v>1</v>
-      </c>
-      <c r="H25" s="7">
-        <f t="shared" si="13"/>
-        <v>1.79436576</v>
-      </c>
-      <c r="I25" s="6">
-        <f t="shared" si="15"/>
-        <v>1</v>
-      </c>
-      <c r="J25" s="8">
-        <f t="shared" si="15"/>
-        <v>1.6974700089599999</v>
-      </c>
-      <c r="K25" s="4">
-        <f t="shared" si="15"/>
-        <v>1</v>
-      </c>
-      <c r="L25" s="7">
-        <f>AVERAGE(F25,H25,J25)</f>
-        <v>1.8098652563200002</v>
-      </c>
-    </row>
-    <row r="26" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D26" s="11"/>
-      <c r="E26" s="2" t="s">
-        <v>18</v>
       </c>
       <c r="F26" s="2"/>
       <c r="G26" s="2" t="s">
@@ -1921,7 +1917,7 @@
       <c r="I26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J26" s="5">
+      <c r="J26" s="39">
         <f>+J25/I25-1</f>
         <v>0.69747000895999989</v>
       </c>
@@ -1929,39 +1925,35 @@
       <c r="L26" s="2"/>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E28" s="12" t="s">
-        <v>25</v>
-      </c>
-      <c r="F28" s="22"/>
-      <c r="G28" s="22"/>
-      <c r="H28" s="22"/>
-      <c r="I28" s="22"/>
-      <c r="J28" s="22"/>
-      <c r="K28" s="22"/>
-      <c r="L28" s="13"/>
+      <c r="E28" s="23" t="s">
+        <v>22</v>
+      </c>
+      <c r="F28" s="24"/>
+      <c r="G28" s="24"/>
+      <c r="H28" s="24"/>
+      <c r="I28" s="24"/>
+      <c r="J28" s="24"/>
+      <c r="K28" s="24"/>
+      <c r="L28" s="25"/>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E29" s="2"/>
-      <c r="F29" s="12" t="s">
+      <c r="F29" s="23" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="13"/>
-      <c r="H29" s="10" t="s">
+      <c r="G29" s="25"/>
+      <c r="H29" s="22" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="10"/>
-      <c r="J29" s="10" t="s">
+      <c r="I29" s="22"/>
+      <c r="J29" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="10"/>
-      <c r="L29" s="23" t="s">
-        <v>23</v>
-      </c>
+      <c r="K29" s="22"/>
+      <c r="L29" s="10"/>
     </row>
     <row r="30" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D30" s="11" t="s">
-        <v>16</v>
-      </c>
+      <c r="D30" s="34"/>
       <c r="E30" s="2" t="s">
         <v>13</v>
       </c>
@@ -1980,7 +1972,7 @@
         <f>H30/$H$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J30" s="7">
+      <c r="J30" s="37">
         <f>+$H$30*(1-$K$9/100)</f>
         <v>1.0179742226399999</v>
       </c>
@@ -1988,13 +1980,10 @@
         <f>+J30/$J$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L30" s="7">
-        <f>AVERAGE(F30,H30,J30)</f>
-        <v>1.0961604142133334</v>
-      </c>
+      <c r="L30" s="7"/>
     </row>
     <row r="31" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D31" s="11"/>
+      <c r="D31" s="34"/>
       <c r="E31" s="2" t="s">
         <v>14</v>
       </c>
@@ -2002,32 +1991,29 @@
         <v>0.38450000000000001</v>
       </c>
       <c r="G31" s="5">
-        <f t="shared" ref="G31:G32" si="16">+F31/$F$33</f>
+        <f t="shared" ref="G31:G32" si="14">+F31/$F$33</f>
         <v>0.19842498555032614</v>
       </c>
       <c r="H31" s="7">
-        <f t="shared" ref="H31:H32" si="17">+F31*(1-$J$9/100)</f>
+        <f t="shared" ref="H31:H32" si="15">+F31*(1-$J$9/100)</f>
         <v>0.35643150000000001</v>
       </c>
       <c r="I31" s="5">
         <f>H31/$H$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J31" s="7">
+      <c r="J31" s="37">
         <f>+$H$31*(1-$K$9/100)</f>
         <v>0.33219415800000002</v>
       </c>
       <c r="K31" s="5">
-        <f t="shared" ref="K31:K33" si="18">+J31/$J$33</f>
+        <f t="shared" ref="K31:K33" si="16">+J31/$J$33</f>
         <v>0.19842498555032617</v>
       </c>
-      <c r="L31" s="7">
-        <f>AVERAGE(F31,H31,J31)</f>
-        <v>0.35770855266666673</v>
-      </c>
+      <c r="L31" s="7"/>
     </row>
     <row r="32" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D32" s="11"/>
+      <c r="D32" s="34"/>
       <c r="E32" s="2" t="s">
         <v>15</v>
       </c>
@@ -2035,34 +2021,31 @@
         <v>0.375</v>
       </c>
       <c r="G32" s="5">
-        <f t="shared" si="16"/>
+        <f t="shared" si="14"/>
         <v>0.19352241763685904</v>
       </c>
       <c r="H32" s="7">
-        <f t="shared" si="17"/>
+        <f t="shared" si="15"/>
         <v>0.34762500000000002</v>
       </c>
       <c r="I32" s="5">
         <f>H32/$H$33</f>
         <v>0.19352241763685904</v>
       </c>
-      <c r="J32" s="7">
+      <c r="J32" s="37">
         <f>+$H$32*(1-$K$9/100)</f>
         <v>0.32398650000000001</v>
       </c>
       <c r="K32" s="5">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="L32" s="7">
-        <f>AVERAGE(F32,H32,J32)</f>
-        <v>0.34887050000000003</v>
-      </c>
+      <c r="L32" s="7"/>
     </row>
     <row r="33" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D33" s="11"/>
+      <c r="D33" s="34"/>
       <c r="E33" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="F33" s="8">
         <f>SUM(F30:F32)</f>
@@ -2080,23 +2063,20 @@
         <f>SUM(I30:I32)</f>
         <v>1</v>
       </c>
-      <c r="J33" s="8">
+      <c r="J33" s="38">
         <f>SUM(J30:J32)</f>
         <v>1.67415488064</v>
       </c>
       <c r="K33" s="4">
-        <f t="shared" si="18"/>
+        <f t="shared" si="16"/>
         <v>1</v>
       </c>
-      <c r="L33" s="7">
-        <f>AVERAGE(F33,H33,J33)</f>
-        <v>1.8027394668800001</v>
-      </c>
+      <c r="L33" s="7"/>
     </row>
     <row r="34" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D34" s="11"/>
+      <c r="D34" s="34"/>
       <c r="E34" s="2" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F34" s="2"/>
       <c r="G34" s="2" t="s">
@@ -2109,22 +2089,33 @@
       <c r="I34" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J34" s="5">
+      <c r="J34" s="39">
         <f>+J33/I33-1</f>
         <v>0.67415488063999995</v>
       </c>
       <c r="K34" s="2"/>
-      <c r="L34" s="24"/>
+      <c r="L34" s="11"/>
     </row>
   </sheetData>
   <mergeCells count="41">
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J12:P12"/>
+    <mergeCell ref="D14:D18"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D22:D26"/>
+    <mergeCell ref="E28:L28"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="E9:E10"/>
@@ -2141,24 +2132,13 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="D30:D34"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D22:D26"/>
-    <mergeCell ref="E28:L28"/>
-    <mergeCell ref="D14:D18"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J12:P12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2174,98 +2154,98 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="C2" s="33">
+      <c r="B2" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="C2" s="18">
         <v>1.2</v>
       </c>
-      <c r="D2" s="26"/>
-      <c r="E2" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="33">
+      <c r="D2" s="13"/>
+      <c r="E2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" s="18">
         <v>0.6</v>
       </c>
-      <c r="G2" s="26"/>
-      <c r="H2" s="32" t="s">
-        <v>29</v>
-      </c>
-      <c r="I2" s="33">
+      <c r="G2" s="13"/>
+      <c r="H2" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="I2" s="18">
         <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="C3" s="34">
+      <c r="B3" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="C3" s="19">
         <f>SQRT(($C$2^2)/3)</f>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E3" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="34">
+      <c r="E3" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="F3" s="19">
         <f>SQRT(($F$2^2)/3)</f>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H3" s="29" t="s">
-        <v>30</v>
-      </c>
-      <c r="I3" s="34">
+      <c r="H3" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="I3" s="19">
         <f>SQRT(($I$2^2)/3)</f>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="C4" s="34">
+      <c r="B4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="19">
         <f t="shared" ref="C4:C5" si="0">SQRT(($C$2^2)/3)</f>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E4" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="34">
+      <c r="E4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="F4" s="19">
         <f t="shared" ref="F4:F5" si="1">SQRT(($F$2^2)/3)</f>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H4" s="29" t="s">
-        <v>31</v>
-      </c>
-      <c r="I4" s="34">
+      <c r="H4" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="19">
         <f t="shared" ref="I4:I5" si="2">SQRT(($I$2^2)/3)</f>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="C5" s="34">
+      <c r="B5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="19">
         <f t="shared" si="0"/>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E5" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="34">
+      <c r="E5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F5" s="19">
         <f t="shared" si="1"/>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H5" s="29" t="s">
-        <v>32</v>
-      </c>
-      <c r="I5" s="34">
+      <c r="H5" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="I5" s="19">
         <f t="shared" si="2"/>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="E12" s="25"/>
+      <c r="E12" s="12"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Guardando cambios de colorimetria y correccion de paquetes
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="720" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D4E38495-5D83-4C02-A15C-130A53967ECC}"/>
+  <xr:revisionPtr revIDLastSave="741" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0903368-7D2F-4EC3-9200-8077735669D3}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
@@ -17,7 +17,7 @@
     <sheet name="CALCULO RECETA" sheetId="1" r:id="rId2"/>
     <sheet name="TOLERANCIA" sheetId="2" r:id="rId3"/>
   </sheets>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="106" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="58">
   <si>
     <t>MEDICIONES</t>
   </si>
@@ -200,6 +200,18 @@
   </si>
   <si>
     <t>Promedio Chroma</t>
+  </si>
+  <si>
+    <t>Lightness (D65)</t>
+  </si>
+  <si>
+    <t>Lightness (TL84)</t>
+  </si>
+  <si>
+    <t>Lightness (A o CWF)</t>
+  </si>
+  <si>
+    <t>Promedio Lightness</t>
   </si>
 </sst>
 </file>
@@ -209,7 +221,7 @@
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
-    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="166" formatCode="0.00000"/>
   </numFmts>
   <fonts count="9" x14ac:knownFonts="1">
     <font>
@@ -298,7 +310,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="10">
     <border>
       <left/>
       <right/>
@@ -376,12 +388,47 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="43">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -430,6 +477,21 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -442,12 +504,21 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -473,21 +544,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="167" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -506,6 +562,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -862,10 +922,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="22" t="s">
+      <c r="H2" s="27" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="22"/>
+      <c r="I2" s="27"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1046,7 +1106,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="20" t="s">
+      <c r="B14" s="25" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="16" t="s">
@@ -1061,45 +1121,45 @@
       <c r="F14" s="16">
         <v>-3.6</v>
       </c>
-      <c r="G14" s="20">
+      <c r="G14" s="25">
         <f>+D15-D14</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H14" s="20">
+      <c r="H14" s="25">
         <f>+E15-E14</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I14" s="20">
+      <c r="I14" s="25">
         <f>+F15-F14</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J14" s="20">
+      <c r="J14" s="25">
         <f>+ABS(G14)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K14" s="20">
+      <c r="K14" s="25">
         <f>+ABS(H14)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L14" s="20">
+      <c r="L14" s="25">
         <f>+ABS(I14)</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="M14" s="21">
+      <c r="M14" s="26">
         <f>+K14/F14</f>
         <v>-0.34166666666666679</v>
       </c>
-      <c r="N14" s="21">
+      <c r="N14" s="26">
         <f>+K14/E14</f>
         <v>-8.6376404494382053E-2</v>
       </c>
-      <c r="O14" s="21">
+      <c r="O14" s="26">
         <f>+L14/F14</f>
         <v>-3.611111111111108E-2</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="20"/>
+      <c r="B15" s="25"/>
       <c r="C15" s="16" t="s">
         <v>31</v>
       </c>
@@ -1112,18 +1172,18 @@
       <c r="F15" s="16">
         <v>-3.47</v>
       </c>
-      <c r="G15" s="20"/>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="21"/>
-      <c r="N15" s="21"/>
-      <c r="O15" s="21"/>
+      <c r="G15" s="25"/>
+      <c r="H15" s="25"/>
+      <c r="I15" s="25"/>
+      <c r="J15" s="25"/>
+      <c r="K15" s="25"/>
+      <c r="L15" s="25"/>
+      <c r="M15" s="26"/>
+      <c r="N15" s="26"/>
+      <c r="O15" s="26"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="20" t="s">
+      <c r="B16" s="25" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="16" t="s">
@@ -1138,45 +1198,45 @@
       <c r="F16" s="16">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G16" s="20">
+      <c r="G16" s="25">
         <f>+D17-D16</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H16" s="20">
+      <c r="H16" s="25">
         <f t="shared" ref="H16:I16" si="2">+E17-E16</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I16" s="20">
+      <c r="I16" s="25">
         <f t="shared" si="2"/>
         <v>-9.39</v>
       </c>
-      <c r="J16" s="20">
+      <c r="J16" s="25">
         <f t="shared" ref="J16:L16" si="3">+ABS(G16)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K16" s="20">
+      <c r="K16" s="25">
         <f t="shared" si="3"/>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L16" s="20">
+      <c r="L16" s="25">
         <f t="shared" si="3"/>
         <v>9.39</v>
       </c>
-      <c r="M16" s="21">
+      <c r="M16" s="26">
         <f>+J16/D16</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="N16" s="21">
+      <c r="N16" s="26">
         <f>+K16/E16</f>
         <v>-5.7165231010180145E-2</v>
       </c>
-      <c r="O16" s="21">
+      <c r="O16" s="26">
         <f t="shared" ref="O16" si="4">+L16/F16</f>
         <v>1.8557312252964429</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="20"/>
+      <c r="B17" s="25"/>
       <c r="C17" s="16" t="s">
         <v>31</v>
       </c>
@@ -1189,18 +1249,18 @@
       <c r="F17" s="16">
         <v>-4.33</v>
       </c>
-      <c r="G17" s="20"/>
-      <c r="H17" s="20"/>
-      <c r="I17" s="20"/>
-      <c r="J17" s="20"/>
-      <c r="K17" s="20"/>
-      <c r="L17" s="20"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="20" t="s">
+      <c r="B18" s="25" t="s">
         <v>41</v>
       </c>
       <c r="C18" s="16" t="s">
@@ -1215,45 +1275,45 @@
       <c r="F18" s="16">
         <v>7.39</v>
       </c>
-      <c r="G18" s="20">
+      <c r="G18" s="25">
         <f>+D19-D18</f>
         <v>-4</v>
       </c>
-      <c r="H18" s="20">
+      <c r="H18" s="25">
         <f t="shared" ref="H18:I18" si="5">+E19-E18</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I18" s="20">
+      <c r="I18" s="25">
         <f t="shared" si="5"/>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J18" s="20">
+      <c r="J18" s="25">
         <f t="shared" ref="J18:L18" si="6">+ABS(G18)</f>
         <v>4</v>
       </c>
-      <c r="K18" s="20">
+      <c r="K18" s="25">
         <f t="shared" si="6"/>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L18" s="20">
+      <c r="L18" s="25">
         <f t="shared" si="6"/>
         <v>0.58999999999999986</v>
       </c>
-      <c r="M18" s="21">
+      <c r="M18" s="26">
         <f>+J18/D18</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="N18" s="21">
+      <c r="N18" s="26">
         <f>+K18/E18</f>
         <v>-5.7884231536926095E-2</v>
       </c>
-      <c r="O18" s="21">
+      <c r="O18" s="26">
         <f t="shared" ref="O18" si="7">+L18/F18</f>
         <v>7.9837618403247615E-2</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="20"/>
+      <c r="B19" s="25"/>
       <c r="C19" s="16" t="s">
         <v>31</v>
       </c>
@@ -1266,15 +1326,15 @@
       <c r="F19" s="16">
         <v>6.8</v>
       </c>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="21"/>
-      <c r="N19" s="21"/>
-      <c r="O19" s="21"/>
+      <c r="G19" s="25"/>
+      <c r="H19" s="25"/>
+      <c r="I19" s="25"/>
+      <c r="J19" s="25"/>
+      <c r="K19" s="25"/>
+      <c r="L19" s="25"/>
+      <c r="M19" s="26"/>
+      <c r="N19" s="26"/>
+      <c r="O19" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="31">
@@ -1316,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F05E7DF8-3200-46CC-8D04-8DEE3E3EFF1F}">
-  <dimension ref="D2:P34"/>
+  <dimension ref="D2:P42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="4" width="9.140625" style="1"/>
@@ -1328,22 +1388,24 @@
     <col min="10" max="10" width="19.140625" style="1" customWidth="1"/>
     <col min="11" max="11" width="18.28515625" style="1" customWidth="1"/>
     <col min="12" max="12" width="10.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="13" max="15" width="9.140625" style="1"/>
+    <col min="13" max="13" width="9.140625" style="1"/>
+    <col min="14" max="14" width="17" style="1" customWidth="1"/>
+    <col min="15" max="15" width="9.140625" style="1"/>
     <col min="16" max="16" width="17.28515625" style="1" customWidth="1"/>
     <col min="17" max="16384" width="9.140625" style="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E2" s="27" t="s">
+      <c r="E2" s="35" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="27"/>
-      <c r="G2" s="27"/>
-      <c r="H2" s="27"/>
-      <c r="I2" s="27"/>
-      <c r="N2" s="33"/>
-      <c r="O2" s="33"/>
-      <c r="P2" s="33"/>
+      <c r="F2" s="35"/>
+      <c r="G2" s="35"/>
+      <c r="H2" s="35"/>
+      <c r="I2" s="35"/>
+      <c r="N2" s="41"/>
+      <c r="O2" s="41"/>
+      <c r="P2" s="41"/>
     </row>
     <row r="3" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E3" s="2"/>
@@ -1376,158 +1438,158 @@
       </c>
     </row>
     <row r="5" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="26" t="s">
+      <c r="E5" s="34" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="31">
+      <c r="F5" s="39">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="31">
+      <c r="G5" s="39">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="32">
+      <c r="H5" s="40">
         <v>0.17</v>
       </c>
-      <c r="I5" s="30">
+      <c r="I5" s="38">
         <v>1.17</v>
       </c>
-      <c r="J5" s="26">
+      <c r="J5" s="34">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="26">
+      <c r="K5" s="34">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="26"/>
-      <c r="F6" s="31"/>
-      <c r="G6" s="31"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="30"/>
-      <c r="J6" s="26"/>
-      <c r="K6" s="26"/>
+      <c r="E6" s="34"/>
+      <c r="F6" s="39"/>
+      <c r="G6" s="39"/>
+      <c r="H6" s="40"/>
+      <c r="I6" s="38"/>
+      <c r="J6" s="34"/>
+      <c r="K6" s="34"/>
       <c r="O6" s="3"/>
     </row>
     <row r="7" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E7" s="22" t="s">
+      <c r="E7" s="27" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="28">
+      <c r="F7" s="36">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="29">
+      <c r="G7" s="37">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="29">
+      <c r="H7" s="37">
         <v>0.1</v>
       </c>
-      <c r="I7" s="22">
+      <c r="I7" s="27">
         <v>0.92</v>
       </c>
-      <c r="J7" s="22">
+      <c r="J7" s="27">
         <f t="shared" ref="J7" si="0">+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="22">
+      <c r="K7" s="27">
         <f t="shared" ref="K7" si="1">+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E8" s="22"/>
-      <c r="F8" s="28"/>
-      <c r="G8" s="29"/>
-      <c r="H8" s="29"/>
-      <c r="I8" s="22"/>
-      <c r="J8" s="22"/>
-      <c r="K8" s="22"/>
+      <c r="E8" s="27"/>
+      <c r="F8" s="36"/>
+      <c r="G8" s="37"/>
+      <c r="H8" s="37"/>
+      <c r="I8" s="27"/>
+      <c r="J8" s="27"/>
+      <c r="K8" s="27"/>
     </row>
     <row r="9" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E9" s="22" t="s">
+      <c r="E9" s="27" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="28">
+      <c r="F9" s="36">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="29">
+      <c r="G9" s="37">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="29">
+      <c r="H9" s="37">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="22">
+      <c r="I9" s="27">
         <v>1.01</v>
       </c>
-      <c r="J9" s="22">
+      <c r="J9" s="27">
         <f t="shared" ref="J9" si="2">+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="22">
+      <c r="K9" s="27">
         <f t="shared" ref="K9" si="3">+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="10" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E10" s="22"/>
-      <c r="F10" s="28"/>
-      <c r="G10" s="29"/>
-      <c r="H10" s="29"/>
-      <c r="I10" s="22"/>
-      <c r="J10" s="22"/>
-      <c r="K10" s="22"/>
+      <c r="E10" s="27"/>
+      <c r="F10" s="36"/>
+      <c r="G10" s="37"/>
+      <c r="H10" s="37"/>
+      <c r="I10" s="27"/>
+      <c r="J10" s="27"/>
+      <c r="K10" s="27"/>
     </row>
     <row r="12" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E12" s="23" t="s">
+      <c r="E12" s="28" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="24"/>
-      <c r="G12" s="24"/>
-      <c r="H12" s="24"/>
-      <c r="I12" s="25"/>
-      <c r="J12" s="23" t="s">
+      <c r="F12" s="33"/>
+      <c r="G12" s="33"/>
+      <c r="H12" s="33"/>
+      <c r="I12" s="29"/>
+      <c r="J12" s="28" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="24"/>
-      <c r="L12" s="24"/>
-      <c r="M12" s="24"/>
-      <c r="N12" s="24"/>
-      <c r="O12" s="24"/>
-      <c r="P12" s="25"/>
+      <c r="K12" s="33"/>
+      <c r="L12" s="33"/>
+      <c r="M12" s="33"/>
+      <c r="N12" s="33"/>
+      <c r="O12" s="33"/>
+      <c r="P12" s="29"/>
     </row>
     <row r="13" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E13" s="2"/>
-      <c r="F13" s="23" t="s">
+      <c r="F13" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="25"/>
-      <c r="H13" s="22" t="s">
+      <c r="G13" s="29"/>
+      <c r="H13" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="22"/>
-      <c r="J13" s="22" t="s">
+      <c r="I13" s="27"/>
+      <c r="J13" s="27" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="22"/>
-      <c r="L13" s="22" t="s">
+      <c r="K13" s="27"/>
+      <c r="L13" s="27" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="22"/>
-      <c r="N13" s="22" t="s">
+      <c r="M13" s="27"/>
+      <c r="N13" s="27" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="22"/>
+      <c r="O13" s="27"/>
       <c r="P13" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D14" s="34"/>
+      <c r="D14" s="42"/>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="35">
+      <c r="F14" s="20">
         <v>1.1782600000000001</v>
       </c>
       <c r="G14" s="5">
@@ -1542,7 +1604,7 @@
         <f>H14/$H$17</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J14" s="37">
+      <c r="J14" s="22">
         <f>+H14*(1-$K$5/100)</f>
         <v>0.99292912808000011</v>
       </c>
@@ -1550,7 +1612,7 @@
         <f>+J14/$J$17</f>
         <v>0.60805259681281487</v>
       </c>
-      <c r="L14" s="37">
+      <c r="L14" s="22">
         <f>+$H$14*(1-$K$7/100)</f>
         <v>1.0276925111199999</v>
       </c>
@@ -1558,7 +1620,7 @@
         <f>+L14/$J$25</f>
         <v>0.60542601972075083</v>
       </c>
-      <c r="N14" s="37">
+      <c r="N14" s="22">
         <f>+$H$14*(1-$K$9/100)</f>
         <v>1.01248353104</v>
       </c>
@@ -1572,11 +1634,11 @@
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D15" s="34"/>
+      <c r="D15" s="42"/>
       <c r="E15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="35">
+      <c r="F15" s="20">
         <v>0.38450000000000001</v>
       </c>
       <c r="G15" s="5">
@@ -1591,7 +1653,7 @@
         <f t="shared" ref="I15:I16" si="4">H15/$H$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J15" s="37">
+      <c r="J15" s="22">
         <f>+H15*(1-$K$5/100)</f>
         <v>0.324021226</v>
       </c>
@@ -1599,7 +1661,7 @@
         <f t="shared" ref="K15:K16" si="5">+J15/$J$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L15" s="37">
+      <c r="L15" s="22">
         <f>$H$15*(1-$K$7/100)</f>
         <v>0.33536551399999998</v>
       </c>
@@ -1607,7 +1669,7 @@
         <f t="shared" ref="M15:M16" si="6">+L15/$J$25</f>
         <v>0.19756785818293812</v>
       </c>
-      <c r="N15" s="37">
+      <c r="N15" s="22">
         <f>+$H$15*(1-$K$9/100)</f>
         <v>0.33040238799999994</v>
       </c>
@@ -1621,11 +1683,11 @@
       </c>
     </row>
     <row r="16" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D16" s="34"/>
+      <c r="D16" s="42"/>
       <c r="E16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="35">
+      <c r="F16" s="20">
         <v>0.375</v>
       </c>
       <c r="G16" s="5">
@@ -1640,7 +1702,7 @@
         <f t="shared" si="4"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="J16" s="37">
+      <c r="J16" s="22">
         <f>+H16*(1-$K$5/100)</f>
         <v>0.3160155</v>
       </c>
@@ -1648,7 +1710,7 @@
         <f t="shared" si="5"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="L16" s="37">
+      <c r="L16" s="22">
         <f>+$H$16*(1-$K$7/100)</f>
         <v>0.32707949999999997</v>
       </c>
@@ -1656,7 +1718,7 @@
         <f t="shared" si="6"/>
         <v>0.19268646766866526</v>
       </c>
-      <c r="N16" s="37">
+      <c r="N16" s="22">
         <f>+$H$16*(1-$K$9/100)</f>
         <v>0.322239</v>
       </c>
@@ -1670,11 +1732,11 @@
       </c>
     </row>
     <row r="17" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D17" s="34"/>
+      <c r="D17" s="42"/>
       <c r="E17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="36">
+      <c r="F17" s="21">
         <f t="shared" ref="F17:M17" si="9">SUM(F14:F16)</f>
         <v>1.9377600000000001</v>
       </c>
@@ -1690,7 +1752,7 @@
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="J17" s="38">
+      <c r="J17" s="23">
         <f>SUM(J14:J16)</f>
         <v>1.6329658540800001</v>
       </c>
@@ -1698,7 +1760,7 @@
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="L17" s="38">
+      <c r="L17" s="23">
         <f t="shared" si="9"/>
         <v>1.6901375251199999</v>
       </c>
@@ -1706,7 +1768,7 @@
         <f t="shared" si="9"/>
         <v>0.99568034557235419</v>
       </c>
-      <c r="N17" s="38">
+      <c r="N17" s="23">
         <f>SUM(N14:N16)</f>
         <v>1.6651249190399999</v>
       </c>
@@ -1720,7 +1782,7 @@
       </c>
     </row>
     <row r="18" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D18" s="34"/>
+      <c r="D18" s="42"/>
       <c r="E18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1735,17 +1797,17 @@
       <c r="I18" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J18" s="39">
+      <c r="J18" s="24">
         <f>+J17/I17-1</f>
         <v>0.63296585408000006</v>
       </c>
       <c r="K18" s="2"/>
-      <c r="L18" s="39">
+      <c r="L18" s="24">
         <f>+L17/K17-1</f>
         <v>0.69013752511999993</v>
       </c>
       <c r="M18" s="2"/>
-      <c r="N18" s="39">
+      <c r="N18" s="24">
         <f>+N17/M17-1</f>
         <v>0.67234888831999995</v>
       </c>
@@ -1753,35 +1815,35 @@
       <c r="P18" s="2"/>
     </row>
     <row r="20" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E20" s="22" t="s">
+      <c r="E20" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="22"/>
-      <c r="G20" s="22"/>
-      <c r="H20" s="22"/>
-      <c r="I20" s="22"/>
-      <c r="J20" s="22"/>
-      <c r="K20" s="22"/>
-      <c r="L20" s="22"/>
+      <c r="F20" s="27"/>
+      <c r="G20" s="27"/>
+      <c r="H20" s="27"/>
+      <c r="I20" s="27"/>
+      <c r="J20" s="27"/>
+      <c r="K20" s="27"/>
+      <c r="L20" s="27"/>
     </row>
     <row r="21" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E21" s="2"/>
-      <c r="F21" s="23" t="s">
+      <c r="F21" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="25"/>
-      <c r="H21" s="22" t="s">
+      <c r="G21" s="29"/>
+      <c r="H21" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="22"/>
-      <c r="J21" s="22" t="s">
+      <c r="I21" s="27"/>
+      <c r="J21" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="22"/>
+      <c r="K21" s="27"/>
       <c r="L21" s="10"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D22" s="34"/>
+      <c r="D22" s="42"/>
       <c r="E22" s="2" t="s">
         <v>13</v>
       </c>
@@ -1800,7 +1862,7 @@
         <f>H22/$H$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J22" s="37">
+      <c r="J22" s="22">
         <f>+$H$22*(1-$K$7/100)</f>
         <v>1.0321510469599999</v>
       </c>
@@ -1811,7 +1873,7 @@
       <c r="L22" s="7"/>
     </row>
     <row r="23" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D23" s="34"/>
+      <c r="D23" s="42"/>
       <c r="E23" s="2" t="s">
         <v>14</v>
       </c>
@@ -1830,7 +1892,7 @@
         <f>H23/$H$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J23" s="37">
+      <c r="J23" s="22">
         <f>+$H$23*(1-$K$7/100)</f>
         <v>0.33682046199999999</v>
       </c>
@@ -1841,7 +1903,7 @@
       <c r="L23" s="7"/>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D24" s="34"/>
+      <c r="D24" s="42"/>
       <c r="E24" s="2" t="s">
         <v>15</v>
       </c>
@@ -1860,7 +1922,7 @@
         <f>H24/$H$25</f>
         <v>0.19352241763685901</v>
       </c>
-      <c r="J24" s="37">
+      <c r="J24" s="22">
         <f>+$H$24*(1-$K$7/100)</f>
         <v>0.32849849999999992</v>
       </c>
@@ -1871,7 +1933,7 @@
       <c r="L24" s="7"/>
     </row>
     <row r="25" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D25" s="34"/>
+      <c r="D25" s="42"/>
       <c r="E25" s="2" t="s">
         <v>16</v>
       </c>
@@ -1891,7 +1953,7 @@
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="J25" s="38">
+      <c r="J25" s="23">
         <f t="shared" si="13"/>
         <v>1.6974700089599999</v>
       </c>
@@ -1902,7 +1964,7 @@
       <c r="L25" s="7"/>
     </row>
     <row r="26" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D26" s="34"/>
+      <c r="D26" s="42"/>
       <c r="E26" s="2" t="s">
         <v>17</v>
       </c>
@@ -1917,7 +1979,7 @@
       <c r="I26" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J26" s="39">
+      <c r="J26" s="24">
         <f>+J25/I25-1</f>
         <v>0.69747000895999989</v>
       </c>
@@ -1925,35 +1987,35 @@
       <c r="L26" s="2"/>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E28" s="23" t="s">
+      <c r="E28" s="28" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="24"/>
-      <c r="G28" s="24"/>
-      <c r="H28" s="24"/>
-      <c r="I28" s="24"/>
-      <c r="J28" s="24"/>
-      <c r="K28" s="24"/>
-      <c r="L28" s="25"/>
+      <c r="F28" s="33"/>
+      <c r="G28" s="33"/>
+      <c r="H28" s="33"/>
+      <c r="I28" s="33"/>
+      <c r="J28" s="33"/>
+      <c r="K28" s="33"/>
+      <c r="L28" s="29"/>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E29" s="2"/>
-      <c r="F29" s="23" t="s">
+      <c r="F29" s="28" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="25"/>
-      <c r="H29" s="22" t="s">
+      <c r="G29" s="29"/>
+      <c r="H29" s="27" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="22"/>
-      <c r="J29" s="22" t="s">
+      <c r="I29" s="27"/>
+      <c r="J29" s="27" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="22"/>
+      <c r="K29" s="27"/>
       <c r="L29" s="10"/>
     </row>
     <row r="30" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D30" s="34"/>
+      <c r="D30" s="42"/>
       <c r="E30" s="2" t="s">
         <v>13</v>
       </c>
@@ -1972,7 +2034,7 @@
         <f>H30/$H$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J30" s="37">
+      <c r="J30" s="22">
         <f>+$H$30*(1-$K$9/100)</f>
         <v>1.0179742226399999</v>
       </c>
@@ -1983,7 +2045,7 @@
       <c r="L30" s="7"/>
     </row>
     <row r="31" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D31" s="34"/>
+      <c r="D31" s="42"/>
       <c r="E31" s="2" t="s">
         <v>14</v>
       </c>
@@ -2002,7 +2064,7 @@
         <f>H31/$H$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J31" s="37">
+      <c r="J31" s="22">
         <f>+$H$31*(1-$K$9/100)</f>
         <v>0.33219415800000002</v>
       </c>
@@ -2013,7 +2075,7 @@
       <c r="L31" s="7"/>
     </row>
     <row r="32" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D32" s="34"/>
+      <c r="D32" s="42"/>
       <c r="E32" s="2" t="s">
         <v>15</v>
       </c>
@@ -2032,7 +2094,7 @@
         <f>H32/$H$33</f>
         <v>0.19352241763685904</v>
       </c>
-      <c r="J32" s="37">
+      <c r="J32" s="22">
         <f>+$H$32*(1-$K$9/100)</f>
         <v>0.32398650000000001</v>
       </c>
@@ -2042,8 +2104,8 @@
       </c>
       <c r="L32" s="7"/>
     </row>
-    <row r="33" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D33" s="34"/>
+    <row r="33" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D33" s="42"/>
       <c r="E33" s="2" t="s">
         <v>16</v>
       </c>
@@ -2063,7 +2125,7 @@
         <f>SUM(I30:I32)</f>
         <v>1</v>
       </c>
-      <c r="J33" s="38">
+      <c r="J33" s="23">
         <f>SUM(J30:J32)</f>
         <v>1.67415488064</v>
       </c>
@@ -2073,8 +2135,8 @@
       </c>
       <c r="L33" s="7"/>
     </row>
-    <row r="34" spans="4:12" x14ac:dyDescent="0.25">
-      <c r="D34" s="34"/>
+    <row r="34" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="D34" s="42"/>
       <c r="E34" s="2" t="s">
         <v>17</v>
       </c>
@@ -2089,15 +2151,237 @@
       <c r="I34" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J34" s="39">
+      <c r="J34" s="24">
         <f>+J33/I33-1</f>
         <v>0.67415488063999995</v>
       </c>
       <c r="K34" s="2"/>
       <c r="L34" s="11"/>
     </row>
+    <row r="36" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E36" s="27" t="s">
+        <v>24</v>
+      </c>
+      <c r="F36" s="27"/>
+      <c r="G36" s="27"/>
+      <c r="H36" s="27" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" s="27"/>
+      <c r="J36" s="27"/>
+      <c r="K36" s="27"/>
+      <c r="L36" s="27"/>
+      <c r="M36" s="27"/>
+      <c r="N36" s="27"/>
+    </row>
+    <row r="37" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E37" s="2"/>
+      <c r="F37" s="28" t="s">
+        <v>10</v>
+      </c>
+      <c r="G37" s="29"/>
+      <c r="H37" s="30" t="s">
+        <v>54</v>
+      </c>
+      <c r="I37" s="30"/>
+      <c r="J37" s="30" t="s">
+        <v>55</v>
+      </c>
+      <c r="K37" s="30"/>
+      <c r="L37" s="31" t="s">
+        <v>56</v>
+      </c>
+      <c r="M37" s="32"/>
+      <c r="N37" s="2" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="38" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E38" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="7">
+        <v>1.1782600000000001</v>
+      </c>
+      <c r="G38" s="5">
+        <f>+F38/$F$17</f>
+        <v>0.60805259681281476</v>
+      </c>
+      <c r="H38" s="7">
+        <f>+F38*(1-$J$5/100)</f>
+        <v>1.08635572</v>
+      </c>
+      <c r="I38" s="5">
+        <f>H38/$H$17</f>
+        <v>0.60805259681281476</v>
+      </c>
+      <c r="J38" s="7">
+        <f>+$F$22*(1-$J$7/100)</f>
+        <v>1.09106876</v>
+      </c>
+      <c r="K38" s="5">
+        <f>J38/$H$25</f>
+        <v>0.60805259681281476</v>
+      </c>
+      <c r="L38" s="7">
+        <f>+$F$30*(1-$J$9/100)</f>
+        <v>1.0922470200000001</v>
+      </c>
+      <c r="M38" s="5">
+        <f>$H$30/$H$33</f>
+        <v>0.60805259681281476</v>
+      </c>
+      <c r="N38" s="4">
+        <f xml:space="preserve"> AVERAGE(H38,J38,L38)</f>
+        <v>1.0898905000000001</v>
+      </c>
+    </row>
+    <row r="39" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E39" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F39" s="7">
+        <v>0.38450000000000001</v>
+      </c>
+      <c r="G39" s="5">
+        <f>+F39/$F$17</f>
+        <v>0.19842498555032614</v>
+      </c>
+      <c r="H39" s="7">
+        <f>+F39*(1-$J$5/100)</f>
+        <v>0.35450899999999996</v>
+      </c>
+      <c r="I39" s="5">
+        <f t="shared" ref="I39:I40" si="17">H39/$H$17</f>
+        <v>0.19842498555032614</v>
+      </c>
+      <c r="J39" s="7">
+        <f>+$F$23*(1-$J$7/100)</f>
+        <v>0.356047</v>
+      </c>
+      <c r="K39" s="5">
+        <f>J39/$H$25</f>
+        <v>0.19842498555032614</v>
+      </c>
+      <c r="L39" s="7">
+        <f>+$F$31*(1-$J$9/100)</f>
+        <v>0.35643150000000001</v>
+      </c>
+      <c r="M39" s="5">
+        <f>$H$31/$H$33</f>
+        <v>0.19842498555032614</v>
+      </c>
+      <c r="N39" s="4">
+        <f t="shared" ref="N39:N41" si="18" xml:space="preserve"> AVERAGE(H39,J39,L39)</f>
+        <v>0.35566249999999999</v>
+      </c>
+    </row>
+    <row r="40" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E40" s="2" t="s">
+        <v>15</v>
+      </c>
+      <c r="F40" s="7">
+        <v>0.375</v>
+      </c>
+      <c r="G40" s="5">
+        <f t="shared" ref="G40" si="19">+F40/$F$17</f>
+        <v>0.19352241763685904</v>
+      </c>
+      <c r="H40" s="7">
+        <f>+F40*(1-$J$5/100)</f>
+        <v>0.34575</v>
+      </c>
+      <c r="I40" s="5">
+        <f t="shared" si="17"/>
+        <v>0.19352241763685907</v>
+      </c>
+      <c r="J40" s="7">
+        <f>+$F$24*(1-$J$7/100)</f>
+        <v>0.34724999999999995</v>
+      </c>
+      <c r="K40" s="5">
+        <f>J40/$H$25</f>
+        <v>0.19352241763685901</v>
+      </c>
+      <c r="L40" s="7">
+        <f>+$F$32*(1-$J$9/100)</f>
+        <v>0.34762500000000002</v>
+      </c>
+      <c r="M40" s="5">
+        <f>$H$32/$H$33</f>
+        <v>0.19352241763685904</v>
+      </c>
+      <c r="N40" s="4">
+        <f t="shared" si="18"/>
+        <v>0.34687499999999999</v>
+      </c>
+    </row>
+    <row r="41" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E41" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F41" s="8">
+        <f t="shared" ref="F41:I41" si="20">SUM(F38:F40)</f>
+        <v>1.9377600000000001</v>
+      </c>
+      <c r="G41" s="6">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="H41" s="8">
+        <f t="shared" si="20"/>
+        <v>1.78661472</v>
+      </c>
+      <c r="I41" s="6">
+        <f t="shared" si="20"/>
+        <v>1</v>
+      </c>
+      <c r="J41" s="7">
+        <f>+$F$25*(1-$J$7/100)</f>
+        <v>1.79436576</v>
+      </c>
+      <c r="K41" s="6">
+        <f t="shared" ref="K41" si="21">SUM(K38:K40)</f>
+        <v>1</v>
+      </c>
+      <c r="L41" s="8">
+        <f>SUM(L38:L40)</f>
+        <v>1.7963035200000002</v>
+      </c>
+      <c r="M41" s="6">
+        <f>SUM(M38:M40)</f>
+        <v>1</v>
+      </c>
+      <c r="N41" s="4">
+        <f t="shared" si="18"/>
+        <v>1.7924280000000001</v>
+      </c>
+    </row>
+    <row r="42" spans="4:14" x14ac:dyDescent="0.25">
+      <c r="E42" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F42" s="2"/>
+      <c r="G42" s="2"/>
+      <c r="H42" s="9">
+        <f ca="1">+$H$42/$F$42-1</f>
+        <v>-7.8000000000000069E-2</v>
+      </c>
+      <c r="I42" s="2"/>
+      <c r="J42" s="5">
+        <f>+$H$25/$F$25-1</f>
+        <v>-7.4000000000000066E-2</v>
+      </c>
+      <c r="K42" s="2"/>
+      <c r="L42" s="5">
+        <f>+$H$33/$F$33-1</f>
+        <v>-7.2999999999999954E-2</v>
+      </c>
+      <c r="M42" s="2"/>
+      <c r="N42" s="7"/>
+    </row>
   </sheetData>
-  <mergeCells count="41">
+  <mergeCells count="47">
     <mergeCell ref="D14:D18"/>
     <mergeCell ref="F29:G29"/>
     <mergeCell ref="H29:I29"/>
@@ -2139,6 +2423,12 @@
     <mergeCell ref="H13:I13"/>
     <mergeCell ref="J13:K13"/>
     <mergeCell ref="J12:P12"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="H36:N36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Integración de ColorimetriaAPI: Controladores de diagnóstico y servicios autónomos
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="741" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F0903368-7D2F-4EC3-9200-8077735669D3}"/>
+  <xr:revisionPtr revIDLastSave="748" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4C7BBB31-40A2-4B6E-97D7-E46E57C4AB0E}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="1" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
@@ -305,7 +305,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="2" tint="-9.9978637043366805E-2"/>
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -428,7 +428,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="43">
+  <cellXfs count="53">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -459,9 +459,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -483,15 +480,6 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -501,12 +489,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -516,34 +534,46 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -922,10 +952,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="27" t="s">
+      <c r="H2" s="23" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="27"/>
+      <c r="I2" s="23"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -937,17 +967,17 @@
       <c r="C3" s="2">
         <v>80.680000000000007</v>
       </c>
-      <c r="D3" s="14">
+      <c r="D3" s="13">
         <f>+C3-B3</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="E3" s="14">
+      <c r="E3" s="13">
         <f>+ABS(D3)</f>
         <v>2.1499999999999915</v>
       </c>
       <c r="F3" s="1"/>
       <c r="G3" s="1"/>
-      <c r="H3" s="15">
+      <c r="H3" s="14">
         <f>+E3/B3</f>
         <v>2.5956778944826651E-2</v>
       </c>
@@ -965,17 +995,17 @@
       <c r="C4" s="2">
         <v>-13.01</v>
       </c>
-      <c r="D4" s="14">
+      <c r="D4" s="13">
         <f t="shared" ref="D4:D5" si="0">+C4-B4</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="E4" s="14">
+      <c r="E4" s="13">
         <f>+ABS(D4)</f>
         <v>1.2300000000000004</v>
       </c>
       <c r="F4" s="1"/>
       <c r="G4" s="1"/>
-      <c r="H4" s="15">
+      <c r="H4" s="14">
         <f>+E4/B4</f>
         <v>-8.6376404494382053E-2</v>
       </c>
@@ -993,17 +1023,17 @@
       <c r="C5" s="2">
         <v>-3.47</v>
       </c>
-      <c r="D5" s="14">
+      <c r="D5" s="13">
         <f t="shared" si="0"/>
         <v>-7.07</v>
       </c>
-      <c r="E5" s="14">
+      <c r="E5" s="13">
         <f>+ABS(D5)</f>
         <v>7.07</v>
       </c>
       <c r="F5" s="1"/>
       <c r="G5" s="1"/>
-      <c r="H5" s="15">
+      <c r="H5" s="14">
         <f t="shared" ref="H5" si="1">+E5/B5</f>
         <v>1.963888888888889</v>
       </c>
@@ -1012,347 +1042,332 @@
       </c>
     </row>
     <row r="8" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B8" s="16"/>
-      <c r="C8" s="16" t="s">
+      <c r="B8" s="15"/>
+      <c r="C8" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="D8" s="16" t="s">
+      <c r="D8" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="E8" s="16" t="s">
+      <c r="E8" s="15" t="s">
         <v>42</v>
       </c>
     </row>
     <row r="9" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B9" s="16" t="s">
+      <c r="B9" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="C9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D9" s="16" t="s">
+      <c r="D9" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E9" s="16" t="s">
+      <c r="E9" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="10" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B10" s="16" t="s">
+      <c r="B10" s="15" t="s">
         <v>8</v>
       </c>
-      <c r="C10" s="16" t="s">
+      <c r="C10" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D10" s="16" t="s">
+      <c r="D10" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E10" s="16" t="s">
+      <c r="E10" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="11" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
+      <c r="B11" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="C11" s="16" t="s">
+      <c r="C11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="D11" s="16" t="s">
+      <c r="D11" s="15" t="s">
         <v>43</v>
       </c>
-      <c r="E11" s="16" t="s">
+      <c r="E11" s="15" t="s">
         <v>43</v>
       </c>
     </row>
     <row r="13" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B13" s="16"/>
-      <c r="C13" s="16"/>
-      <c r="D13" s="16" t="s">
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15" t="s">
         <v>40</v>
       </c>
-      <c r="E13" s="16" t="s">
+      <c r="E13" s="15" t="s">
         <v>41</v>
       </c>
-      <c r="F13" s="16" t="s">
+      <c r="F13" s="15" t="s">
         <v>42</v>
       </c>
-      <c r="G13" s="16" t="s">
+      <c r="G13" s="15" t="s">
         <v>44</v>
       </c>
-      <c r="H13" s="16" t="s">
+      <c r="H13" s="15" t="s">
         <v>45</v>
       </c>
-      <c r="I13" s="16" t="s">
+      <c r="I13" s="15" t="s">
         <v>46</v>
       </c>
-      <c r="J13" s="16" t="s">
+      <c r="J13" s="15" t="s">
         <v>47</v>
       </c>
-      <c r="K13" s="16" t="s">
+      <c r="K13" s="15" t="s">
         <v>48</v>
       </c>
-      <c r="L13" s="16" t="s">
+      <c r="L13" s="15" t="s">
         <v>49</v>
       </c>
-      <c r="M13" s="16" t="s">
+      <c r="M13" s="15" t="s">
         <v>50</v>
       </c>
-      <c r="N13" s="16" t="s">
+      <c r="N13" s="15" t="s">
         <v>51</v>
       </c>
-      <c r="O13" s="16" t="s">
+      <c r="O13" s="15" t="s">
         <v>52</v>
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="25" t="s">
+      <c r="B14" s="21" t="s">
         <v>7</v>
       </c>
-      <c r="C14" s="16" t="s">
+      <c r="C14" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D14" s="16">
+      <c r="D14" s="15">
         <v>82.83</v>
       </c>
-      <c r="E14" s="16">
+      <c r="E14" s="15">
         <v>-14.24</v>
       </c>
-      <c r="F14" s="16">
+      <c r="F14" s="15">
         <v>-3.6</v>
       </c>
-      <c r="G14" s="25">
+      <c r="G14" s="21">
         <f>+D15-D14</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="21">
         <f>+E15-E14</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I14" s="25">
+      <c r="I14" s="21">
         <f>+F15-F14</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J14" s="25">
+      <c r="J14" s="21">
         <f>+ABS(G14)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K14" s="25">
+      <c r="K14" s="21">
         <f>+ABS(H14)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L14" s="25">
+      <c r="L14" s="21">
         <f>+ABS(I14)</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="M14" s="26">
+      <c r="M14" s="22">
         <f>+K14/F14</f>
         <v>-0.34166666666666679</v>
       </c>
-      <c r="N14" s="26">
+      <c r="N14" s="22">
         <f>+K14/E14</f>
         <v>-8.6376404494382053E-2</v>
       </c>
-      <c r="O14" s="26">
+      <c r="O14" s="22">
         <f>+L14/F14</f>
         <v>-3.611111111111108E-2</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="25"/>
-      <c r="C15" s="16" t="s">
+      <c r="B15" s="21"/>
+      <c r="C15" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D15" s="16">
+      <c r="D15" s="15">
         <v>80.680000000000007</v>
       </c>
-      <c r="E15" s="16">
+      <c r="E15" s="15">
         <v>-13.01</v>
       </c>
-      <c r="F15" s="16">
+      <c r="F15" s="15">
         <v>-3.47</v>
       </c>
-      <c r="G15" s="25"/>
-      <c r="H15" s="25"/>
-      <c r="I15" s="25"/>
-      <c r="J15" s="25"/>
-      <c r="K15" s="25"/>
-      <c r="L15" s="25"/>
-      <c r="M15" s="26"/>
-      <c r="N15" s="26"/>
-      <c r="O15" s="26"/>
+      <c r="G15" s="21"/>
+      <c r="H15" s="21"/>
+      <c r="I15" s="21"/>
+      <c r="J15" s="21"/>
+      <c r="K15" s="21"/>
+      <c r="L15" s="21"/>
+      <c r="M15" s="22"/>
+      <c r="N15" s="22"/>
+      <c r="O15" s="22"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="25" t="s">
+      <c r="B16" s="21" t="s">
         <v>8</v>
       </c>
-      <c r="C16" s="16" t="s">
+      <c r="C16" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="16">
+      <c r="D16" s="15">
         <v>81.81</v>
       </c>
-      <c r="E16" s="16">
+      <c r="E16" s="15">
         <v>-12.77</v>
       </c>
-      <c r="F16" s="16">
+      <c r="F16" s="15">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G16" s="25">
+      <c r="G16" s="21">
         <f>+D17-D16</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H16" s="25">
+      <c r="H16" s="21">
         <f t="shared" ref="H16:I16" si="2">+E17-E16</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I16" s="25">
+      <c r="I16" s="21">
         <f t="shared" si="2"/>
         <v>-9.39</v>
       </c>
-      <c r="J16" s="25">
+      <c r="J16" s="21">
         <f t="shared" ref="J16:L16" si="3">+ABS(G16)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K16" s="25">
+      <c r="K16" s="21">
         <f t="shared" si="3"/>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L16" s="25">
+      <c r="L16" s="21">
         <f t="shared" si="3"/>
         <v>9.39</v>
       </c>
-      <c r="M16" s="26">
+      <c r="M16" s="22">
         <f>+J16/D16</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="N16" s="26">
+      <c r="N16" s="22">
         <f>+K16/E16</f>
         <v>-5.7165231010180145E-2</v>
       </c>
-      <c r="O16" s="26">
+      <c r="O16" s="22">
         <f t="shared" ref="O16" si="4">+L16/F16</f>
         <v>1.8557312252964429</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="25"/>
-      <c r="C17" s="16" t="s">
+      <c r="B17" s="21"/>
+      <c r="C17" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="16">
+      <c r="D17" s="15">
         <v>79.78</v>
       </c>
-      <c r="E17" s="16">
+      <c r="E17" s="15">
         <v>-12.04</v>
       </c>
-      <c r="F17" s="16">
+      <c r="F17" s="15">
         <v>-4.33</v>
       </c>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="26"/>
-      <c r="N17" s="26"/>
-      <c r="O17" s="26"/>
+      <c r="G17" s="21"/>
+      <c r="H17" s="21"/>
+      <c r="I17" s="21"/>
+      <c r="J17" s="21"/>
+      <c r="K17" s="21"/>
+      <c r="L17" s="21"/>
+      <c r="M17" s="22"/>
+      <c r="N17" s="22"/>
+      <c r="O17" s="22"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="25" t="s">
+      <c r="B18" s="21" t="s">
         <v>41</v>
       </c>
-      <c r="C18" s="16" t="s">
+      <c r="C18" s="15" t="s">
         <v>30</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="15">
         <v>80.94</v>
       </c>
-      <c r="E18" s="16">
+      <c r="E18" s="15">
         <v>-15.03</v>
       </c>
-      <c r="F18" s="16">
+      <c r="F18" s="15">
         <v>7.39</v>
       </c>
-      <c r="G18" s="25">
+      <c r="G18" s="21">
         <f>+D19-D18</f>
         <v>-4</v>
       </c>
-      <c r="H18" s="25">
+      <c r="H18" s="21">
         <f t="shared" ref="H18:I18" si="5">+E19-E18</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I18" s="25">
+      <c r="I18" s="21">
         <f t="shared" si="5"/>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J18" s="25">
+      <c r="J18" s="21">
         <f t="shared" ref="J18:L18" si="6">+ABS(G18)</f>
         <v>4</v>
       </c>
-      <c r="K18" s="25">
+      <c r="K18" s="21">
         <f t="shared" si="6"/>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L18" s="25">
+      <c r="L18" s="21">
         <f t="shared" si="6"/>
         <v>0.58999999999999986</v>
       </c>
-      <c r="M18" s="26">
+      <c r="M18" s="22">
         <f>+J18/D18</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="N18" s="26">
+      <c r="N18" s="22">
         <f>+K18/E18</f>
         <v>-5.7884231536926095E-2</v>
       </c>
-      <c r="O18" s="26">
+      <c r="O18" s="22">
         <f t="shared" ref="O18" si="7">+L18/F18</f>
         <v>7.9837618403247615E-2</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="25"/>
-      <c r="C19" s="16" t="s">
+      <c r="B19" s="21"/>
+      <c r="C19" s="15" t="s">
         <v>31</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="15">
         <v>76.94</v>
       </c>
-      <c r="E19" s="16">
+      <c r="E19" s="15">
         <v>-14.16</v>
       </c>
-      <c r="F19" s="16">
+      <c r="F19" s="15">
         <v>6.8</v>
       </c>
-      <c r="G19" s="25"/>
-      <c r="H19" s="25"/>
-      <c r="I19" s="25"/>
-      <c r="J19" s="25"/>
-      <c r="K19" s="25"/>
-      <c r="L19" s="25"/>
-      <c r="M19" s="26"/>
-      <c r="N19" s="26"/>
-      <c r="O19" s="26"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="22"/>
+      <c r="N19" s="22"/>
+      <c r="O19" s="22"/>
     </row>
   </sheetData>
   <mergeCells count="31">
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="J18:J19"/>
     <mergeCell ref="L18:L19"/>
     <mergeCell ref="M18:M19"/>
     <mergeCell ref="N18:N19"/>
@@ -1369,6 +1384,21 @@
     <mergeCell ref="O14:O15"/>
     <mergeCell ref="K16:K17"/>
     <mergeCell ref="K14:K15"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="J18:J19"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1396,16 +1426,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E2" s="35" t="s">
+      <c r="E2" s="30" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="35"/>
-      <c r="G2" s="35"/>
-      <c r="H2" s="35"/>
-      <c r="I2" s="35"/>
-      <c r="N2" s="41"/>
-      <c r="O2" s="41"/>
-      <c r="P2" s="41"/>
+      <c r="F2" s="30"/>
+      <c r="G2" s="30"/>
+      <c r="H2" s="30"/>
+      <c r="I2" s="30"/>
+      <c r="N2" s="28"/>
+      <c r="O2" s="28"/>
+      <c r="P2" s="28"/>
     </row>
     <row r="3" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E3" s="2"/>
@@ -1438,158 +1468,158 @@
       </c>
     </row>
     <row r="5" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="34" t="s">
+      <c r="E5" s="29" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="39">
+      <c r="F5" s="34">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="39">
+      <c r="G5" s="34">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="40">
+      <c r="H5" s="35">
         <v>0.17</v>
       </c>
-      <c r="I5" s="38">
+      <c r="I5" s="33">
         <v>1.17</v>
       </c>
-      <c r="J5" s="34">
+      <c r="J5" s="29">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="34">
+      <c r="K5" s="29">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="34"/>
-      <c r="F6" s="39"/>
-      <c r="G6" s="39"/>
-      <c r="H6" s="40"/>
-      <c r="I6" s="38"/>
-      <c r="J6" s="34"/>
-      <c r="K6" s="34"/>
+      <c r="E6" s="29"/>
+      <c r="F6" s="34"/>
+      <c r="G6" s="34"/>
+      <c r="H6" s="35"/>
+      <c r="I6" s="33"/>
+      <c r="J6" s="29"/>
+      <c r="K6" s="29"/>
       <c r="O6" s="3"/>
     </row>
     <row r="7" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E7" s="27" t="s">
+      <c r="E7" s="23" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="36">
+      <c r="F7" s="31">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="37">
+      <c r="G7" s="32">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="37">
+      <c r="H7" s="32">
         <v>0.1</v>
       </c>
-      <c r="I7" s="27">
+      <c r="I7" s="23">
         <v>0.92</v>
       </c>
-      <c r="J7" s="27">
+      <c r="J7" s="23">
         <f t="shared" ref="J7" si="0">+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="27">
+      <c r="K7" s="23">
         <f t="shared" ref="K7" si="1">+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E8" s="27"/>
-      <c r="F8" s="36"/>
-      <c r="G8" s="37"/>
-      <c r="H8" s="37"/>
-      <c r="I8" s="27"/>
-      <c r="J8" s="27"/>
-      <c r="K8" s="27"/>
+      <c r="E8" s="23"/>
+      <c r="F8" s="31"/>
+      <c r="G8" s="32"/>
+      <c r="H8" s="32"/>
+      <c r="I8" s="23"/>
+      <c r="J8" s="23"/>
+      <c r="K8" s="23"/>
     </row>
     <row r="9" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E9" s="27" t="s">
+      <c r="E9" s="23" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="36">
+      <c r="F9" s="31">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="37">
+      <c r="G9" s="32">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="37">
+      <c r="H9" s="32">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="27">
+      <c r="I9" s="23">
         <v>1.01</v>
       </c>
-      <c r="J9" s="27">
+      <c r="J9" s="23">
         <f t="shared" ref="J9" si="2">+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="27">
+      <c r="K9" s="23">
         <f t="shared" ref="K9" si="3">+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="10" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E10" s="27"/>
-      <c r="F10" s="36"/>
-      <c r="G10" s="37"/>
-      <c r="H10" s="37"/>
-      <c r="I10" s="27"/>
-      <c r="J10" s="27"/>
-      <c r="K10" s="27"/>
+      <c r="E10" s="23"/>
+      <c r="F10" s="31"/>
+      <c r="G10" s="32"/>
+      <c r="H10" s="32"/>
+      <c r="I10" s="23"/>
+      <c r="J10" s="23"/>
+      <c r="K10" s="23"/>
     </row>
     <row r="12" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E12" s="28" t="s">
+      <c r="E12" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="33"/>
-      <c r="G12" s="33"/>
-      <c r="H12" s="33"/>
-      <c r="I12" s="29"/>
-      <c r="J12" s="28" t="s">
+      <c r="F12" s="27"/>
+      <c r="G12" s="27"/>
+      <c r="H12" s="27"/>
+      <c r="I12" s="26"/>
+      <c r="J12" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="33"/>
-      <c r="L12" s="33"/>
-      <c r="M12" s="33"/>
-      <c r="N12" s="33"/>
-      <c r="O12" s="33"/>
-      <c r="P12" s="29"/>
+      <c r="K12" s="27"/>
+      <c r="L12" s="27"/>
+      <c r="M12" s="27"/>
+      <c r="N12" s="27"/>
+      <c r="O12" s="27"/>
+      <c r="P12" s="26"/>
     </row>
     <row r="13" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E13" s="2"/>
-      <c r="F13" s="28" t="s">
+      <c r="F13" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="29"/>
-      <c r="H13" s="27" t="s">
+      <c r="G13" s="26"/>
+      <c r="H13" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="27"/>
-      <c r="J13" s="27" t="s">
+      <c r="I13" s="23"/>
+      <c r="J13" s="23" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="27"/>
-      <c r="L13" s="27" t="s">
+      <c r="K13" s="23"/>
+      <c r="L13" s="23" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="27"/>
-      <c r="N13" s="27" t="s">
+      <c r="M13" s="23"/>
+      <c r="N13" s="23" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="27"/>
+      <c r="O13" s="23"/>
       <c r="P13" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D14" s="42"/>
+      <c r="D14" s="24"/>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="F14" s="20">
+      <c r="F14" s="19">
         <v>1.1782600000000001</v>
       </c>
       <c r="G14" s="5">
@@ -1600,45 +1630,45 @@
         <f>+F14*(1-$J$5/100)</f>
         <v>1.08635572</v>
       </c>
-      <c r="I14" s="5">
+      <c r="I14" s="39">
         <f>H14/$H$17</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J14" s="22">
+      <c r="J14" s="40">
         <f>+H14*(1-$K$5/100)</f>
         <v>0.99292912808000011</v>
       </c>
-      <c r="K14" s="5">
+      <c r="K14" s="39">
         <f>+J14/$J$17</f>
         <v>0.60805259681281487</v>
       </c>
-      <c r="L14" s="22">
+      <c r="L14" s="40">
         <f>+$H$14*(1-$K$7/100)</f>
         <v>1.0276925111199999</v>
       </c>
-      <c r="M14" s="5">
+      <c r="M14" s="39">
         <f>+L14/$J$25</f>
         <v>0.60542601972075083</v>
       </c>
-      <c r="N14" s="22">
+      <c r="N14" s="40">
         <f>+$H$14*(1-$K$9/100)</f>
         <v>1.01248353104</v>
       </c>
-      <c r="O14" s="5">
+      <c r="O14" s="39">
         <f>+N14/$J$33</f>
         <v>0.60477291721835513</v>
       </c>
-      <c r="P14" s="4">
+      <c r="P14" s="41">
         <f>AVERAGE(J14,L14,N14)</f>
         <v>1.0110350567466666</v>
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D15" s="42"/>
+      <c r="D15" s="24"/>
       <c r="E15" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="F15" s="20">
+      <c r="F15" s="19">
         <v>0.38450000000000001</v>
       </c>
       <c r="G15" s="5">
@@ -1649,45 +1679,45 @@
         <f>+F15*(1-$J$5/100)</f>
         <v>0.35450899999999996</v>
       </c>
-      <c r="I15" s="5">
+      <c r="I15" s="39">
         <f t="shared" ref="I15:I16" si="4">H15/$H$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J15" s="22">
+      <c r="J15" s="40">
         <f>+H15*(1-$K$5/100)</f>
         <v>0.324021226</v>
       </c>
-      <c r="K15" s="5">
+      <c r="K15" s="39">
         <f t="shared" ref="K15:K16" si="5">+J15/$J$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L15" s="22">
+      <c r="L15" s="40">
         <f>$H$15*(1-$K$7/100)</f>
         <v>0.33536551399999998</v>
       </c>
-      <c r="M15" s="5">
+      <c r="M15" s="39">
         <f t="shared" ref="M15:M16" si="6">+L15/$J$25</f>
         <v>0.19756785818293812</v>
       </c>
-      <c r="N15" s="22">
+      <c r="N15" s="40">
         <f>+$H$15*(1-$K$9/100)</f>
         <v>0.33040238799999994</v>
       </c>
-      <c r="O15" s="5">
+      <c r="O15" s="39">
         <f t="shared" ref="O15:O17" si="7">+N15/$J$33</f>
         <v>0.19735473212233082</v>
       </c>
-      <c r="P15" s="4">
+      <c r="P15" s="41">
         <f>AVERAGE(J15,L15,N15)</f>
         <v>0.32992970933333332</v>
       </c>
     </row>
     <row r="16" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D16" s="42"/>
+      <c r="D16" s="24"/>
       <c r="E16" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="F16" s="20">
+      <c r="F16" s="19">
         <v>0.375</v>
       </c>
       <c r="G16" s="5">
@@ -1698,45 +1728,45 @@
         <f>+F16*(1-$J$5/100)</f>
         <v>0.34575</v>
       </c>
-      <c r="I16" s="5">
+      <c r="I16" s="39">
         <f t="shared" si="4"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="J16" s="22">
+      <c r="J16" s="40">
         <f>+H16*(1-$K$5/100)</f>
         <v>0.3160155</v>
       </c>
-      <c r="K16" s="5">
+      <c r="K16" s="39">
         <f t="shared" si="5"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="L16" s="22">
+      <c r="L16" s="40">
         <f>+$H$16*(1-$K$7/100)</f>
         <v>0.32707949999999997</v>
       </c>
-      <c r="M16" s="5">
+      <c r="M16" s="39">
         <f t="shared" si="6"/>
         <v>0.19268646766866526</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="40">
         <f>+$H$16*(1-$K$9/100)</f>
         <v>0.322239</v>
       </c>
-      <c r="O16" s="5">
+      <c r="O16" s="39">
         <f t="shared" si="7"/>
         <v>0.19247860740149306</v>
       </c>
-      <c r="P16" s="4">
+      <c r="P16" s="41">
         <f>AVERAGE(J16,L16,N16)</f>
         <v>0.32177799999999995</v>
       </c>
     </row>
     <row r="17" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D17" s="42"/>
+      <c r="D17" s="24"/>
       <c r="E17" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="21">
+      <c r="F17" s="20">
         <f t="shared" ref="F17:M17" si="9">SUM(F14:F16)</f>
         <v>1.9377600000000001</v>
       </c>
@@ -1748,41 +1778,41 @@
         <f t="shared" si="9"/>
         <v>1.78661472</v>
       </c>
-      <c r="I17" s="6">
+      <c r="I17" s="42">
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="J17" s="23">
+      <c r="J17" s="43">
         <f>SUM(J14:J16)</f>
         <v>1.6329658540800001</v>
       </c>
-      <c r="K17" s="4">
+      <c r="K17" s="41">
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="L17" s="23">
+      <c r="L17" s="43">
         <f t="shared" si="9"/>
         <v>1.6901375251199999</v>
       </c>
-      <c r="M17" s="4">
+      <c r="M17" s="41">
         <f t="shared" si="9"/>
         <v>0.99568034557235419</v>
       </c>
-      <c r="N17" s="23">
+      <c r="N17" s="43">
         <f>SUM(N14:N16)</f>
         <v>1.6651249190399999</v>
       </c>
-      <c r="O17" s="4">
+      <c r="O17" s="41">
         <f t="shared" si="7"/>
         <v>0.99460625674217906</v>
       </c>
-      <c r="P17" s="4">
+      <c r="P17" s="41">
         <f>AVERAGE(J17,L17,N17)</f>
         <v>1.66274276608</v>
       </c>
     </row>
     <row r="18" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D18" s="42"/>
+      <c r="D18" s="24"/>
       <c r="E18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1794,404 +1824,430 @@
         <f>+H17/F17-1</f>
         <v>-7.8000000000000069E-2</v>
       </c>
-      <c r="I18" s="2" t="s">
+      <c r="I18" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="J18" s="24">
+      <c r="J18" s="39">
         <f>+J17/I17-1</f>
         <v>0.63296585408000006</v>
       </c>
-      <c r="K18" s="2"/>
-      <c r="L18" s="24">
+      <c r="K18" s="44"/>
+      <c r="L18" s="39">
         <f>+L17/K17-1</f>
         <v>0.69013752511999993</v>
       </c>
-      <c r="M18" s="2"/>
-      <c r="N18" s="24">
+      <c r="M18" s="44"/>
+      <c r="N18" s="39">
         <f>+N17/M17-1</f>
         <v>0.67234888831999995</v>
       </c>
-      <c r="O18" s="2"/>
-      <c r="P18" s="2"/>
+      <c r="O18" s="44"/>
+      <c r="P18" s="44"/>
     </row>
     <row r="20" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E20" s="27" t="s">
+      <c r="E20" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="27"/>
-      <c r="G20" s="27"/>
-      <c r="H20" s="27"/>
-      <c r="I20" s="27"/>
-      <c r="J20" s="27"/>
-      <c r="K20" s="27"/>
-      <c r="L20" s="27"/>
+      <c r="F20" s="23"/>
+      <c r="G20" s="23"/>
+      <c r="H20" s="23"/>
+      <c r="I20" s="23"/>
+      <c r="J20" s="23"/>
+      <c r="K20" s="23"/>
+      <c r="L20" s="23"/>
     </row>
     <row r="21" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E21" s="2"/>
-      <c r="F21" s="28" t="s">
+      <c r="E21" s="44"/>
+      <c r="F21" s="45" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="29"/>
-      <c r="H21" s="27" t="s">
+      <c r="G21" s="46"/>
+      <c r="H21" s="47" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="27"/>
-      <c r="J21" s="27" t="s">
+      <c r="I21" s="47"/>
+      <c r="J21" s="47" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="27"/>
-      <c r="L21" s="10"/>
+      <c r="K21" s="47"/>
+      <c r="L21" s="48"/>
+      <c r="M21" s="49"/>
+      <c r="N21" s="49"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D22" s="42"/>
-      <c r="E22" s="2" t="s">
+      <c r="D22" s="24"/>
+      <c r="E22" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="7">
+      <c r="F22" s="40">
         <v>1.1782600000000001</v>
       </c>
-      <c r="G22" s="5">
+      <c r="G22" s="39">
         <f>+F22/$F$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="H22" s="7">
+      <c r="H22" s="40">
         <f>+F22*(1-$J$7/100)</f>
         <v>1.09106876</v>
       </c>
-      <c r="I22" s="5">
+      <c r="I22" s="39">
         <f>H22/$H$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J22" s="22">
+      <c r="J22" s="40">
         <f>+$H$22*(1-$K$7/100)</f>
         <v>1.0321510469599999</v>
       </c>
-      <c r="K22" s="5">
+      <c r="K22" s="39">
         <f>+J22/$J$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L22" s="7"/>
+      <c r="L22" s="40"/>
+      <c r="M22" s="49"/>
+      <c r="N22" s="49"/>
     </row>
     <row r="23" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D23" s="42"/>
-      <c r="E23" s="2" t="s">
+      <c r="D23" s="24"/>
+      <c r="E23" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="F23" s="7">
+      <c r="F23" s="40">
         <v>0.38450000000000001</v>
       </c>
-      <c r="G23" s="5">
+      <c r="G23" s="39">
         <f t="shared" ref="G23:G24" si="10">+F23/$F$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="H23" s="7">
+      <c r="H23" s="40">
         <f t="shared" ref="H23:H25" si="11">+F23*(1-$J$7/100)</f>
         <v>0.356047</v>
       </c>
-      <c r="I23" s="5">
+      <c r="I23" s="39">
         <f>H23/$H$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J23" s="22">
+      <c r="J23" s="40">
         <f>+$H$23*(1-$K$7/100)</f>
         <v>0.33682046199999999</v>
       </c>
-      <c r="K23" s="5">
+      <c r="K23" s="39">
         <f t="shared" ref="K23:K24" si="12">+J23/$J$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L23" s="7"/>
+      <c r="L23" s="40"/>
+      <c r="M23" s="49"/>
+      <c r="N23" s="49"/>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D24" s="42"/>
-      <c r="E24" s="2" t="s">
+      <c r="D24" s="24"/>
+      <c r="E24" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="7">
+      <c r="F24" s="40">
         <v>0.375</v>
       </c>
-      <c r="G24" s="5">
+      <c r="G24" s="39">
         <f t="shared" si="10"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="H24" s="7">
+      <c r="H24" s="40">
         <f t="shared" si="11"/>
         <v>0.34724999999999995</v>
       </c>
-      <c r="I24" s="5">
+      <c r="I24" s="39">
         <f>H24/$H$25</f>
         <v>0.19352241763685901</v>
       </c>
-      <c r="J24" s="22">
+      <c r="J24" s="40">
         <f>+$H$24*(1-$K$7/100)</f>
         <v>0.32849849999999992</v>
       </c>
-      <c r="K24" s="5">
+      <c r="K24" s="39">
         <f t="shared" si="12"/>
         <v>0.19352241763685901</v>
       </c>
-      <c r="L24" s="7"/>
+      <c r="L24" s="40"/>
+      <c r="M24" s="49"/>
+      <c r="N24" s="49"/>
     </row>
     <row r="25" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D25" s="42"/>
-      <c r="E25" s="2" t="s">
+      <c r="D25" s="24"/>
+      <c r="E25" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="8">
+      <c r="F25" s="43">
         <f t="shared" ref="F25:K25" si="13">SUM(F22:F24)</f>
         <v>1.9377600000000001</v>
       </c>
-      <c r="G25" s="6">
+      <c r="G25" s="42">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="H25" s="7">
+      <c r="H25" s="40">
         <f t="shared" si="11"/>
         <v>1.79436576</v>
       </c>
-      <c r="I25" s="6">
+      <c r="I25" s="42">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="J25" s="23">
+      <c r="J25" s="43">
         <f t="shared" si="13"/>
         <v>1.6974700089599999</v>
       </c>
-      <c r="K25" s="4">
+      <c r="K25" s="41">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="L25" s="7"/>
+      <c r="L25" s="40"/>
+      <c r="M25" s="49"/>
+      <c r="N25" s="49"/>
     </row>
     <row r="26" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D26" s="42"/>
-      <c r="E26" s="2" t="s">
+      <c r="D26" s="24"/>
+      <c r="E26" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="2"/>
-      <c r="G26" s="2" t="s">
+      <c r="F26" s="44"/>
+      <c r="G26" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="5">
+      <c r="H26" s="39">
         <f>+H25/F25-1</f>
         <v>-7.4000000000000066E-2</v>
       </c>
-      <c r="I26" s="2" t="s">
+      <c r="I26" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="J26" s="24">
+      <c r="J26" s="39">
         <f>+J25/I25-1</f>
         <v>0.69747000895999989</v>
       </c>
-      <c r="K26" s="2"/>
-      <c r="L26" s="2"/>
+      <c r="K26" s="44"/>
+      <c r="L26" s="44"/>
+      <c r="M26" s="49"/>
+      <c r="N26" s="49"/>
+    </row>
+    <row r="27" spans="4:16" x14ac:dyDescent="0.25">
+      <c r="E27" s="49"/>
+      <c r="F27" s="49"/>
+      <c r="G27" s="49"/>
+      <c r="H27" s="49"/>
+      <c r="I27" s="49"/>
+      <c r="J27" s="49"/>
+      <c r="K27" s="49"/>
+      <c r="L27" s="49"/>
+      <c r="M27" s="49"/>
+      <c r="N27" s="49"/>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E28" s="28" t="s">
+      <c r="E28" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="33"/>
-      <c r="G28" s="33"/>
-      <c r="H28" s="33"/>
-      <c r="I28" s="33"/>
-      <c r="J28" s="33"/>
-      <c r="K28" s="33"/>
-      <c r="L28" s="29"/>
+      <c r="F28" s="50"/>
+      <c r="G28" s="50"/>
+      <c r="H28" s="50"/>
+      <c r="I28" s="50"/>
+      <c r="J28" s="50"/>
+      <c r="K28" s="50"/>
+      <c r="L28" s="46"/>
+      <c r="M28" s="49"/>
+      <c r="N28" s="49"/>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E29" s="2"/>
-      <c r="F29" s="28" t="s">
+      <c r="F29" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="29"/>
-      <c r="H29" s="27" t="s">
+      <c r="G29" s="26"/>
+      <c r="H29" s="23" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="27"/>
-      <c r="J29" s="27" t="s">
+      <c r="I29" s="23"/>
+      <c r="J29" s="23" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="27"/>
+      <c r="K29" s="23"/>
       <c r="L29" s="10"/>
     </row>
-    <row r="30" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D30" s="42"/>
-      <c r="E30" s="2" t="s">
+    <row r="30" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D30" s="51"/>
+      <c r="E30" s="44" t="s">
         <v>13</v>
       </c>
-      <c r="F30" s="7">
+      <c r="F30" s="40">
         <v>1.1782600000000001</v>
       </c>
-      <c r="G30" s="5">
+      <c r="G30" s="39">
         <f>+F30/$F$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="H30" s="7">
+      <c r="H30" s="40">
         <f>+F30*(1-$J$9/100)</f>
         <v>1.0922470200000001</v>
       </c>
-      <c r="I30" s="5">
+      <c r="I30" s="39">
         <f>H30/$H$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J30" s="22">
+      <c r="J30" s="40">
         <f>+$H$30*(1-$K$9/100)</f>
         <v>1.0179742226399999</v>
       </c>
-      <c r="K30" s="5">
+      <c r="K30" s="39">
         <f>+J30/$J$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L30" s="7"/>
-    </row>
-    <row r="31" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D31" s="42"/>
-      <c r="E31" s="2" t="s">
+      <c r="L30" s="40"/>
+    </row>
+    <row r="31" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D31" s="51"/>
+      <c r="E31" s="44" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="7">
+      <c r="F31" s="40">
         <v>0.38450000000000001</v>
       </c>
-      <c r="G31" s="5">
+      <c r="G31" s="39">
         <f t="shared" ref="G31:G32" si="14">+F31/$F$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="H31" s="7">
+      <c r="H31" s="40">
         <f t="shared" ref="H31:H32" si="15">+F31*(1-$J$9/100)</f>
         <v>0.35643150000000001</v>
       </c>
-      <c r="I31" s="5">
+      <c r="I31" s="39">
         <f>H31/$H$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J31" s="22">
+      <c r="J31" s="40">
         <f>+$H$31*(1-$K$9/100)</f>
         <v>0.33219415800000002</v>
       </c>
-      <c r="K31" s="5">
+      <c r="K31" s="39">
         <f t="shared" ref="K31:K33" si="16">+J31/$J$33</f>
         <v>0.19842498555032617</v>
       </c>
-      <c r="L31" s="7"/>
-    </row>
-    <row r="32" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D32" s="42"/>
-      <c r="E32" s="2" t="s">
+      <c r="L31" s="40"/>
+    </row>
+    <row r="32" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D32" s="51"/>
+      <c r="E32" s="44" t="s">
         <v>15</v>
       </c>
-      <c r="F32" s="7">
+      <c r="F32" s="40">
         <v>0.375</v>
       </c>
-      <c r="G32" s="5">
+      <c r="G32" s="39">
         <f t="shared" si="14"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="H32" s="7">
+      <c r="H32" s="40">
         <f t="shared" si="15"/>
         <v>0.34762500000000002</v>
       </c>
-      <c r="I32" s="5">
+      <c r="I32" s="39">
         <f>H32/$H$33</f>
         <v>0.19352241763685904</v>
       </c>
-      <c r="J32" s="22">
+      <c r="J32" s="40">
         <f>+$H$32*(1-$K$9/100)</f>
         <v>0.32398650000000001</v>
       </c>
-      <c r="K32" s="5">
+      <c r="K32" s="39">
         <f t="shared" si="16"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="L32" s="7"/>
-    </row>
-    <row r="33" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D33" s="42"/>
-      <c r="E33" s="2" t="s">
+      <c r="L32" s="40"/>
+    </row>
+    <row r="33" spans="4:14" s="49" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D33" s="51"/>
+      <c r="E33" s="44" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="8">
+      <c r="F33" s="43">
         <f>SUM(F30:F32)</f>
         <v>1.9377600000000001</v>
       </c>
-      <c r="G33" s="6">
+      <c r="G33" s="42">
         <f>SUM(G30:G32)</f>
         <v>1</v>
       </c>
-      <c r="H33" s="8">
+      <c r="H33" s="43">
         <f>SUM(H30:H32)</f>
         <v>1.7963035200000002</v>
       </c>
-      <c r="I33" s="6">
+      <c r="I33" s="42">
         <f>SUM(I30:I32)</f>
         <v>1</v>
       </c>
-      <c r="J33" s="23">
+      <c r="J33" s="43">
         <f>SUM(J30:J32)</f>
         <v>1.67415488064</v>
       </c>
-      <c r="K33" s="4">
+      <c r="K33" s="41">
         <f t="shared" si="16"/>
         <v>1</v>
       </c>
-      <c r="L33" s="7"/>
-    </row>
-    <row r="34" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="D34" s="42"/>
-      <c r="E34" s="2" t="s">
+      <c r="L33" s="40"/>
+    </row>
+    <row r="34" spans="4:14" s="49" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D34" s="51"/>
+      <c r="E34" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="F34" s="2"/>
-      <c r="G34" s="2" t="s">
+      <c r="F34" s="44"/>
+      <c r="G34" s="44" t="s">
         <v>2</v>
       </c>
-      <c r="H34" s="5">
+      <c r="H34" s="39">
         <f>+H33/F33-1</f>
         <v>-7.2999999999999954E-2</v>
       </c>
-      <c r="I34" s="2" t="s">
+      <c r="I34" s="44" t="s">
         <v>3</v>
       </c>
-      <c r="J34" s="24">
+      <c r="J34" s="39">
         <f>+J33/I33-1</f>
         <v>0.67415488063999995</v>
       </c>
-      <c r="K34" s="2"/>
-      <c r="L34" s="11"/>
+      <c r="K34" s="44"/>
+      <c r="L34" s="52"/>
     </row>
     <row r="36" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="E36" s="27" t="s">
+      <c r="E36" s="23" t="s">
         <v>24</v>
       </c>
-      <c r="F36" s="27"/>
-      <c r="G36" s="27"/>
-      <c r="H36" s="27" t="s">
+      <c r="F36" s="23"/>
+      <c r="G36" s="23"/>
+      <c r="H36" s="23" t="s">
         <v>21</v>
       </c>
-      <c r="I36" s="27"/>
-      <c r="J36" s="27"/>
-      <c r="K36" s="27"/>
-      <c r="L36" s="27"/>
-      <c r="M36" s="27"/>
-      <c r="N36" s="27"/>
+      <c r="I36" s="23"/>
+      <c r="J36" s="23"/>
+      <c r="K36" s="23"/>
+      <c r="L36" s="23"/>
+      <c r="M36" s="23"/>
+      <c r="N36" s="23"/>
     </row>
     <row r="37" spans="4:14" x14ac:dyDescent="0.25">
       <c r="E37" s="2"/>
-      <c r="F37" s="28" t="s">
+      <c r="F37" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="G37" s="29"/>
-      <c r="H37" s="30" t="s">
+      <c r="G37" s="26"/>
+      <c r="H37" s="36" t="s">
         <v>54</v>
       </c>
-      <c r="I37" s="30"/>
-      <c r="J37" s="30" t="s">
+      <c r="I37" s="36"/>
+      <c r="J37" s="36" t="s">
         <v>55</v>
       </c>
-      <c r="K37" s="30"/>
-      <c r="L37" s="31" t="s">
+      <c r="K37" s="36"/>
+      <c r="L37" s="37" t="s">
         <v>56</v>
       </c>
-      <c r="M37" s="32"/>
+      <c r="M37" s="38"/>
       <c r="N37" s="2" t="s">
         <v>57</v>
       </c>
@@ -2382,24 +2438,19 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="D14:D18"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="E20:L20"/>
-    <mergeCell ref="D30:D34"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D22:D26"/>
-    <mergeCell ref="E28:L28"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="H36:N36"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J12:P12"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="E9:E10"/>
@@ -2416,19 +2467,24 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J12:P12"/>
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="H36:N36"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D22:D26"/>
+    <mergeCell ref="E28:L28"/>
+    <mergeCell ref="D14:D18"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="E20:L20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -2444,98 +2500,98 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="C2" s="18">
+      <c r="C2" s="17">
         <v>1.2</v>
       </c>
-      <c r="D2" s="13"/>
-      <c r="E2" s="17" t="s">
+      <c r="D2" s="12"/>
+      <c r="E2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="F2" s="18">
+      <c r="F2" s="17">
         <v>0.6</v>
       </c>
-      <c r="G2" s="13"/>
-      <c r="H2" s="17" t="s">
+      <c r="G2" s="12"/>
+      <c r="H2" s="16" t="s">
         <v>26</v>
       </c>
-      <c r="I2" s="18">
+      <c r="I2" s="17">
         <v>1.8</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B3" s="16" t="s">
+      <c r="B3" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="C3" s="19">
+      <c r="C3" s="18">
         <f>SQRT(($C$2^2)/3)</f>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="F3" s="19">
+      <c r="F3" s="18">
         <f>SQRT(($F$2^2)/3)</f>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H3" s="16" t="s">
+      <c r="H3" s="15" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="19">
+      <c r="I3" s="18">
         <f>SQRT(($I$2^2)/3)</f>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B4" s="16" t="s">
+      <c r="B4" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="19">
+      <c r="C4" s="18">
         <f t="shared" ref="C4:C5" si="0">SQRT(($C$2^2)/3)</f>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E4" s="16" t="s">
+      <c r="E4" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="19">
+      <c r="F4" s="18">
         <f t="shared" ref="F4:F5" si="1">SQRT(($F$2^2)/3)</f>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H4" s="16" t="s">
+      <c r="H4" s="15" t="s">
         <v>28</v>
       </c>
-      <c r="I4" s="19">
+      <c r="I4" s="18">
         <f t="shared" ref="I4:I5" si="2">SQRT(($I$2^2)/3)</f>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B5" s="16" t="s">
+      <c r="B5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="C5" s="19">
+      <c r="C5" s="18">
         <f t="shared" si="0"/>
         <v>0.69282032302755092</v>
       </c>
-      <c r="E5" s="16" t="s">
+      <c r="E5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="F5" s="19">
+      <c r="F5" s="18">
         <f t="shared" si="1"/>
         <v>0.34641016151377546</v>
       </c>
-      <c r="H5" s="16" t="s">
+      <c r="H5" s="15" t="s">
         <v>29</v>
       </c>
-      <c r="I5" s="19">
+      <c r="I5" s="18">
         <f t="shared" si="2"/>
         <v>1.0392304845413265</v>
       </c>
     </row>
     <row r="12" spans="2:9" ht="16.5" x14ac:dyDescent="0.25">
-      <c r="E12" s="12"/>
+      <c r="E12" s="11"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
ajustes de shadereport y extractores
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -480,6 +480,33 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -489,91 +516,64 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="5" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="3" borderId="1" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="9" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="10" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -952,10 +952,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="23" t="s">
+      <c r="H2" s="32" t="s">
         <v>33</v>
       </c>
-      <c r="I2" s="23"/>
+      <c r="I2" s="32"/>
     </row>
     <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" s="2" t="s">
@@ -1136,7 +1136,7 @@
       </c>
     </row>
     <row r="14" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B14" s="21" t="s">
+      <c r="B14" s="30" t="s">
         <v>7</v>
       </c>
       <c r="C14" s="15" t="s">
@@ -1151,45 +1151,45 @@
       <c r="F14" s="15">
         <v>-3.6</v>
       </c>
-      <c r="G14" s="21">
+      <c r="G14" s="30">
         <f>+D15-D14</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H14" s="21">
+      <c r="H14" s="30">
         <f>+E15-E14</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I14" s="21">
+      <c r="I14" s="30">
         <f>+F15-F14</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J14" s="21">
+      <c r="J14" s="30">
         <f>+ABS(G14)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K14" s="21">
+      <c r="K14" s="30">
         <f>+ABS(H14)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L14" s="21">
+      <c r="L14" s="30">
         <f>+ABS(I14)</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="M14" s="22">
+      <c r="M14" s="31">
         <f>+K14/F14</f>
         <v>-0.34166666666666679</v>
       </c>
-      <c r="N14" s="22">
+      <c r="N14" s="31">
         <f>+K14/E14</f>
         <v>-8.6376404494382053E-2</v>
       </c>
-      <c r="O14" s="22">
+      <c r="O14" s="31">
         <f>+L14/F14</f>
         <v>-3.611111111111108E-2</v>
       </c>
     </row>
     <row r="15" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B15" s="21"/>
+      <c r="B15" s="30"/>
       <c r="C15" s="15" t="s">
         <v>31</v>
       </c>
@@ -1202,18 +1202,18 @@
       <c r="F15" s="15">
         <v>-3.47</v>
       </c>
-      <c r="G15" s="21"/>
-      <c r="H15" s="21"/>
-      <c r="I15" s="21"/>
-      <c r="J15" s="21"/>
-      <c r="K15" s="21"/>
-      <c r="L15" s="21"/>
-      <c r="M15" s="22"/>
-      <c r="N15" s="22"/>
-      <c r="O15" s="22"/>
+      <c r="G15" s="30"/>
+      <c r="H15" s="30"/>
+      <c r="I15" s="30"/>
+      <c r="J15" s="30"/>
+      <c r="K15" s="30"/>
+      <c r="L15" s="30"/>
+      <c r="M15" s="31"/>
+      <c r="N15" s="31"/>
+      <c r="O15" s="31"/>
     </row>
     <row r="16" spans="1:15" x14ac:dyDescent="0.25">
-      <c r="B16" s="21" t="s">
+      <c r="B16" s="30" t="s">
         <v>8</v>
       </c>
       <c r="C16" s="15" t="s">
@@ -1228,45 +1228,45 @@
       <c r="F16" s="15">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G16" s="21">
+      <c r="G16" s="30">
         <f>+D17-D16</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H16" s="21">
+      <c r="H16" s="30">
         <f t="shared" ref="H16:I16" si="2">+E17-E16</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I16" s="21">
+      <c r="I16" s="30">
         <f t="shared" si="2"/>
         <v>-9.39</v>
       </c>
-      <c r="J16" s="21">
+      <c r="J16" s="30">
         <f t="shared" ref="J16:L16" si="3">+ABS(G16)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K16" s="21">
+      <c r="K16" s="30">
         <f t="shared" si="3"/>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L16" s="21">
+      <c r="L16" s="30">
         <f t="shared" si="3"/>
         <v>9.39</v>
       </c>
-      <c r="M16" s="22">
+      <c r="M16" s="31">
         <f>+J16/D16</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="N16" s="22">
+      <c r="N16" s="31">
         <f>+K16/E16</f>
         <v>-5.7165231010180145E-2</v>
       </c>
-      <c r="O16" s="22">
+      <c r="O16" s="31">
         <f t="shared" ref="O16" si="4">+L16/F16</f>
         <v>1.8557312252964429</v>
       </c>
     </row>
     <row r="17" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B17" s="21"/>
+      <c r="B17" s="30"/>
       <c r="C17" s="15" t="s">
         <v>31</v>
       </c>
@@ -1279,18 +1279,18 @@
       <c r="F17" s="15">
         <v>-4.33</v>
       </c>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="22"/>
-      <c r="N17" s="22"/>
-      <c r="O17" s="22"/>
+      <c r="G17" s="30"/>
+      <c r="H17" s="30"/>
+      <c r="I17" s="30"/>
+      <c r="J17" s="30"/>
+      <c r="K17" s="30"/>
+      <c r="L17" s="30"/>
+      <c r="M17" s="31"/>
+      <c r="N17" s="31"/>
+      <c r="O17" s="31"/>
     </row>
     <row r="18" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B18" s="21" t="s">
+      <c r="B18" s="30" t="s">
         <v>41</v>
       </c>
       <c r="C18" s="15" t="s">
@@ -1305,45 +1305,45 @@
       <c r="F18" s="15">
         <v>7.39</v>
       </c>
-      <c r="G18" s="21">
+      <c r="G18" s="30">
         <f>+D19-D18</f>
         <v>-4</v>
       </c>
-      <c r="H18" s="21">
+      <c r="H18" s="30">
         <f t="shared" ref="H18:I18" si="5">+E19-E18</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I18" s="21">
+      <c r="I18" s="30">
         <f t="shared" si="5"/>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J18" s="21">
+      <c r="J18" s="30">
         <f t="shared" ref="J18:L18" si="6">+ABS(G18)</f>
         <v>4</v>
       </c>
-      <c r="K18" s="21">
+      <c r="K18" s="30">
         <f t="shared" si="6"/>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L18" s="21">
+      <c r="L18" s="30">
         <f t="shared" si="6"/>
         <v>0.58999999999999986</v>
       </c>
-      <c r="M18" s="22">
+      <c r="M18" s="31">
         <f>+J18/D18</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="N18" s="22">
+      <c r="N18" s="31">
         <f>+K18/E18</f>
         <v>-5.7884231536926095E-2</v>
       </c>
-      <c r="O18" s="22">
+      <c r="O18" s="31">
         <f t="shared" ref="O18" si="7">+L18/F18</f>
         <v>7.9837618403247615E-2</v>
       </c>
     </row>
     <row r="19" spans="2:15" x14ac:dyDescent="0.25">
-      <c r="B19" s="21"/>
+      <c r="B19" s="30"/>
       <c r="C19" s="15" t="s">
         <v>31</v>
       </c>
@@ -1356,18 +1356,33 @@
       <c r="F19" s="15">
         <v>6.8</v>
       </c>
-      <c r="G19" s="21"/>
-      <c r="H19" s="21"/>
-      <c r="I19" s="21"/>
-      <c r="J19" s="21"/>
-      <c r="K19" s="21"/>
-      <c r="L19" s="21"/>
-      <c r="M19" s="22"/>
-      <c r="N19" s="22"/>
-      <c r="O19" s="22"/>
+      <c r="G19" s="30"/>
+      <c r="H19" s="30"/>
+      <c r="I19" s="30"/>
+      <c r="J19" s="30"/>
+      <c r="K19" s="30"/>
+      <c r="L19" s="30"/>
+      <c r="M19" s="31"/>
+      <c r="N19" s="31"/>
+      <c r="O19" s="31"/>
     </row>
   </sheetData>
   <mergeCells count="31">
+    <mergeCell ref="B14:B15"/>
+    <mergeCell ref="G14:G15"/>
+    <mergeCell ref="H14:H15"/>
+    <mergeCell ref="I14:I15"/>
+    <mergeCell ref="J14:J15"/>
+    <mergeCell ref="B16:B17"/>
+    <mergeCell ref="G16:G17"/>
+    <mergeCell ref="H16:H17"/>
+    <mergeCell ref="I16:I17"/>
+    <mergeCell ref="J16:J17"/>
+    <mergeCell ref="B18:B19"/>
+    <mergeCell ref="G18:G19"/>
+    <mergeCell ref="H18:H19"/>
+    <mergeCell ref="I18:I19"/>
+    <mergeCell ref="J18:J19"/>
     <mergeCell ref="L18:L19"/>
     <mergeCell ref="M18:M19"/>
     <mergeCell ref="N18:N19"/>
@@ -1384,21 +1399,6 @@
     <mergeCell ref="O14:O15"/>
     <mergeCell ref="K16:K17"/>
     <mergeCell ref="K14:K15"/>
-    <mergeCell ref="B18:B19"/>
-    <mergeCell ref="G18:G19"/>
-    <mergeCell ref="H18:H19"/>
-    <mergeCell ref="I18:I19"/>
-    <mergeCell ref="J18:J19"/>
-    <mergeCell ref="B16:B17"/>
-    <mergeCell ref="G16:G17"/>
-    <mergeCell ref="H16:H17"/>
-    <mergeCell ref="I16:I17"/>
-    <mergeCell ref="J16:J17"/>
-    <mergeCell ref="B14:B15"/>
-    <mergeCell ref="G14:G15"/>
-    <mergeCell ref="H14:H15"/>
-    <mergeCell ref="I14:I15"/>
-    <mergeCell ref="J14:J15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1426,16 +1426,16 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E2" s="30" t="s">
+      <c r="E2" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="F2" s="30"/>
-      <c r="G2" s="30"/>
-      <c r="H2" s="30"/>
-      <c r="I2" s="30"/>
-      <c r="N2" s="28"/>
-      <c r="O2" s="28"/>
-      <c r="P2" s="28"/>
+      <c r="F2" s="40"/>
+      <c r="G2" s="40"/>
+      <c r="H2" s="40"/>
+      <c r="I2" s="40"/>
+      <c r="N2" s="46"/>
+      <c r="O2" s="46"/>
+      <c r="P2" s="46"/>
     </row>
     <row r="3" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E3" s="2"/>
@@ -1468,154 +1468,154 @@
       </c>
     </row>
     <row r="5" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E5" s="29" t="s">
+      <c r="E5" s="39" t="s">
         <v>7</v>
       </c>
-      <c r="F5" s="34">
+      <c r="F5" s="44">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="34">
+      <c r="G5" s="44">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="35">
+      <c r="H5" s="45">
         <v>0.17</v>
       </c>
-      <c r="I5" s="33">
+      <c r="I5" s="43">
         <v>1.17</v>
       </c>
-      <c r="J5" s="29">
+      <c r="J5" s="39">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="29">
+      <c r="K5" s="39">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
     </row>
     <row r="6" spans="4:16" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="29"/>
-      <c r="F6" s="34"/>
-      <c r="G6" s="34"/>
-      <c r="H6" s="35"/>
-      <c r="I6" s="33"/>
-      <c r="J6" s="29"/>
-      <c r="K6" s="29"/>
+      <c r="E6" s="39"/>
+      <c r="F6" s="44"/>
+      <c r="G6" s="44"/>
+      <c r="H6" s="45"/>
+      <c r="I6" s="43"/>
+      <c r="J6" s="39"/>
+      <c r="K6" s="39"/>
       <c r="O6" s="3"/>
     </row>
     <row r="7" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E7" s="23" t="s">
+      <c r="E7" s="32" t="s">
         <v>8</v>
       </c>
-      <c r="F7" s="31">
+      <c r="F7" s="41">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="32">
+      <c r="G7" s="42">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="32">
+      <c r="H7" s="42">
         <v>0.1</v>
       </c>
-      <c r="I7" s="23">
+      <c r="I7" s="32">
         <v>0.92</v>
       </c>
-      <c r="J7" s="23">
+      <c r="J7" s="32">
         <f t="shared" ref="J7" si="0">+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="23">
+      <c r="K7" s="32">
         <f t="shared" ref="K7" si="1">+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
     </row>
     <row r="8" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E8" s="23"/>
-      <c r="F8" s="31"/>
-      <c r="G8" s="32"/>
-      <c r="H8" s="32"/>
-      <c r="I8" s="23"/>
-      <c r="J8" s="23"/>
-      <c r="K8" s="23"/>
+      <c r="E8" s="32"/>
+      <c r="F8" s="41"/>
+      <c r="G8" s="42"/>
+      <c r="H8" s="42"/>
+      <c r="I8" s="32"/>
+      <c r="J8" s="32"/>
+      <c r="K8" s="32"/>
     </row>
     <row r="9" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E9" s="23" t="s">
+      <c r="E9" s="32" t="s">
         <v>9</v>
       </c>
-      <c r="F9" s="31">
+      <c r="F9" s="41">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="32">
+      <c r="G9" s="42">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="32">
+      <c r="H9" s="42">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="23">
+      <c r="I9" s="32">
         <v>1.01</v>
       </c>
-      <c r="J9" s="23">
+      <c r="J9" s="32">
         <f t="shared" ref="J9" si="2">+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="23">
+      <c r="K9" s="32">
         <f t="shared" ref="K9" si="3">+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
     </row>
     <row r="10" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E10" s="23"/>
-      <c r="F10" s="31"/>
-      <c r="G10" s="32"/>
-      <c r="H10" s="32"/>
-      <c r="I10" s="23"/>
-      <c r="J10" s="23"/>
-      <c r="K10" s="23"/>
+      <c r="E10" s="32"/>
+      <c r="F10" s="41"/>
+      <c r="G10" s="42"/>
+      <c r="H10" s="42"/>
+      <c r="I10" s="32"/>
+      <c r="J10" s="32"/>
+      <c r="K10" s="32"/>
     </row>
     <row r="12" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E12" s="25" t="s">
+      <c r="E12" s="33" t="s">
         <v>24</v>
       </c>
-      <c r="F12" s="27"/>
-      <c r="G12" s="27"/>
-      <c r="H12" s="27"/>
-      <c r="I12" s="26"/>
-      <c r="J12" s="25" t="s">
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="34"/>
+      <c r="J12" s="33" t="s">
         <v>21</v>
       </c>
-      <c r="K12" s="27"/>
-      <c r="L12" s="27"/>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27"/>
-      <c r="O12" s="27"/>
-      <c r="P12" s="26"/>
+      <c r="K12" s="38"/>
+      <c r="L12" s="38"/>
+      <c r="M12" s="38"/>
+      <c r="N12" s="38"/>
+      <c r="O12" s="38"/>
+      <c r="P12" s="34"/>
     </row>
     <row r="13" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E13" s="2"/>
-      <c r="F13" s="25" t="s">
+      <c r="F13" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="G13" s="26"/>
-      <c r="H13" s="23" t="s">
+      <c r="G13" s="34"/>
+      <c r="H13" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="I13" s="23"/>
-      <c r="J13" s="23" t="s">
+      <c r="I13" s="32"/>
+      <c r="J13" s="32" t="s">
         <v>18</v>
       </c>
-      <c r="K13" s="23"/>
-      <c r="L13" s="23" t="s">
+      <c r="K13" s="32"/>
+      <c r="L13" s="32" t="s">
         <v>19</v>
       </c>
-      <c r="M13" s="23"/>
-      <c r="N13" s="23" t="s">
+      <c r="M13" s="32"/>
+      <c r="N13" s="32" t="s">
         <v>20</v>
       </c>
-      <c r="O13" s="23"/>
+      <c r="O13" s="32"/>
       <c r="P13" s="2" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="14" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D14" s="24"/>
+      <c r="D14" s="51"/>
       <c r="E14" s="2" t="s">
         <v>13</v>
       </c>
@@ -1630,41 +1630,41 @@
         <f>+F14*(1-$J$5/100)</f>
         <v>1.08635572</v>
       </c>
-      <c r="I14" s="39">
+      <c r="I14" s="21">
         <f>H14/$H$17</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J14" s="40">
+      <c r="J14" s="22">
         <f>+H14*(1-$K$5/100)</f>
         <v>0.99292912808000011</v>
       </c>
-      <c r="K14" s="39">
+      <c r="K14" s="21">
         <f>+J14/$J$17</f>
         <v>0.60805259681281487</v>
       </c>
-      <c r="L14" s="40">
+      <c r="L14" s="22">
         <f>+$H$14*(1-$K$7/100)</f>
         <v>1.0276925111199999</v>
       </c>
-      <c r="M14" s="39">
+      <c r="M14" s="21">
         <f>+L14/$J$25</f>
         <v>0.60542601972075083</v>
       </c>
-      <c r="N14" s="40">
+      <c r="N14" s="22">
         <f>+$H$14*(1-$K$9/100)</f>
         <v>1.01248353104</v>
       </c>
-      <c r="O14" s="39">
+      <c r="O14" s="21">
         <f>+N14/$J$33</f>
         <v>0.60477291721835513</v>
       </c>
-      <c r="P14" s="41">
+      <c r="P14" s="23">
         <f>AVERAGE(J14,L14,N14)</f>
         <v>1.0110350567466666</v>
       </c>
     </row>
     <row r="15" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D15" s="24"/>
+      <c r="D15" s="51"/>
       <c r="E15" s="2" t="s">
         <v>14</v>
       </c>
@@ -1679,41 +1679,41 @@
         <f>+F15*(1-$J$5/100)</f>
         <v>0.35450899999999996</v>
       </c>
-      <c r="I15" s="39">
+      <c r="I15" s="21">
         <f t="shared" ref="I15:I16" si="4">H15/$H$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J15" s="40">
+      <c r="J15" s="22">
         <f>+H15*(1-$K$5/100)</f>
         <v>0.324021226</v>
       </c>
-      <c r="K15" s="39">
+      <c r="K15" s="21">
         <f t="shared" ref="K15:K16" si="5">+J15/$J$17</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L15" s="40">
+      <c r="L15" s="22">
         <f>$H$15*(1-$K$7/100)</f>
         <v>0.33536551399999998</v>
       </c>
-      <c r="M15" s="39">
+      <c r="M15" s="21">
         <f t="shared" ref="M15:M16" si="6">+L15/$J$25</f>
         <v>0.19756785818293812</v>
       </c>
-      <c r="N15" s="40">
+      <c r="N15" s="22">
         <f>+$H$15*(1-$K$9/100)</f>
         <v>0.33040238799999994</v>
       </c>
-      <c r="O15" s="39">
+      <c r="O15" s="21">
         <f t="shared" ref="O15:O17" si="7">+N15/$J$33</f>
         <v>0.19735473212233082</v>
       </c>
-      <c r="P15" s="41">
+      <c r="P15" s="23">
         <f>AVERAGE(J15,L15,N15)</f>
         <v>0.32992970933333332</v>
       </c>
     </row>
     <row r="16" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D16" s="24"/>
+      <c r="D16" s="51"/>
       <c r="E16" s="2" t="s">
         <v>15</v>
       </c>
@@ -1728,41 +1728,41 @@
         <f>+F16*(1-$J$5/100)</f>
         <v>0.34575</v>
       </c>
-      <c r="I16" s="39">
+      <c r="I16" s="21">
         <f t="shared" si="4"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="J16" s="40">
+      <c r="J16" s="22">
         <f>+H16*(1-$K$5/100)</f>
         <v>0.3160155</v>
       </c>
-      <c r="K16" s="39">
+      <c r="K16" s="21">
         <f t="shared" si="5"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="L16" s="40">
+      <c r="L16" s="22">
         <f>+$H$16*(1-$K$7/100)</f>
         <v>0.32707949999999997</v>
       </c>
-      <c r="M16" s="39">
+      <c r="M16" s="21">
         <f t="shared" si="6"/>
         <v>0.19268646766866526</v>
       </c>
-      <c r="N16" s="40">
+      <c r="N16" s="22">
         <f>+$H$16*(1-$K$9/100)</f>
         <v>0.322239</v>
       </c>
-      <c r="O16" s="39">
+      <c r="O16" s="21">
         <f t="shared" si="7"/>
         <v>0.19247860740149306</v>
       </c>
-      <c r="P16" s="41">
+      <c r="P16" s="23">
         <f>AVERAGE(J16,L16,N16)</f>
         <v>0.32177799999999995</v>
       </c>
     </row>
     <row r="17" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D17" s="24"/>
+      <c r="D17" s="51"/>
       <c r="E17" s="2" t="s">
         <v>16</v>
       </c>
@@ -1778,41 +1778,41 @@
         <f t="shared" si="9"/>
         <v>1.78661472</v>
       </c>
-      <c r="I17" s="42">
+      <c r="I17" s="24">
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="J17" s="43">
+      <c r="J17" s="25">
         <f>SUM(J14:J16)</f>
         <v>1.6329658540800001</v>
       </c>
-      <c r="K17" s="41">
+      <c r="K17" s="23">
         <f t="shared" si="9"/>
         <v>1</v>
       </c>
-      <c r="L17" s="43">
+      <c r="L17" s="25">
         <f t="shared" si="9"/>
         <v>1.6901375251199999</v>
       </c>
-      <c r="M17" s="41">
+      <c r="M17" s="23">
         <f t="shared" si="9"/>
         <v>0.99568034557235419</v>
       </c>
-      <c r="N17" s="43">
+      <c r="N17" s="25">
         <f>SUM(N14:N16)</f>
         <v>1.6651249190399999</v>
       </c>
-      <c r="O17" s="41">
+      <c r="O17" s="23">
         <f t="shared" si="7"/>
         <v>0.99460625674217906</v>
       </c>
-      <c r="P17" s="41">
+      <c r="P17" s="23">
         <f>AVERAGE(J17,L17,N17)</f>
         <v>1.66274276608</v>
       </c>
     </row>
     <row r="18" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D18" s="24"/>
+      <c r="D18" s="51"/>
       <c r="E18" s="2" t="s">
         <v>17</v>
       </c>
@@ -1824,430 +1824,430 @@
         <f>+H17/F17-1</f>
         <v>-7.8000000000000069E-2</v>
       </c>
-      <c r="I18" s="44" t="s">
+      <c r="I18" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="J18" s="39">
+      <c r="J18" s="21">
         <f>+J17/I17-1</f>
         <v>0.63296585408000006</v>
       </c>
-      <c r="K18" s="44"/>
-      <c r="L18" s="39">
+      <c r="K18" s="26"/>
+      <c r="L18" s="21">
         <f>+L17/K17-1</f>
         <v>0.69013752511999993</v>
       </c>
-      <c r="M18" s="44"/>
-      <c r="N18" s="39">
+      <c r="M18" s="26"/>
+      <c r="N18" s="21">
         <f>+N17/M17-1</f>
         <v>0.67234888831999995</v>
       </c>
-      <c r="O18" s="44"/>
-      <c r="P18" s="44"/>
+      <c r="O18" s="26"/>
+      <c r="P18" s="26"/>
     </row>
     <row r="20" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E20" s="23" t="s">
+      <c r="E20" s="32" t="s">
         <v>23</v>
       </c>
-      <c r="F20" s="23"/>
-      <c r="G20" s="23"/>
-      <c r="H20" s="23"/>
-      <c r="I20" s="23"/>
-      <c r="J20" s="23"/>
-      <c r="K20" s="23"/>
-      <c r="L20" s="23"/>
+      <c r="F20" s="32"/>
+      <c r="G20" s="32"/>
+      <c r="H20" s="32"/>
+      <c r="I20" s="32"/>
+      <c r="J20" s="32"/>
+      <c r="K20" s="32"/>
+      <c r="L20" s="32"/>
     </row>
     <row r="21" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E21" s="44"/>
-      <c r="F21" s="45" t="s">
+      <c r="E21" s="26"/>
+      <c r="F21" s="48" t="s">
         <v>10</v>
       </c>
-      <c r="G21" s="46"/>
-      <c r="H21" s="47" t="s">
+      <c r="G21" s="49"/>
+      <c r="H21" s="50" t="s">
         <v>11</v>
       </c>
-      <c r="I21" s="47"/>
-      <c r="J21" s="47" t="s">
+      <c r="I21" s="50"/>
+      <c r="J21" s="50" t="s">
         <v>12</v>
       </c>
-      <c r="K21" s="47"/>
-      <c r="L21" s="48"/>
-      <c r="M21" s="49"/>
-      <c r="N21" s="49"/>
+      <c r="K21" s="50"/>
+      <c r="L21" s="27"/>
+      <c r="M21" s="28"/>
+      <c r="N21" s="28"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D22" s="24"/>
-      <c r="E22" s="44" t="s">
+      <c r="D22" s="51"/>
+      <c r="E22" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="F22" s="40">
+      <c r="F22" s="22">
         <v>1.1782600000000001</v>
       </c>
-      <c r="G22" s="39">
+      <c r="G22" s="21">
         <f>+F22/$F$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="H22" s="40">
+      <c r="H22" s="22">
         <f>+F22*(1-$J$7/100)</f>
         <v>1.09106876</v>
       </c>
-      <c r="I22" s="39">
+      <c r="I22" s="21">
         <f>H22/$H$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J22" s="40">
+      <c r="J22" s="22">
         <f>+$H$22*(1-$K$7/100)</f>
         <v>1.0321510469599999</v>
       </c>
-      <c r="K22" s="39">
+      <c r="K22" s="21">
         <f>+J22/$J$25</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L22" s="40"/>
-      <c r="M22" s="49"/>
-      <c r="N22" s="49"/>
+      <c r="L22" s="22"/>
+      <c r="M22" s="28"/>
+      <c r="N22" s="28"/>
     </row>
     <row r="23" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D23" s="24"/>
-      <c r="E23" s="44" t="s">
+      <c r="D23" s="51"/>
+      <c r="E23" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="F23" s="40">
+      <c r="F23" s="22">
         <v>0.38450000000000001</v>
       </c>
-      <c r="G23" s="39">
+      <c r="G23" s="21">
         <f t="shared" ref="G23:G24" si="10">+F23/$F$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="H23" s="40">
+      <c r="H23" s="22">
         <f t="shared" ref="H23:H25" si="11">+F23*(1-$J$7/100)</f>
         <v>0.356047</v>
       </c>
-      <c r="I23" s="39">
+      <c r="I23" s="21">
         <f>H23/$H$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J23" s="40">
+      <c r="J23" s="22">
         <f>+$H$23*(1-$K$7/100)</f>
         <v>0.33682046199999999</v>
       </c>
-      <c r="K23" s="39">
+      <c r="K23" s="21">
         <f t="shared" ref="K23:K24" si="12">+J23/$J$25</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="L23" s="40"/>
-      <c r="M23" s="49"/>
-      <c r="N23" s="49"/>
+      <c r="L23" s="22"/>
+      <c r="M23" s="28"/>
+      <c r="N23" s="28"/>
     </row>
     <row r="24" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D24" s="24"/>
-      <c r="E24" s="44" t="s">
+      <c r="D24" s="51"/>
+      <c r="E24" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="F24" s="40">
+      <c r="F24" s="22">
         <v>0.375</v>
       </c>
-      <c r="G24" s="39">
+      <c r="G24" s="21">
         <f t="shared" si="10"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="H24" s="40">
+      <c r="H24" s="22">
         <f t="shared" si="11"/>
         <v>0.34724999999999995</v>
       </c>
-      <c r="I24" s="39">
+      <c r="I24" s="21">
         <f>H24/$H$25</f>
         <v>0.19352241763685901</v>
       </c>
-      <c r="J24" s="40">
+      <c r="J24" s="22">
         <f>+$H$24*(1-$K$7/100)</f>
         <v>0.32849849999999992</v>
       </c>
-      <c r="K24" s="39">
+      <c r="K24" s="21">
         <f t="shared" si="12"/>
         <v>0.19352241763685901</v>
       </c>
-      <c r="L24" s="40"/>
-      <c r="M24" s="49"/>
-      <c r="N24" s="49"/>
+      <c r="L24" s="22"/>
+      <c r="M24" s="28"/>
+      <c r="N24" s="28"/>
     </row>
     <row r="25" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D25" s="24"/>
-      <c r="E25" s="44" t="s">
+      <c r="D25" s="51"/>
+      <c r="E25" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F25" s="43">
+      <c r="F25" s="25">
         <f t="shared" ref="F25:K25" si="13">SUM(F22:F24)</f>
         <v>1.9377600000000001</v>
       </c>
-      <c r="G25" s="42">
+      <c r="G25" s="24">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="H25" s="40">
+      <c r="H25" s="22">
         <f t="shared" si="11"/>
         <v>1.79436576</v>
       </c>
-      <c r="I25" s="42">
+      <c r="I25" s="24">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="J25" s="43">
+      <c r="J25" s="25">
         <f t="shared" si="13"/>
         <v>1.6974700089599999</v>
       </c>
-      <c r="K25" s="41">
+      <c r="K25" s="23">
         <f t="shared" si="13"/>
         <v>1</v>
       </c>
-      <c r="L25" s="40"/>
-      <c r="M25" s="49"/>
-      <c r="N25" s="49"/>
+      <c r="L25" s="22"/>
+      <c r="M25" s="28"/>
+      <c r="N25" s="28"/>
     </row>
     <row r="26" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="D26" s="24"/>
-      <c r="E26" s="44" t="s">
+      <c r="D26" s="51"/>
+      <c r="E26" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="F26" s="44"/>
-      <c r="G26" s="44" t="s">
+      <c r="F26" s="26"/>
+      <c r="G26" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="H26" s="39">
+      <c r="H26" s="21">
         <f>+H25/F25-1</f>
         <v>-7.4000000000000066E-2</v>
       </c>
-      <c r="I26" s="44" t="s">
+      <c r="I26" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="J26" s="39">
+      <c r="J26" s="21">
         <f>+J25/I25-1</f>
         <v>0.69747000895999989</v>
       </c>
-      <c r="K26" s="44"/>
-      <c r="L26" s="44"/>
-      <c r="M26" s="49"/>
-      <c r="N26" s="49"/>
+      <c r="K26" s="26"/>
+      <c r="L26" s="26"/>
+      <c r="M26" s="28"/>
+      <c r="N26" s="28"/>
     </row>
     <row r="27" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E27" s="49"/>
-      <c r="F27" s="49"/>
-      <c r="G27" s="49"/>
-      <c r="H27" s="49"/>
-      <c r="I27" s="49"/>
-      <c r="J27" s="49"/>
-      <c r="K27" s="49"/>
-      <c r="L27" s="49"/>
-      <c r="M27" s="49"/>
-      <c r="N27" s="49"/>
+      <c r="E27" s="28"/>
+      <c r="F27" s="28"/>
+      <c r="G27" s="28"/>
+      <c r="H27" s="28"/>
+      <c r="I27" s="28"/>
+      <c r="J27" s="28"/>
+      <c r="K27" s="28"/>
+      <c r="L27" s="28"/>
+      <c r="M27" s="28"/>
+      <c r="N27" s="28"/>
     </row>
     <row r="28" spans="4:16" x14ac:dyDescent="0.25">
-      <c r="E28" s="45" t="s">
+      <c r="E28" s="48" t="s">
         <v>22</v>
       </c>
-      <c r="F28" s="50"/>
-      <c r="G28" s="50"/>
-      <c r="H28" s="50"/>
-      <c r="I28" s="50"/>
-      <c r="J28" s="50"/>
-      <c r="K28" s="50"/>
-      <c r="L28" s="46"/>
-      <c r="M28" s="49"/>
-      <c r="N28" s="49"/>
+      <c r="F28" s="52"/>
+      <c r="G28" s="52"/>
+      <c r="H28" s="52"/>
+      <c r="I28" s="52"/>
+      <c r="J28" s="52"/>
+      <c r="K28" s="52"/>
+      <c r="L28" s="49"/>
+      <c r="M28" s="28"/>
+      <c r="N28" s="28"/>
     </row>
     <row r="29" spans="4:16" x14ac:dyDescent="0.25">
       <c r="E29" s="2"/>
-      <c r="F29" s="25" t="s">
+      <c r="F29" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="G29" s="26"/>
-      <c r="H29" s="23" t="s">
+      <c r="G29" s="34"/>
+      <c r="H29" s="32" t="s">
         <v>11</v>
       </c>
-      <c r="I29" s="23"/>
-      <c r="J29" s="23" t="s">
+      <c r="I29" s="32"/>
+      <c r="J29" s="32" t="s">
         <v>12</v>
       </c>
-      <c r="K29" s="23"/>
+      <c r="K29" s="32"/>
       <c r="L29" s="10"/>
     </row>
-    <row r="30" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D30" s="51"/>
-      <c r="E30" s="44" t="s">
+    <row r="30" spans="4:16" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D30" s="47"/>
+      <c r="E30" s="26" t="s">
         <v>13</v>
       </c>
-      <c r="F30" s="40">
+      <c r="F30" s="22">
         <v>1.1782600000000001</v>
       </c>
-      <c r="G30" s="39">
+      <c r="G30" s="21">
         <f>+F30/$F$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="H30" s="40">
+      <c r="H30" s="22">
         <f>+F30*(1-$J$9/100)</f>
         <v>1.0922470200000001</v>
       </c>
-      <c r="I30" s="39">
+      <c r="I30" s="21">
         <f>H30/$H$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="J30" s="40">
+      <c r="J30" s="22">
         <f>+$H$30*(1-$K$9/100)</f>
         <v>1.0179742226399999</v>
       </c>
-      <c r="K30" s="39">
+      <c r="K30" s="21">
         <f>+J30/$J$33</f>
         <v>0.60805259681281476</v>
       </c>
-      <c r="L30" s="40"/>
-    </row>
-    <row r="31" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="51"/>
-      <c r="E31" s="44" t="s">
+      <c r="L30" s="22"/>
+    </row>
+    <row r="31" spans="4:16" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D31" s="47"/>
+      <c r="E31" s="26" t="s">
         <v>14</v>
       </c>
-      <c r="F31" s="40">
+      <c r="F31" s="22">
         <v>0.38450000000000001</v>
       </c>
-      <c r="G31" s="39">
+      <c r="G31" s="21">
         <f t="shared" ref="G31:G32" si="14">+F31/$F$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="H31" s="40">
+      <c r="H31" s="22">
         <f t="shared" ref="H31:H32" si="15">+F31*(1-$J$9/100)</f>
         <v>0.35643150000000001</v>
       </c>
-      <c r="I31" s="39">
+      <c r="I31" s="21">
         <f>H31/$H$33</f>
         <v>0.19842498555032614</v>
       </c>
-      <c r="J31" s="40">
+      <c r="J31" s="22">
         <f>+$H$31*(1-$K$9/100)</f>
         <v>0.33219415800000002</v>
       </c>
-      <c r="K31" s="39">
+      <c r="K31" s="21">
         <f t="shared" ref="K31:K33" si="16">+J31/$J$33</f>
         <v>0.19842498555032617</v>
       </c>
-      <c r="L31" s="40"/>
-    </row>
-    <row r="32" spans="4:16" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="51"/>
-      <c r="E32" s="44" t="s">
+      <c r="L31" s="22"/>
+    </row>
+    <row r="32" spans="4:16" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D32" s="47"/>
+      <c r="E32" s="26" t="s">
         <v>15</v>
       </c>
-      <c r="F32" s="40">
+      <c r="F32" s="22">
         <v>0.375</v>
       </c>
-      <c r="G32" s="39">
+      <c r="G32" s="21">
         <f t="shared" si="14"/>
         <v>0.19352241763685904</v>
       </c>
-      <c r="H32" s="40">
+      <c r="H32" s="22">
         <f t="shared" si="15"/>
         <v>0.34762500000000002</v>
       </c>
-      <c r="I32" s="39">
+      <c r="I32" s="21">
         <f>H32/$H$33</f>
         <v>0.19352241763685904</v>
       </c>
-      <c r="J32" s="40">
+      <c r="J32" s="22">
         <f>+$H$32*(1-$K$9/100)</f>
         <v>0.32398650000000001</v>
       </c>
-      <c r="K32" s="39">
+      <c r="K32" s="21">
         <f t="shared" si="16"/>
         <v>0.19352241763685907</v>
       </c>
-      <c r="L32" s="40"/>
-    </row>
-    <row r="33" spans="4:14" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="51"/>
-      <c r="E33" s="44" t="s">
+      <c r="L32" s="22"/>
+    </row>
+    <row r="33" spans="4:14" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D33" s="47"/>
+      <c r="E33" s="26" t="s">
         <v>16</v>
       </c>
-      <c r="F33" s="43">
+      <c r="F33" s="25">
         <f>SUM(F30:F32)</f>
         <v>1.9377600000000001</v>
       </c>
-      <c r="G33" s="42">
+      <c r="G33" s="24">
         <f>SUM(G30:G32)</f>
         <v>1</v>
       </c>
-      <c r="H33" s="43">
+      <c r="H33" s="25">
         <f>SUM(H30:H32)</f>
         <v>1.7963035200000002</v>
       </c>
-      <c r="I33" s="42">
+      <c r="I33" s="24">
         <f>SUM(I30:I32)</f>
         <v>1</v>
       </c>
-      <c r="J33" s="43">
+      <c r="J33" s="25">
         <f>SUM(J30:J32)</f>
         <v>1.67415488064</v>
       </c>
-      <c r="K33" s="41">
+      <c r="K33" s="23">
         <f t="shared" si="16"/>
         <v>1</v>
       </c>
-      <c r="L33" s="40"/>
-    </row>
-    <row r="34" spans="4:14" s="49" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="D34" s="51"/>
-      <c r="E34" s="44" t="s">
+      <c r="L33" s="22"/>
+    </row>
+    <row r="34" spans="4:14" s="28" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="D34" s="47"/>
+      <c r="E34" s="26" t="s">
         <v>17</v>
       </c>
-      <c r="F34" s="44"/>
-      <c r="G34" s="44" t="s">
+      <c r="F34" s="26"/>
+      <c r="G34" s="26" t="s">
         <v>2</v>
       </c>
-      <c r="H34" s="39">
+      <c r="H34" s="21">
         <f>+H33/F33-1</f>
         <v>-7.2999999999999954E-2</v>
       </c>
-      <c r="I34" s="44" t="s">
+      <c r="I34" s="26" t="s">
         <v>3</v>
       </c>
-      <c r="J34" s="39">
+      <c r="J34" s="21">
         <f>+J33/I33-1</f>
         <v>0.67415488063999995</v>
       </c>
-      <c r="K34" s="44"/>
-      <c r="L34" s="52"/>
+      <c r="K34" s="26"/>
+      <c r="L34" s="29"/>
     </row>
     <row r="36" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="E36" s="23" t="s">
+      <c r="E36" s="32" t="s">
         <v>24</v>
       </c>
-      <c r="F36" s="23"/>
-      <c r="G36" s="23"/>
-      <c r="H36" s="23" t="s">
+      <c r="F36" s="32"/>
+      <c r="G36" s="32"/>
+      <c r="H36" s="32" t="s">
         <v>21</v>
       </c>
-      <c r="I36" s="23"/>
-      <c r="J36" s="23"/>
-      <c r="K36" s="23"/>
-      <c r="L36" s="23"/>
-      <c r="M36" s="23"/>
-      <c r="N36" s="23"/>
+      <c r="I36" s="32"/>
+      <c r="J36" s="32"/>
+      <c r="K36" s="32"/>
+      <c r="L36" s="32"/>
+      <c r="M36" s="32"/>
+      <c r="N36" s="32"/>
     </row>
     <row r="37" spans="4:14" x14ac:dyDescent="0.25">
       <c r="E37" s="2"/>
-      <c r="F37" s="25" t="s">
+      <c r="F37" s="33" t="s">
         <v>10</v>
       </c>
-      <c r="G37" s="26"/>
-      <c r="H37" s="36" t="s">
+      <c r="G37" s="34"/>
+      <c r="H37" s="35" t="s">
         <v>54</v>
       </c>
-      <c r="I37" s="36"/>
-      <c r="J37" s="36" t="s">
+      <c r="I37" s="35"/>
+      <c r="J37" s="35" t="s">
         <v>55</v>
       </c>
-      <c r="K37" s="36"/>
-      <c r="L37" s="37" t="s">
+      <c r="K37" s="35"/>
+      <c r="L37" s="36" t="s">
         <v>56</v>
       </c>
-      <c r="M37" s="38"/>
+      <c r="M37" s="37"/>
       <c r="N37" s="2" t="s">
         <v>57</v>
       </c>
@@ -2438,19 +2438,24 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="E36:G36"/>
-    <mergeCell ref="F37:G37"/>
-    <mergeCell ref="H37:I37"/>
-    <mergeCell ref="J37:K37"/>
-    <mergeCell ref="L37:M37"/>
-    <mergeCell ref="H36:N36"/>
-    <mergeCell ref="L13:M13"/>
-    <mergeCell ref="N13:O13"/>
-    <mergeCell ref="E12:I12"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="H13:I13"/>
-    <mergeCell ref="J13:K13"/>
-    <mergeCell ref="J12:P12"/>
+    <mergeCell ref="D14:D18"/>
+    <mergeCell ref="F29:G29"/>
+    <mergeCell ref="H29:I29"/>
+    <mergeCell ref="J29:K29"/>
+    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="D30:D34"/>
+    <mergeCell ref="F21:G21"/>
+    <mergeCell ref="H21:I21"/>
+    <mergeCell ref="J21:K21"/>
+    <mergeCell ref="D22:D26"/>
+    <mergeCell ref="E28:L28"/>
+    <mergeCell ref="N2:P2"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="E9:E10"/>
@@ -2467,24 +2472,19 @@
     <mergeCell ref="F7:F8"/>
     <mergeCell ref="G7:G8"/>
     <mergeCell ref="H7:H8"/>
-    <mergeCell ref="N2:P2"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="D30:D34"/>
-    <mergeCell ref="F21:G21"/>
-    <mergeCell ref="H21:I21"/>
-    <mergeCell ref="J21:K21"/>
-    <mergeCell ref="D22:D26"/>
-    <mergeCell ref="E28:L28"/>
-    <mergeCell ref="D14:D18"/>
-    <mergeCell ref="F29:G29"/>
-    <mergeCell ref="H29:I29"/>
-    <mergeCell ref="J29:K29"/>
-    <mergeCell ref="E20:L20"/>
+    <mergeCell ref="L13:M13"/>
+    <mergeCell ref="N13:O13"/>
+    <mergeCell ref="E12:I12"/>
+    <mergeCell ref="F13:G13"/>
+    <mergeCell ref="H13:I13"/>
+    <mergeCell ref="J13:K13"/>
+    <mergeCell ref="J12:P12"/>
+    <mergeCell ref="E36:G36"/>
+    <mergeCell ref="F37:G37"/>
+    <mergeCell ref="H37:I37"/>
+    <mergeCell ref="J37:K37"/>
+    <mergeCell ref="L37:M37"/>
+    <mergeCell ref="H36:N36"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Limpieza de archivos duplicados y copias de seguridad manuales
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="843" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{7729FC3C-BFA3-4B1F-9682-C06889AED32E}"/>
+  <xr:revisionPtr revIDLastSave="845" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E90F0389-14EF-5126-90FC-55F9316E030E}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13020" activeTab="2" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
+    <workbookView xWindow="8880" yWindow="2070" windowWidth="12525" windowHeight="8490" activeTab="2" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
   <sheets>
     <sheet name="CALCULO SAMPLE COMPARISON " sheetId="3" r:id="rId1"/>
@@ -572,61 +572,61 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="8" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="7" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="6" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -731,10 +731,6 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1073,13 +1069,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="35" t="s">
+      <c r="A1" s="34" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="35"/>
-      <c r="C1" s="35"/>
-      <c r="D1" s="35"/>
-      <c r="E1" s="35"/>
+      <c r="B1" s="34"/>
+      <c r="C1" s="34"/>
+      <c r="D1" s="34"/>
+      <c r="E1" s="34"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1309,7 +1305,7 @@
       </c>
     </row>
     <row r="15" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="34" t="s">
+      <c r="B15" s="35" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -1324,27 +1320,27 @@
       <c r="F15" s="28">
         <v>-3.6</v>
       </c>
-      <c r="G15" s="34">
+      <c r="G15" s="35">
         <f>+D16-D15</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H15" s="34">
+      <c r="H15" s="35">
         <f>+E16-E15</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I15" s="34">
+      <c r="I15" s="35">
         <f>+F16-F15</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J15" s="34">
+      <c r="J15" s="35">
         <f>+ABS(G15)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K15" s="34">
+      <c r="K15" s="35">
         <f>+ABS(H15)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L15" s="34">
+      <c r="L15" s="35">
         <f>+ABS(I15)</f>
         <v>0.12999999999999989</v>
       </c>
@@ -1386,7 +1382,7 @@
       </c>
     </row>
     <row r="16" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="34"/>
+      <c r="B16" s="35"/>
       <c r="C16" s="7" t="s">
         <v>26</v>
       </c>
@@ -1399,15 +1395,15 @@
       <c r="F16" s="28">
         <v>-3.47</v>
       </c>
-      <c r="G16" s="34"/>
-      <c r="H16" s="34"/>
-      <c r="I16" s="34"/>
-      <c r="J16" s="34"/>
-      <c r="K16" s="34"/>
-      <c r="L16" s="34"/>
-      <c r="M16" s="34"/>
-      <c r="N16" s="34"/>
-      <c r="O16" s="34"/>
+      <c r="G16" s="35"/>
+      <c r="H16" s="35"/>
+      <c r="I16" s="35"/>
+      <c r="J16" s="35"/>
+      <c r="K16" s="35"/>
+      <c r="L16" s="35"/>
+      <c r="M16" s="35"/>
+      <c r="N16" s="35"/>
+      <c r="O16" s="35"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
@@ -1416,7 +1412,7 @@
       <c r="U16" s="7"/>
     </row>
     <row r="17" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="34" t="s">
+      <c r="B17" s="35" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -1431,27 +1427,27 @@
       <c r="F17" s="28">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G17" s="34">
+      <c r="G17" s="35">
         <f>+D18-D17</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H17" s="34">
+      <c r="H17" s="35">
         <f>+E18-E17</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I17" s="34">
+      <c r="I17" s="35">
         <f>+F18-F17</f>
         <v>-9.39</v>
       </c>
-      <c r="J17" s="34">
+      <c r="J17" s="35">
         <f>+ABS(G17)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K17" s="34">
+      <c r="K17" s="35">
         <f>+ABS(H17)</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L17" s="34">
+      <c r="L17" s="35">
         <f>+ABS(I17)</f>
         <v>9.39</v>
       </c>
@@ -1493,7 +1489,7 @@
       </c>
     </row>
     <row r="18" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="34"/>
+      <c r="B18" s="35"/>
       <c r="C18" s="7" t="s">
         <v>26</v>
       </c>
@@ -1506,15 +1502,15 @@
       <c r="F18" s="28">
         <v>-4.33</v>
       </c>
-      <c r="G18" s="34"/>
-      <c r="H18" s="34"/>
-      <c r="I18" s="34"/>
-      <c r="J18" s="34"/>
-      <c r="K18" s="34"/>
-      <c r="L18" s="34"/>
-      <c r="M18" s="34"/>
-      <c r="N18" s="34"/>
-      <c r="O18" s="34"/>
+      <c r="G18" s="35"/>
+      <c r="H18" s="35"/>
+      <c r="I18" s="35"/>
+      <c r="J18" s="35"/>
+      <c r="K18" s="35"/>
+      <c r="L18" s="35"/>
+      <c r="M18" s="35"/>
+      <c r="N18" s="35"/>
+      <c r="O18" s="35"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
@@ -1523,7 +1519,7 @@
       <c r="U18" s="7"/>
     </row>
     <row r="19" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="34" t="s">
+      <c r="B19" s="35" t="s">
         <v>36</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -1538,27 +1534,27 @@
       <c r="F19" s="28">
         <v>7.39</v>
       </c>
-      <c r="G19" s="34">
+      <c r="G19" s="35">
         <f>+D20-D19</f>
         <v>-4</v>
       </c>
-      <c r="H19" s="34">
+      <c r="H19" s="35">
         <f>+E20-E19</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I19" s="34">
+      <c r="I19" s="35">
         <f>+F20-F19</f>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J19" s="34">
+      <c r="J19" s="35">
         <f>+ABS(G19)</f>
         <v>4</v>
       </c>
-      <c r="K19" s="34">
+      <c r="K19" s="35">
         <f>+ABS(H19)</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L19" s="34">
+      <c r="L19" s="35">
         <f>+ABS(I19)</f>
         <v>0.58999999999999986</v>
       </c>
@@ -1600,7 +1596,7 @@
       </c>
     </row>
     <row r="20" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="34"/>
+      <c r="B20" s="35"/>
       <c r="C20" s="7" t="s">
         <v>26</v>
       </c>
@@ -1613,15 +1609,15 @@
       <c r="F20" s="28">
         <v>6.8</v>
       </c>
-      <c r="G20" s="34"/>
-      <c r="H20" s="34"/>
-      <c r="I20" s="34"/>
-      <c r="J20" s="34"/>
-      <c r="K20" s="34"/>
-      <c r="L20" s="34"/>
-      <c r="M20" s="34"/>
-      <c r="N20" s="34"/>
-      <c r="O20" s="34"/>
+      <c r="G20" s="35"/>
+      <c r="H20" s="35"/>
+      <c r="I20" s="35"/>
+      <c r="J20" s="35"/>
+      <c r="K20" s="35"/>
+      <c r="L20" s="35"/>
+      <c r="M20" s="35"/>
+      <c r="N20" s="35"/>
+      <c r="O20" s="35"/>
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
@@ -1675,6 +1671,22 @@
     </row>
   </sheetData>
   <mergeCells count="32">
+    <mergeCell ref="K15:K16"/>
+    <mergeCell ref="B19:B20"/>
+    <mergeCell ref="G19:G20"/>
+    <mergeCell ref="H19:H20"/>
+    <mergeCell ref="I19:I20"/>
+    <mergeCell ref="J19:J20"/>
+    <mergeCell ref="B17:B18"/>
+    <mergeCell ref="G17:G18"/>
+    <mergeCell ref="H17:H18"/>
+    <mergeCell ref="I17:I18"/>
+    <mergeCell ref="J17:J18"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="G15:G16"/>
+    <mergeCell ref="H15:H16"/>
+    <mergeCell ref="I15:I16"/>
+    <mergeCell ref="J15:J16"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="L19:L20"/>
     <mergeCell ref="M19:M20"/>
@@ -1691,22 +1703,6 @@
     <mergeCell ref="N15:N16"/>
     <mergeCell ref="O15:O16"/>
     <mergeCell ref="K17:K18"/>
-    <mergeCell ref="K15:K16"/>
-    <mergeCell ref="B19:B20"/>
-    <mergeCell ref="G19:G20"/>
-    <mergeCell ref="H19:H20"/>
-    <mergeCell ref="I19:I20"/>
-    <mergeCell ref="J19:J20"/>
-    <mergeCell ref="B17:B18"/>
-    <mergeCell ref="G17:G18"/>
-    <mergeCell ref="H17:H18"/>
-    <mergeCell ref="I17:I18"/>
-    <mergeCell ref="J17:J18"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="G15:G16"/>
-    <mergeCell ref="H15:H16"/>
-    <mergeCell ref="I15:I16"/>
-    <mergeCell ref="J15:J16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1786,7 +1782,7 @@
       <c r="N4" s="2"/>
     </row>
     <row r="5" spans="4:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E5" s="39" t="s">
+      <c r="E5" s="50" t="s">
         <v>6</v>
       </c>
       <c r="F5" s="47">
@@ -1801,11 +1797,11 @@
       <c r="I5" s="45">
         <v>1.17</v>
       </c>
-      <c r="J5" s="39">
+      <c r="J5" s="50">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="40">
+      <c r="K5" s="51">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
@@ -1823,13 +1819,13 @@
       </c>
     </row>
     <row r="6" spans="4:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="39"/>
+      <c r="E6" s="50"/>
       <c r="F6" s="48"/>
       <c r="G6" s="48"/>
       <c r="H6" s="48"/>
       <c r="I6" s="46"/>
-      <c r="J6" s="39"/>
-      <c r="K6" s="40"/>
+      <c r="J6" s="50"/>
+      <c r="K6" s="51"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
@@ -1854,7 +1850,7 @@
         <f>+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="41">
+      <c r="K7" s="38">
         <f>+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
@@ -1878,7 +1874,7 @@
       <c r="H8" s="43"/>
       <c r="I8" s="43"/>
       <c r="J8" s="37"/>
-      <c r="K8" s="41"/>
+      <c r="K8" s="38"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -1903,7 +1899,7 @@
         <f>+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="41">
+      <c r="K9" s="38">
         <f>+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
@@ -1927,7 +1923,7 @@
       <c r="H10" s="43"/>
       <c r="I10" s="43"/>
       <c r="J10" s="37"/>
-      <c r="K10" s="41"/>
+      <c r="K10" s="38"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -1938,18 +1934,18 @@
       <c r="H11" s="9"/>
     </row>
     <row r="12" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="41" t="s">
+      <c r="E12" s="38" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="50"/>
-      <c r="G12" s="50"/>
-      <c r="H12" s="50"/>
-      <c r="I12" s="50"/>
-      <c r="J12" s="50"/>
-      <c r="K12" s="50"/>
-      <c r="L12" s="50"/>
-      <c r="M12" s="50"/>
-      <c r="N12" s="51"/>
+      <c r="F12" s="39"/>
+      <c r="G12" s="39"/>
+      <c r="H12" s="39"/>
+      <c r="I12" s="39"/>
+      <c r="J12" s="39"/>
+      <c r="K12" s="39"/>
+      <c r="L12" s="39"/>
+      <c r="M12" s="39"/>
+      <c r="N12" s="40"/>
     </row>
     <row r="13" spans="4:14" x14ac:dyDescent="0.25">
       <c r="E13" s="37" t="s">
@@ -1959,13 +1955,13 @@
       <c r="G13" s="37"/>
       <c r="H13" s="37"/>
       <c r="I13" s="37"/>
-      <c r="J13" s="41" t="s">
+      <c r="J13" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="50"/>
-      <c r="L13" s="50"/>
-      <c r="M13" s="50"/>
-      <c r="N13" s="51"/>
+      <c r="K13" s="39"/>
+      <c r="L13" s="39"/>
+      <c r="M13" s="39"/>
+      <c r="N13" s="40"/>
     </row>
     <row r="14" spans="4:14" x14ac:dyDescent="0.2">
       <c r="E14" s="2"/>
@@ -1992,7 +1988,7 @@
       </c>
     </row>
     <row r="15" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D15" s="38"/>
+      <c r="D15" s="52"/>
       <c r="E15" s="29" t="s">
         <v>12</v>
       </c>
@@ -2028,7 +2024,7 @@
       <c r="N15" s="26"/>
     </row>
     <row r="16" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="38"/>
+      <c r="D16" s="52"/>
       <c r="E16" s="29" t="s">
         <v>13</v>
       </c>
@@ -2060,7 +2056,7 @@
       <c r="N16" s="2"/>
     </row>
     <row r="17" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="38"/>
+      <c r="D17" s="52"/>
       <c r="E17" s="29" t="s">
         <v>14</v>
       </c>
@@ -2092,7 +2088,7 @@
       <c r="N17" s="2"/>
     </row>
     <row r="18" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="38"/>
+      <c r="D18" s="52"/>
       <c r="E18" s="2" t="s">
         <v>15</v>
       </c>
@@ -2134,7 +2130,7 @@
       </c>
     </row>
     <row r="19" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D19" s="38"/>
+      <c r="D19" s="52"/>
       <c r="E19" s="2" t="s">
         <v>16</v>
       </c>
@@ -2156,20 +2152,20 @@
       <c r="O19" s="27"/>
     </row>
     <row r="21" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E21" s="52" t="s">
+      <c r="E21" s="41" t="s">
         <v>55</v>
       </c>
-      <c r="F21" s="35"/>
-      <c r="G21" s="35"/>
-      <c r="H21" s="35"/>
-      <c r="I21" s="35"/>
-      <c r="J21" s="35"/>
-      <c r="K21" s="35"/>
-      <c r="L21" s="35"/>
-      <c r="M21" s="35"/>
-      <c r="N21" s="35"/>
-      <c r="O21" s="35"/>
-      <c r="P21" s="35"/>
+      <c r="F21" s="34"/>
+      <c r="G21" s="34"/>
+      <c r="H21" s="34"/>
+      <c r="I21" s="34"/>
+      <c r="J21" s="34"/>
+      <c r="K21" s="34"/>
+      <c r="L21" s="34"/>
+      <c r="M21" s="34"/>
+      <c r="N21" s="34"/>
+      <c r="O21" s="34"/>
+      <c r="P21" s="34"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E22" s="2"/>
@@ -2200,7 +2196,7 @@
       </c>
     </row>
     <row r="23" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="38"/>
+      <c r="D23" s="52"/>
       <c r="E23" s="29" t="s">
         <v>12</v>
       </c>
@@ -2240,7 +2236,7 @@
       <c r="P23" s="2"/>
     </row>
     <row r="24" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="38"/>
+      <c r="D24" s="52"/>
       <c r="E24" s="29" t="s">
         <v>13</v>
       </c>
@@ -2280,7 +2276,7 @@
       <c r="P24" s="2"/>
     </row>
     <row r="25" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="38"/>
+      <c r="D25" s="52"/>
       <c r="E25" s="29" t="s">
         <v>14</v>
       </c>
@@ -2320,7 +2316,7 @@
       <c r="P25" s="2"/>
     </row>
     <row r="26" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D26" s="38"/>
+      <c r="D26" s="52"/>
       <c r="E26" s="2" t="s">
         <v>15</v>
       </c>
@@ -2370,7 +2366,7 @@
       </c>
     </row>
     <row r="27" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D27" s="38"/>
+      <c r="D27" s="52"/>
       <c r="E27" s="2" t="s">
         <v>16</v>
       </c>
@@ -2403,20 +2399,20 @@
       <c r="P27" s="2"/>
     </row>
     <row r="29" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E29" s="52" t="s">
+      <c r="E29" s="41" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="35"/>
-      <c r="G29" s="35"/>
-      <c r="H29" s="35"/>
-      <c r="I29" s="35"/>
-      <c r="J29" s="35"/>
-      <c r="K29" s="35"/>
-      <c r="L29" s="35"/>
-      <c r="M29" s="35"/>
-      <c r="N29" s="35"/>
-      <c r="O29" s="35"/>
-      <c r="P29" s="35"/>
+      <c r="F29" s="34"/>
+      <c r="G29" s="34"/>
+      <c r="H29" s="34"/>
+      <c r="I29" s="34"/>
+      <c r="J29" s="34"/>
+      <c r="K29" s="34"/>
+      <c r="L29" s="34"/>
+      <c r="M29" s="34"/>
+      <c r="N29" s="34"/>
+      <c r="O29" s="34"/>
+      <c r="P29" s="34"/>
     </row>
     <row r="30" spans="4:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="E30" s="2"/>
@@ -2447,7 +2443,7 @@
       </c>
     </row>
     <row r="31" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="38"/>
+      <c r="D31" s="52"/>
       <c r="E31" s="29" t="s">
         <v>12</v>
       </c>
@@ -2487,7 +2483,7 @@
       <c r="P31" s="2"/>
     </row>
     <row r="32" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="38"/>
+      <c r="D32" s="52"/>
       <c r="E32" s="29" t="s">
         <v>13</v>
       </c>
@@ -2527,7 +2523,7 @@
       <c r="P32" s="2"/>
     </row>
     <row r="33" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="38"/>
+      <c r="D33" s="52"/>
       <c r="E33" s="29" t="s">
         <v>14</v>
       </c>
@@ -2567,7 +2563,7 @@
       <c r="P33" s="2"/>
     </row>
     <row r="34" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D34" s="38"/>
+      <c r="D34" s="52"/>
       <c r="E34" s="2" t="s">
         <v>15</v>
       </c>
@@ -2617,7 +2613,7 @@
       </c>
     </row>
     <row r="35" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D35" s="38"/>
+      <c r="D35" s="52"/>
       <c r="E35" s="2" t="s">
         <v>16</v>
       </c>
@@ -2655,17 +2651,17 @@
       </c>
       <c r="F38" s="37"/>
       <c r="G38" s="37"/>
-      <c r="H38" s="41" t="s">
+      <c r="H38" s="38" t="s">
         <v>19</v>
       </c>
-      <c r="I38" s="50"/>
-      <c r="J38" s="50"/>
-      <c r="K38" s="50"/>
-      <c r="L38" s="50"/>
-      <c r="M38" s="50"/>
-      <c r="N38" s="50"/>
-      <c r="O38" s="50"/>
-      <c r="P38" s="51"/>
+      <c r="I38" s="39"/>
+      <c r="J38" s="39"/>
+      <c r="K38" s="39"/>
+      <c r="L38" s="39"/>
+      <c r="M38" s="39"/>
+      <c r="N38" s="39"/>
+      <c r="O38" s="39"/>
+      <c r="P38" s="40"/>
     </row>
     <row r="39" spans="4:16" ht="25.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="E39" s="2"/>
@@ -2890,15 +2886,28 @@
     </row>
   </sheetData>
   <mergeCells count="47">
-    <mergeCell ref="E12:N12"/>
-    <mergeCell ref="J13:N13"/>
-    <mergeCell ref="E21:P21"/>
-    <mergeCell ref="E29:P29"/>
-    <mergeCell ref="H38:P38"/>
-    <mergeCell ref="E13:I13"/>
-    <mergeCell ref="F14:G14"/>
-    <mergeCell ref="H14:I14"/>
-    <mergeCell ref="J14:K14"/>
+    <mergeCell ref="F39:G39"/>
+    <mergeCell ref="H39:I39"/>
+    <mergeCell ref="J39:K39"/>
+    <mergeCell ref="L39:M39"/>
+    <mergeCell ref="D15:D19"/>
+    <mergeCell ref="F30:G30"/>
+    <mergeCell ref="H30:I30"/>
+    <mergeCell ref="J30:K30"/>
+    <mergeCell ref="L22:M22"/>
+    <mergeCell ref="L30:M30"/>
+    <mergeCell ref="D31:D35"/>
+    <mergeCell ref="F22:G22"/>
+    <mergeCell ref="H22:I22"/>
+    <mergeCell ref="J22:K22"/>
+    <mergeCell ref="D23:D27"/>
+    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="K5:K6"/>
+    <mergeCell ref="K7:K8"/>
+    <mergeCell ref="K9:K10"/>
     <mergeCell ref="E2:I2"/>
     <mergeCell ref="F9:F10"/>
     <mergeCell ref="G9:G10"/>
@@ -2915,28 +2924,15 @@
     <mergeCell ref="E5:E6"/>
     <mergeCell ref="E7:E8"/>
     <mergeCell ref="E9:E10"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="K5:K6"/>
-    <mergeCell ref="K7:K8"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="F39:G39"/>
-    <mergeCell ref="H39:I39"/>
-    <mergeCell ref="J39:K39"/>
-    <mergeCell ref="L39:M39"/>
-    <mergeCell ref="D15:D19"/>
-    <mergeCell ref="F30:G30"/>
-    <mergeCell ref="H30:I30"/>
-    <mergeCell ref="J30:K30"/>
-    <mergeCell ref="L22:M22"/>
-    <mergeCell ref="L30:M30"/>
-    <mergeCell ref="D31:D35"/>
-    <mergeCell ref="F22:G22"/>
-    <mergeCell ref="H22:I22"/>
-    <mergeCell ref="J22:K22"/>
-    <mergeCell ref="D23:D27"/>
-    <mergeCell ref="E38:G38"/>
+    <mergeCell ref="E12:N12"/>
+    <mergeCell ref="J13:N13"/>
+    <mergeCell ref="E21:P21"/>
+    <mergeCell ref="E29:P29"/>
+    <mergeCell ref="H38:P38"/>
+    <mergeCell ref="E13:I13"/>
+    <mergeCell ref="F14:G14"/>
+    <mergeCell ref="H14:I14"/>
+    <mergeCell ref="J14:K14"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Descripción clara de tus cambios (ej: Refactorización de validaciones y limpieza de archivos temporales)
</commit_message>
<xml_diff>
--- a/Color/LogicDocs/calculos a realizar con el programa.xlsx
+++ b/Color/LogicDocs/calculos a realizar con el programa.xlsx
@@ -8,19 +8,20 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://coatsplc-my.sharepoint.com/personal/elkinduvan_quebradaguapacha_coats_com/Documents/Escritorio/Colorimetria/Color/LogicDocs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="845" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{E90F0389-14EF-5126-90FC-55F9316E030E}"/>
+  <xr:revisionPtr revIDLastSave="908" documentId="8_{9F78D261-5971-4E36-A791-098E2ABB119D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{54F6AF0F-B377-4726-8376-D1F0331E542D}"/>
   <bookViews>
-    <workbookView xWindow="8880" yWindow="2070" windowWidth="12525" windowHeight="8490" activeTab="2" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
+    <workbookView xWindow="8880" yWindow="2070" windowWidth="12525" windowHeight="10590" firstSheet="1" activeTab="3" xr2:uid="{74F1A0B1-3ED8-4C59-B930-9B261CE40F5C}"/>
   </bookViews>
   <sheets>
     <sheet name="CALCULO SAMPLE COMPARISON " sheetId="3" r:id="rId1"/>
     <sheet name="CALCULO SHADE HISTORY REPORT" sheetId="1" r:id="rId2"/>
     <sheet name="TOLERANCIA" sheetId="2" r:id="rId3"/>
+    <sheet name="CALCULO NUEVA RECETA" sheetId="4" r:id="rId4"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId4"/>
+    <externalReference r:id="rId5"/>
   </externalReferences>
-  <calcPr calcId="191028" iterateDelta="1E-4"/>
+  <calcPr calcId="191028"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="106">
   <si>
     <t>CMC(2.1)</t>
   </si>
@@ -272,17 +273,131 @@
   </si>
   <si>
     <t>calculos HUE</t>
+  </si>
+  <si>
+    <r>
+      <t>Prioridad de Operación:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> Se especifica que el ajuste es multiplicativo y secuencial. Primero se ajusta la carga total (fuerza) y sobre ese resultado se aplica la corrección tonal.</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve"> Análisis (shade History Report)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Deltas  </t>
+  </si>
+  <si>
+    <t>%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Factor </t>
+  </si>
+  <si>
+    <t>DL (fuerza)</t>
+  </si>
+  <si>
+    <t>DH (matiz)</t>
+  </si>
+  <si>
+    <r>
+      <t>Identificación de Colorante Clave:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> El ajuste DH se aplicó únicamente al colarante principal </t>
+    </r>
+  </si>
+  <si>
+    <t>Colarante</t>
+  </si>
+  <si>
+    <t>% Receta Original</t>
+  </si>
+  <si>
+    <t>Ajuste  DL</t>
+  </si>
+  <si>
+    <t>Ajuste DH</t>
+  </si>
+  <si>
+    <t>% Receta Nueva</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Foron NAVY S-RD: </t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>Foron RUBINE SE-RD:</t>
+  </si>
+  <si>
+    <t>Foron BRI YELLOW SE-RD:</t>
+  </si>
+  <si>
+    <t>Tipo de Alerta</t>
+  </si>
+  <si>
+    <t>Condición Técnica</t>
+  </si>
+  <si>
+    <t>Mensaje en Pantalla</t>
+  </si>
+  <si>
+    <t>Saturación Crítica</t>
+  </si>
+  <si>
+    <t>"ALERTA: Límite de saturación excedido. Posible desprendimiento de color."</t>
+  </si>
+  <si>
+    <t>Sobre-corrección</t>
+  </si>
+  <si>
+    <t>"AVISO: Ajuste agresivo detectado. Se recomienda verificar pesaje inicial."</t>
+  </si>
+  <si>
+    <t>Incompatibilidad</t>
+  </si>
+  <si>
+    <t>"ERROR: Se requiere adición de colorante externo no presente en receta base."</t>
+  </si>
+  <si>
+    <t>La concentración nueva supera el 4.5% - 5.0% (depende de la fibra).</t>
+  </si>
+  <si>
+    <t>El ajuste de matiz DH sugiere agregar un colorante que no está en la receta original.</t>
+  </si>
+  <si>
+    <t>El factor de ajuste total DL * DH es mayor a 1.30 (+30%).</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="0.000"/>
+    <numFmt numFmtId="166" formatCode="0.0"/>
+    <numFmt numFmtId="167" formatCode="0.00000"/>
+    <numFmt numFmtId="168" formatCode="0.000000"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -308,7 +423,7 @@
       <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
@@ -320,7 +435,7 @@
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <charset val="1"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
@@ -364,6 +479,19 @@
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -491,7 +619,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="53">
+  <cellXfs count="75">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -572,6 +700,53 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -628,6 +803,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -731,6 +915,10 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1069,13 +1257,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="34" t="s">
+      <c r="A1" s="53" t="s">
         <v>76</v>
       </c>
-      <c r="B1" s="34"/>
-      <c r="C1" s="34"/>
-      <c r="D1" s="34"/>
-      <c r="E1" s="34"/>
+      <c r="B1" s="53"/>
+      <c r="C1" s="53"/>
+      <c r="D1" s="53"/>
+      <c r="E1" s="53"/>
       <c r="F1" s="1"/>
       <c r="G1" s="1"/>
       <c r="H1" s="1"/>
@@ -1094,10 +1282,10 @@
       </c>
       <c r="F2" s="1"/>
       <c r="G2" s="1"/>
-      <c r="H2" s="37" t="s">
+      <c r="H2" s="56" t="s">
         <v>28</v>
       </c>
-      <c r="I2" s="37"/>
+      <c r="I2" s="56"/>
       <c r="J2" s="11"/>
       <c r="K2" s="11"/>
       <c r="L2" s="11"/>
@@ -1305,7 +1493,7 @@
       </c>
     </row>
     <row r="15" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B15" s="35" t="s">
+      <c r="B15" s="54" t="s">
         <v>6</v>
       </c>
       <c r="C15" s="7" t="s">
@@ -1320,39 +1508,39 @@
       <c r="F15" s="28">
         <v>-3.6</v>
       </c>
-      <c r="G15" s="35">
+      <c r="G15" s="54">
         <f>+D16-D15</f>
         <v>-2.1499999999999915</v>
       </c>
-      <c r="H15" s="35">
+      <c r="H15" s="54">
         <f>+E16-E15</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="I15" s="35">
+      <c r="I15" s="54">
         <f>+F16-F15</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="J15" s="35">
+      <c r="J15" s="54">
         <f>+ABS(G15)</f>
         <v>2.1499999999999915</v>
       </c>
-      <c r="K15" s="35">
+      <c r="K15" s="54">
         <f>+ABS(H15)</f>
         <v>1.2300000000000004</v>
       </c>
-      <c r="L15" s="35">
+      <c r="L15" s="54">
         <f>+ABS(I15)</f>
         <v>0.12999999999999989</v>
       </c>
-      <c r="M15" s="36">
+      <c r="M15" s="55">
         <f>+K15/F15</f>
         <v>-0.34166666666666679</v>
       </c>
-      <c r="N15" s="36">
+      <c r="N15" s="55">
         <f>+K15/E15</f>
         <v>-8.6376404494382053E-2</v>
       </c>
-      <c r="O15" s="36">
+      <c r="O15" s="55">
         <f>+L15/F15</f>
         <v>-3.611111111111108E-2</v>
       </c>
@@ -1382,7 +1570,7 @@
       </c>
     </row>
     <row r="16" spans="1:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="35"/>
+      <c r="B16" s="54"/>
       <c r="C16" s="7" t="s">
         <v>26</v>
       </c>
@@ -1395,15 +1583,15 @@
       <c r="F16" s="28">
         <v>-3.47</v>
       </c>
-      <c r="G16" s="35"/>
-      <c r="H16" s="35"/>
-      <c r="I16" s="35"/>
-      <c r="J16" s="35"/>
-      <c r="K16" s="35"/>
-      <c r="L16" s="35"/>
-      <c r="M16" s="35"/>
-      <c r="N16" s="35"/>
-      <c r="O16" s="35"/>
+      <c r="G16" s="54"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="54"/>
+      <c r="L16" s="54"/>
+      <c r="M16" s="54"/>
+      <c r="N16" s="54"/>
+      <c r="O16" s="54"/>
       <c r="P16" s="7"/>
       <c r="Q16" s="7"/>
       <c r="R16" s="7"/>
@@ -1412,7 +1600,7 @@
       <c r="U16" s="7"/>
     </row>
     <row r="17" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B17" s="35" t="s">
+      <c r="B17" s="54" t="s">
         <v>7</v>
       </c>
       <c r="C17" s="7" t="s">
@@ -1427,39 +1615,39 @@
       <c r="F17" s="28">
         <v>5.0599999999999996</v>
       </c>
-      <c r="G17" s="35">
+      <c r="G17" s="54">
         <f>+D18-D17</f>
         <v>-2.0300000000000011</v>
       </c>
-      <c r="H17" s="35">
+      <c r="H17" s="54">
         <f>+E18-E17</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="I17" s="35">
+      <c r="I17" s="54">
         <f>+F18-F17</f>
         <v>-9.39</v>
       </c>
-      <c r="J17" s="35">
+      <c r="J17" s="54">
         <f>+ABS(G17)</f>
         <v>2.0300000000000011</v>
       </c>
-      <c r="K17" s="35">
+      <c r="K17" s="54">
         <f>+ABS(H17)</f>
         <v>0.73000000000000043</v>
       </c>
-      <c r="L17" s="35">
+      <c r="L17" s="54">
         <f>+ABS(I17)</f>
         <v>9.39</v>
       </c>
-      <c r="M17" s="36">
+      <c r="M17" s="55">
         <f>+J17/D17</f>
         <v>2.4813592470358161E-2</v>
       </c>
-      <c r="N17" s="36">
+      <c r="N17" s="55">
         <f>+K17/E17</f>
         <v>-5.7165231010180145E-2</v>
       </c>
-      <c r="O17" s="36">
+      <c r="O17" s="55">
         <f>+L17/F17</f>
         <v>1.8557312252964429</v>
       </c>
@@ -1489,7 +1677,7 @@
       </c>
     </row>
     <row r="18" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B18" s="35"/>
+      <c r="B18" s="54"/>
       <c r="C18" s="7" t="s">
         <v>26</v>
       </c>
@@ -1502,15 +1690,15 @@
       <c r="F18" s="28">
         <v>-4.33</v>
       </c>
-      <c r="G18" s="35"/>
-      <c r="H18" s="35"/>
-      <c r="I18" s="35"/>
-      <c r="J18" s="35"/>
-      <c r="K18" s="35"/>
-      <c r="L18" s="35"/>
-      <c r="M18" s="35"/>
-      <c r="N18" s="35"/>
-      <c r="O18" s="35"/>
+      <c r="G18" s="54"/>
+      <c r="H18" s="54"/>
+      <c r="I18" s="54"/>
+      <c r="J18" s="54"/>
+      <c r="K18" s="54"/>
+      <c r="L18" s="54"/>
+      <c r="M18" s="54"/>
+      <c r="N18" s="54"/>
+      <c r="O18" s="54"/>
       <c r="P18" s="7"/>
       <c r="Q18" s="7"/>
       <c r="R18" s="7"/>
@@ -1519,7 +1707,7 @@
       <c r="U18" s="7"/>
     </row>
     <row r="19" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B19" s="35" t="s">
+      <c r="B19" s="54" t="s">
         <v>36</v>
       </c>
       <c r="C19" s="7" t="s">
@@ -1534,39 +1722,39 @@
       <c r="F19" s="28">
         <v>7.39</v>
       </c>
-      <c r="G19" s="35">
+      <c r="G19" s="54">
         <f>+D20-D19</f>
         <v>-4</v>
       </c>
-      <c r="H19" s="35">
+      <c r="H19" s="54">
         <f>+E20-E19</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="I19" s="35">
+      <c r="I19" s="54">
         <f>+F20-F19</f>
         <v>-0.58999999999999986</v>
       </c>
-      <c r="J19" s="35">
+      <c r="J19" s="54">
         <f>+ABS(G19)</f>
         <v>4</v>
       </c>
-      <c r="K19" s="35">
+      <c r="K19" s="54">
         <f>+ABS(H19)</f>
         <v>0.86999999999999922</v>
       </c>
-      <c r="L19" s="35">
+      <c r="L19" s="54">
         <f>+ABS(I19)</f>
         <v>0.58999999999999986</v>
       </c>
-      <c r="M19" s="36">
+      <c r="M19" s="55">
         <f>+J19/D19</f>
         <v>4.9419322955275513E-2</v>
       </c>
-      <c r="N19" s="36">
+      <c r="N19" s="55">
         <f>+K19/E19</f>
         <v>-5.7884231536926095E-2</v>
       </c>
-      <c r="O19" s="36">
+      <c r="O19" s="55">
         <f>+L19/F19</f>
         <v>7.9837618403247615E-2</v>
       </c>
@@ -1596,7 +1784,7 @@
       </c>
     </row>
     <row r="20" spans="2:21" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="B20" s="35"/>
+      <c r="B20" s="54"/>
       <c r="C20" s="7" t="s">
         <v>26</v>
       </c>
@@ -1609,15 +1797,15 @@
       <c r="F20" s="28">
         <v>6.8</v>
       </c>
-      <c r="G20" s="35"/>
-      <c r="H20" s="35"/>
-      <c r="I20" s="35"/>
-      <c r="J20" s="35"/>
-      <c r="K20" s="35"/>
-      <c r="L20" s="35"/>
-      <c r="M20" s="35"/>
-      <c r="N20" s="35"/>
-      <c r="O20" s="35"/>
+      <c r="G20" s="54"/>
+      <c r="H20" s="54"/>
+      <c r="I20" s="54"/>
+      <c r="J20" s="54"/>
+      <c r="K20" s="54"/>
+      <c r="L20" s="54"/>
+      <c r="M20" s="54"/>
+      <c r="N20" s="54"/>
+      <c r="O20" s="54"/>
       <c r="P20" s="7"/>
       <c r="Q20" s="7"/>
       <c r="R20" s="7"/>
@@ -1731,13 +1919,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E2" s="37" t="s">
+      <c r="E2" s="56" t="s">
         <v>53</v>
       </c>
-      <c r="F2" s="37"/>
-      <c r="G2" s="37"/>
-      <c r="H2" s="37"/>
-      <c r="I2" s="37"/>
+      <c r="F2" s="56"/>
+      <c r="G2" s="56"/>
+      <c r="H2" s="56"/>
+      <c r="I2" s="56"/>
     </row>
     <row r="3" spans="4:14" x14ac:dyDescent="0.2">
       <c r="E3" s="2"/>
@@ -1782,26 +1970,26 @@
       <c r="N4" s="2"/>
     </row>
     <row r="5" spans="4:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E5" s="50" t="s">
+      <c r="E5" s="69" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="47">
+      <c r="F5" s="66">
         <v>-0.78</v>
       </c>
-      <c r="G5" s="47">
+      <c r="G5" s="66">
         <v>-0.86</v>
       </c>
-      <c r="H5" s="49">
+      <c r="H5" s="68">
         <v>0.17</v>
       </c>
-      <c r="I5" s="45">
+      <c r="I5" s="64">
         <v>1.17</v>
       </c>
-      <c r="J5" s="50">
+      <c r="J5" s="69">
         <f>+ABS(F5*10)</f>
         <v>7.8000000000000007</v>
       </c>
-      <c r="K5" s="51">
+      <c r="K5" s="70">
         <f>+ABS(G5*10)</f>
         <v>8.6</v>
       </c>
@@ -1819,38 +2007,38 @@
       </c>
     </row>
     <row r="6" spans="4:14" ht="20.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E6" s="50"/>
-      <c r="F6" s="48"/>
-      <c r="G6" s="48"/>
-      <c r="H6" s="48"/>
-      <c r="I6" s="46"/>
-      <c r="J6" s="50"/>
-      <c r="K6" s="51"/>
+      <c r="E6" s="69"/>
+      <c r="F6" s="67"/>
+      <c r="G6" s="67"/>
+      <c r="H6" s="67"/>
+      <c r="I6" s="65"/>
+      <c r="J6" s="69"/>
+      <c r="K6" s="70"/>
       <c r="L6" s="2"/>
       <c r="M6" s="2"/>
       <c r="N6" s="2"/>
     </row>
     <row r="7" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E7" s="37" t="s">
+      <c r="E7" s="56" t="s">
         <v>7</v>
       </c>
-      <c r="F7" s="42">
+      <c r="F7" s="61">
         <v>-0.74</v>
       </c>
-      <c r="G7" s="44">
+      <c r="G7" s="63">
         <v>-0.54</v>
       </c>
-      <c r="H7" s="44">
+      <c r="H7" s="63">
         <v>0.1</v>
       </c>
-      <c r="I7" s="43">
+      <c r="I7" s="62">
         <v>0.92</v>
       </c>
-      <c r="J7" s="37">
+      <c r="J7" s="56">
         <f>+ABS(F7*10)</f>
         <v>7.4</v>
       </c>
-      <c r="K7" s="38">
+      <c r="K7" s="57">
         <f>+ABS(G7*10)</f>
         <v>5.4</v>
       </c>
@@ -1868,38 +2056,38 @@
       </c>
     </row>
     <row r="8" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E8" s="37"/>
-      <c r="F8" s="43"/>
-      <c r="G8" s="43"/>
-      <c r="H8" s="43"/>
-      <c r="I8" s="43"/>
-      <c r="J8" s="37"/>
-      <c r="K8" s="38"/>
+      <c r="E8" s="56"/>
+      <c r="F8" s="62"/>
+      <c r="G8" s="62"/>
+      <c r="H8" s="62"/>
+      <c r="I8" s="62"/>
+      <c r="J8" s="56"/>
+      <c r="K8" s="57"/>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
     </row>
     <row r="9" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="E9" s="37" t="s">
+      <c r="E9" s="56" t="s">
         <v>8</v>
       </c>
-      <c r="F9" s="42">
+      <c r="F9" s="61">
         <v>-0.73</v>
       </c>
-      <c r="G9" s="44">
+      <c r="G9" s="63">
         <v>-0.68</v>
       </c>
-      <c r="H9" s="44">
+      <c r="H9" s="63">
         <v>-0.12</v>
       </c>
-      <c r="I9" s="43">
+      <c r="I9" s="62">
         <v>1.01</v>
       </c>
-      <c r="J9" s="37">
+      <c r="J9" s="56">
         <f>+ABS(F9*10)</f>
         <v>7.3</v>
       </c>
-      <c r="K9" s="38">
+      <c r="K9" s="57">
         <f>+ABS(G9*10)</f>
         <v>6.8000000000000007</v>
       </c>
@@ -1917,13 +2105,13 @@
       </c>
     </row>
     <row r="10" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E10" s="37"/>
-      <c r="F10" s="43"/>
-      <c r="G10" s="43"/>
-      <c r="H10" s="43"/>
-      <c r="I10" s="43"/>
-      <c r="J10" s="37"/>
-      <c r="K10" s="38"/>
+      <c r="E10" s="56"/>
+      <c r="F10" s="62"/>
+      <c r="G10" s="62"/>
+      <c r="H10" s="62"/>
+      <c r="I10" s="62"/>
+      <c r="J10" s="56"/>
+      <c r="K10" s="57"/>
       <c r="L10" s="2"/>
       <c r="M10" s="2"/>
       <c r="N10" s="2"/>
@@ -1934,49 +2122,49 @@
       <c r="H11" s="9"/>
     </row>
     <row r="12" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E12" s="38" t="s">
+      <c r="E12" s="57" t="s">
         <v>51</v>
       </c>
-      <c r="F12" s="39"/>
-      <c r="G12" s="39"/>
-      <c r="H12" s="39"/>
-      <c r="I12" s="39"/>
-      <c r="J12" s="39"/>
-      <c r="K12" s="39"/>
-      <c r="L12" s="39"/>
-      <c r="M12" s="39"/>
-      <c r="N12" s="40"/>
+      <c r="F12" s="58"/>
+      <c r="G12" s="58"/>
+      <c r="H12" s="58"/>
+      <c r="I12" s="58"/>
+      <c r="J12" s="58"/>
+      <c r="K12" s="58"/>
+      <c r="L12" s="58"/>
+      <c r="M12" s="58"/>
+      <c r="N12" s="59"/>
     </row>
     <row r="13" spans="4:14" x14ac:dyDescent="0.25">
-      <c r="E13" s="37" t="s">
+      <c r="E13" s="56" t="s">
         <v>52</v>
       </c>
-      <c r="F13" s="37"/>
-      <c r="G13" s="37"/>
-      <c r="H13" s="37"/>
-      <c r="I13" s="37"/>
-      <c r="J13" s="38" t="s">
+      <c r="F13" s="56"/>
+      <c r="G13" s="56"/>
+      <c r="H13" s="56"/>
+      <c r="I13" s="56"/>
+      <c r="J13" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="K13" s="39"/>
-      <c r="L13" s="39"/>
-      <c r="M13" s="39"/>
-      <c r="N13" s="40"/>
+      <c r="K13" s="58"/>
+      <c r="L13" s="58"/>
+      <c r="M13" s="58"/>
+      <c r="N13" s="59"/>
     </row>
     <row r="14" spans="4:14" x14ac:dyDescent="0.2">
       <c r="E14" s="2"/>
-      <c r="F14" s="37" t="s">
+      <c r="F14" s="56" t="s">
         <v>54</v>
       </c>
-      <c r="G14" s="37"/>
-      <c r="H14" s="37" t="s">
+      <c r="G14" s="56"/>
+      <c r="H14" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="I14" s="37"/>
-      <c r="J14" s="37" t="s">
+      <c r="I14" s="56"/>
+      <c r="J14" s="56" t="s">
         <v>17</v>
       </c>
-      <c r="K14" s="37"/>
+      <c r="K14" s="56"/>
       <c r="L14" s="26" t="s">
         <v>68</v>
       </c>
@@ -1988,7 +2176,7 @@
       </c>
     </row>
     <row r="15" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D15" s="52"/>
+      <c r="D15" s="71"/>
       <c r="E15" s="29" t="s">
         <v>12</v>
       </c>
@@ -2024,7 +2212,7 @@
       <c r="N15" s="26"/>
     </row>
     <row r="16" spans="4:14" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D16" s="52"/>
+      <c r="D16" s="71"/>
       <c r="E16" s="29" t="s">
         <v>13</v>
       </c>
@@ -2056,7 +2244,7 @@
       <c r="N16" s="2"/>
     </row>
     <row r="17" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D17" s="52"/>
+      <c r="D17" s="71"/>
       <c r="E17" s="29" t="s">
         <v>14</v>
       </c>
@@ -2088,7 +2276,7 @@
       <c r="N17" s="2"/>
     </row>
     <row r="18" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D18" s="52"/>
+      <c r="D18" s="71"/>
       <c r="E18" s="2" t="s">
         <v>15</v>
       </c>
@@ -2130,7 +2318,7 @@
       </c>
     </row>
     <row r="19" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D19" s="52"/>
+      <c r="D19" s="71"/>
       <c r="E19" s="2" t="s">
         <v>16</v>
       </c>
@@ -2152,39 +2340,39 @@
       <c r="O19" s="27"/>
     </row>
     <row r="21" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E21" s="41" t="s">
+      <c r="E21" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="F21" s="34"/>
-      <c r="G21" s="34"/>
-      <c r="H21" s="34"/>
-      <c r="I21" s="34"/>
-      <c r="J21" s="34"/>
-      <c r="K21" s="34"/>
-      <c r="L21" s="34"/>
-      <c r="M21" s="34"/>
-      <c r="N21" s="34"/>
-      <c r="O21" s="34"/>
-      <c r="P21" s="34"/>
+      <c r="F21" s="53"/>
+      <c r="G21" s="53"/>
+      <c r="H21" s="53"/>
+      <c r="I21" s="53"/>
+      <c r="J21" s="53"/>
+      <c r="K21" s="53"/>
+      <c r="L21" s="53"/>
+      <c r="M21" s="53"/>
+      <c r="N21" s="53"/>
+      <c r="O21" s="53"/>
+      <c r="P21" s="53"/>
     </row>
     <row r="22" spans="4:16" x14ac:dyDescent="0.2">
       <c r="E22" s="2"/>
-      <c r="F22" s="37" t="s">
+      <c r="F22" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="G22" s="37"/>
-      <c r="H22" s="37" t="s">
+      <c r="G22" s="56"/>
+      <c r="H22" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="I22" s="37"/>
-      <c r="J22" s="37" t="s">
+      <c r="I22" s="56"/>
+      <c r="J22" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="K22" s="37"/>
-      <c r="L22" s="37" t="s">
+      <c r="K22" s="56"/>
+      <c r="L22" s="56" t="s">
         <v>75</v>
       </c>
-      <c r="M22" s="37"/>
+      <c r="M22" s="56"/>
       <c r="N22" s="26" t="s">
         <v>60</v>
       </c>
@@ -2196,7 +2384,7 @@
       </c>
     </row>
     <row r="23" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D23" s="52"/>
+      <c r="D23" s="71"/>
       <c r="E23" s="29" t="s">
         <v>12</v>
       </c>
@@ -2236,7 +2424,7 @@
       <c r="P23" s="2"/>
     </row>
     <row r="24" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D24" s="52"/>
+      <c r="D24" s="71"/>
       <c r="E24" s="29" t="s">
         <v>13</v>
       </c>
@@ -2276,7 +2464,7 @@
       <c r="P24" s="2"/>
     </row>
     <row r="25" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D25" s="52"/>
+      <c r="D25" s="71"/>
       <c r="E25" s="29" t="s">
         <v>14</v>
       </c>
@@ -2316,7 +2504,7 @@
       <c r="P25" s="2"/>
     </row>
     <row r="26" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D26" s="52"/>
+      <c r="D26" s="71"/>
       <c r="E26" s="2" t="s">
         <v>15</v>
       </c>
@@ -2366,7 +2554,7 @@
       </c>
     </row>
     <row r="27" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D27" s="52"/>
+      <c r="D27" s="71"/>
       <c r="E27" s="2" t="s">
         <v>16</v>
       </c>
@@ -2399,39 +2587,39 @@
       <c r="P27" s="2"/>
     </row>
     <row r="29" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E29" s="41" t="s">
+      <c r="E29" s="60" t="s">
         <v>56</v>
       </c>
-      <c r="F29" s="34"/>
-      <c r="G29" s="34"/>
-      <c r="H29" s="34"/>
-      <c r="I29" s="34"/>
-      <c r="J29" s="34"/>
-      <c r="K29" s="34"/>
-      <c r="L29" s="34"/>
-      <c r="M29" s="34"/>
-      <c r="N29" s="34"/>
-      <c r="O29" s="34"/>
-      <c r="P29" s="34"/>
+      <c r="F29" s="53"/>
+      <c r="G29" s="53"/>
+      <c r="H29" s="53"/>
+      <c r="I29" s="53"/>
+      <c r="J29" s="53"/>
+      <c r="K29" s="53"/>
+      <c r="L29" s="53"/>
+      <c r="M29" s="53"/>
+      <c r="N29" s="53"/>
+      <c r="O29" s="53"/>
+      <c r="P29" s="53"/>
     </row>
     <row r="30" spans="4:16" ht="25.5" x14ac:dyDescent="0.2">
       <c r="E30" s="2"/>
-      <c r="F30" s="37" t="s">
+      <c r="F30" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="G30" s="37"/>
-      <c r="H30" s="37" t="s">
+      <c r="G30" s="56"/>
+      <c r="H30" s="56" t="s">
         <v>10</v>
       </c>
-      <c r="I30" s="37"/>
-      <c r="J30" s="37" t="s">
+      <c r="I30" s="56"/>
+      <c r="J30" s="56" t="s">
         <v>11</v>
       </c>
-      <c r="K30" s="37"/>
-      <c r="L30" s="37" t="s">
+      <c r="K30" s="56"/>
+      <c r="L30" s="56" t="s">
         <v>18</v>
       </c>
-      <c r="M30" s="37"/>
+      <c r="M30" s="56"/>
       <c r="N30" s="26" t="s">
         <v>60</v>
       </c>
@@ -2443,7 +2631,7 @@
       </c>
     </row>
     <row r="31" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D31" s="52"/>
+      <c r="D31" s="71"/>
       <c r="E31" s="29" t="s">
         <v>12</v>
       </c>
@@ -2483,7 +2671,7 @@
       <c r="P31" s="2"/>
     </row>
     <row r="32" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D32" s="52"/>
+      <c r="D32" s="71"/>
       <c r="E32" s="29" t="s">
         <v>13</v>
       </c>
@@ -2523,7 +2711,7 @@
       <c r="P32" s="2"/>
     </row>
     <row r="33" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="D33" s="52"/>
+      <c r="D33" s="71"/>
       <c r="E33" s="29" t="s">
         <v>14</v>
       </c>
@@ -2563,7 +2751,7 @@
       <c r="P33" s="2"/>
     </row>
     <row r="34" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D34" s="52"/>
+      <c r="D34" s="71"/>
       <c r="E34" s="2" t="s">
         <v>15</v>
       </c>
@@ -2613,7 +2801,7 @@
       </c>
     </row>
     <row r="35" spans="4:16" ht="15" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="D35" s="52"/>
+      <c r="D35" s="71"/>
       <c r="E35" s="2" t="s">
         <v>16</v>
       </c>
@@ -2646,41 +2834,41 @@
       <c r="P35" s="2"/>
     </row>
     <row r="38" spans="4:16" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="E38" s="37" t="s">
+      <c r="E38" s="56" t="s">
         <v>57</v>
       </c>
-      <c r="F38" s="37"/>
-      <c r="G38" s="37"/>
-      <c r="H38" s="38" t="s">
+      <c r="F38" s="56"/>
+      <c r="G38" s="56"/>
+      <c r="H38" s="57" t="s">
         <v>19</v>
       </c>
-      <c r="I38" s="39"/>
-      <c r="J38" s="39"/>
-      <c r="K38" s="39"/>
-      <c r="L38" s="39"/>
-      <c r="M38" s="39"/>
-      <c r="N38" s="39"/>
-      <c r="O38" s="39"/>
-      <c r="P38" s="40"/>
+      <c r="I38" s="58"/>
+      <c r="J38" s="58"/>
+      <c r="K38" s="58"/>
+      <c r="L38" s="58"/>
+      <c r="M38" s="58"/>
+      <c r="N38" s="58"/>
+      <c r="O38" s="58"/>
+      <c r="P38" s="59"/>
     </row>
     <row r="39" spans="4:16" ht="25.5" hidden="1" x14ac:dyDescent="0.2">
       <c r="E39" s="2"/>
-      <c r="F39" s="37" t="s">
+      <c r="F39" s="56" t="s">
         <v>9</v>
       </c>
-      <c r="G39" s="37"/>
-      <c r="H39" s="37" t="s">
+      <c r="G39" s="56"/>
+      <c r="H39" s="56" t="s">
         <v>48</v>
       </c>
-      <c r="I39" s="37"/>
-      <c r="J39" s="37" t="s">
+      <c r="I39" s="56"/>
+      <c r="J39" s="56" t="s">
         <v>49</v>
       </c>
-      <c r="K39" s="37"/>
-      <c r="L39" s="37" t="s">
+      <c r="K39" s="56"/>
+      <c r="L39" s="56" t="s">
         <v>50</v>
       </c>
-      <c r="M39" s="37"/>
+      <c r="M39" s="56"/>
       <c r="N39" s="19" t="s">
         <v>71</v>
       </c>
@@ -3069,4 +3257,245 @@
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1BD7E673-853E-4343-94E1-725EDA103DB7}">
+  <dimension ref="B2:J19"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="20.42578125" customWidth="1"/>
+    <col min="3" max="3" width="11.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.85546875" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="18" customWidth="1"/>
+    <col min="9" max="9" width="29" customWidth="1"/>
+    <col min="10" max="10" width="36" customWidth="1"/>
+    <col min="12" max="13" width="9.140625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H2" s="72" t="s">
+        <v>77</v>
+      </c>
+      <c r="I2" s="72"/>
+    </row>
+    <row r="3" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H3" s="72"/>
+      <c r="I3" s="72"/>
+    </row>
+    <row r="4" spans="2:10" ht="27.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="73" t="s">
+        <v>78</v>
+      </c>
+      <c r="C4" s="73"/>
+      <c r="D4" s="73"/>
+      <c r="E4" s="7"/>
+      <c r="H4" s="72"/>
+      <c r="I4" s="72"/>
+    </row>
+    <row r="5" spans="2:10" ht="22.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="34" t="s">
+        <v>79</v>
+      </c>
+      <c r="C5" s="35" t="s">
+        <v>80</v>
+      </c>
+      <c r="D5" s="36" t="s">
+        <v>81</v>
+      </c>
+      <c r="E5" s="7"/>
+      <c r="H5" s="72"/>
+      <c r="I5" s="72"/>
+    </row>
+    <row r="6" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B6" s="37" t="s">
+        <v>82</v>
+      </c>
+      <c r="C6" s="38">
+        <v>9.1</v>
+      </c>
+      <c r="D6" s="8">
+        <f>1+(C6/100)</f>
+        <v>1.091</v>
+      </c>
+      <c r="E6" s="7"/>
+      <c r="H6" s="72"/>
+      <c r="I6" s="72"/>
+    </row>
+    <row r="7" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B7" s="39" t="s">
+        <v>83</v>
+      </c>
+      <c r="C7" s="38">
+        <v>13</v>
+      </c>
+      <c r="D7" s="7">
+        <f>1+(C7/100)</f>
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="E7" s="7"/>
+    </row>
+    <row r="8" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H8" s="72" t="s">
+        <v>84</v>
+      </c>
+      <c r="I8" s="72"/>
+    </row>
+    <row r="9" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H9" s="72"/>
+      <c r="I9" s="72"/>
+    </row>
+    <row r="10" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B10" s="36" t="s">
+        <v>85</v>
+      </c>
+      <c r="C10" s="40" t="s">
+        <v>86</v>
+      </c>
+      <c r="D10" s="41" t="s">
+        <v>87</v>
+      </c>
+      <c r="E10" s="41" t="s">
+        <v>88</v>
+      </c>
+      <c r="F10" s="41" t="s">
+        <v>89</v>
+      </c>
+      <c r="H10" s="72"/>
+      <c r="I10" s="72"/>
+    </row>
+    <row r="11" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B11" s="37" t="s">
+        <v>90</v>
+      </c>
+      <c r="C11" s="7">
+        <v>1.1782600000000001</v>
+      </c>
+      <c r="D11" s="7">
+        <f>$D$6</f>
+        <v>1.091</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F11" s="42">
+        <f>C11*D11</f>
+        <v>1.2854816600000001</v>
+      </c>
+      <c r="H11" s="72"/>
+      <c r="I11" s="72"/>
+    </row>
+    <row r="12" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B12" s="37" t="s">
+        <v>92</v>
+      </c>
+      <c r="C12" s="42">
+        <v>0.38450000000000001</v>
+      </c>
+      <c r="D12" s="7">
+        <f t="shared" ref="D12:D13" si="0">$D$6</f>
+        <v>1.091</v>
+      </c>
+      <c r="E12" s="7">
+        <f>$D$7</f>
+        <v>1.1299999999999999</v>
+      </c>
+      <c r="F12" s="42">
+        <f>((C12*D12)*E12)</f>
+        <v>0.47402313499999998</v>
+      </c>
+      <c r="G12" s="43"/>
+      <c r="H12" s="72"/>
+      <c r="I12" s="72"/>
+    </row>
+    <row r="13" spans="2:10" ht="30" x14ac:dyDescent="0.25">
+      <c r="B13" s="44" t="s">
+        <v>93</v>
+      </c>
+      <c r="C13" s="42">
+        <v>0.375</v>
+      </c>
+      <c r="D13" s="7">
+        <f t="shared" si="0"/>
+        <v>1.091</v>
+      </c>
+      <c r="E13" s="7" t="s">
+        <v>91</v>
+      </c>
+      <c r="F13" s="42">
+        <f>C13*D13</f>
+        <v>0.40912499999999996</v>
+      </c>
+    </row>
+    <row r="14" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="H14" s="47" t="s">
+        <v>94</v>
+      </c>
+      <c r="I14" s="47" t="s">
+        <v>95</v>
+      </c>
+      <c r="J14" s="48" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="15" spans="2:10" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="B15" s="74"/>
+      <c r="C15" s="74"/>
+      <c r="H15" s="45" t="s">
+        <v>97</v>
+      </c>
+      <c r="I15" s="45" t="s">
+        <v>103</v>
+      </c>
+      <c r="J15" s="46" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="2:10" ht="42.75" x14ac:dyDescent="0.25">
+      <c r="B16" s="6"/>
+      <c r="C16" s="49"/>
+      <c r="H16" s="45" t="s">
+        <v>99</v>
+      </c>
+      <c r="I16" s="45" t="s">
+        <v>105</v>
+      </c>
+      <c r="J16" s="45" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="17" spans="2:10" ht="57" x14ac:dyDescent="0.25">
+      <c r="B17" s="50"/>
+      <c r="C17" s="51"/>
+      <c r="H17" s="45" t="s">
+        <v>101</v>
+      </c>
+      <c r="I17" s="45" t="s">
+        <v>104</v>
+      </c>
+      <c r="J17" s="46" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="18" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B18" s="50"/>
+      <c r="C18" s="51"/>
+    </row>
+    <row r="19" spans="2:10" x14ac:dyDescent="0.25">
+      <c r="B19" s="52"/>
+      <c r="C19" s="51"/>
+    </row>
+  </sheetData>
+  <mergeCells count="4">
+    <mergeCell ref="H2:I6"/>
+    <mergeCell ref="B4:D4"/>
+    <mergeCell ref="H8:I12"/>
+    <mergeCell ref="B15:C15"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <ignoredErrors>
+    <ignoredError sqref="F12" formula="1"/>
+  </ignoredErrors>
+</worksheet>
 </file>
</xml_diff>